<commit_message>
founder sign-off recorded: D1-D14 accepted by Jaime Tanori, 2026-10-21; workbook W00-02/03 marked Done
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="583">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -491,6 +491,9 @@
     <t>Four ADRs marked Accepted with a name and date</t>
   </si>
   <si>
+    <t>✅ Done — D1/D5/D11/D14 marked Accepted, name+date in 05-kickoff-pack §2</t>
+  </si>
+  <si>
     <t>W00-03</t>
   </si>
   <si>
@@ -501,6 +504,9 @@
   </si>
   <si>
     <t>Fourteen of fourteen Accepted</t>
+  </si>
+  <si>
+    <t>✅ Done — 14/14 ADRs marked Accepted, name+date in 05-kickoff-pack §2</t>
   </si>
   <si>
     <t>W00-04</t>
@@ -3207,12 +3213,12 @@
         <v>155</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>51</v>
@@ -3224,10 +3230,10 @@
         <v>146</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G7" s="12">
         <v>0.25</v>
@@ -3239,15 +3245,15 @@
         <v>152</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>51</v>
@@ -3256,13 +3262,13 @@
         <v>145</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G8" s="12">
         <v>0.5</v>
@@ -3274,7 +3280,7 @@
         <v>61</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="K8" s="11" t="s">
         <v>151</v>
@@ -3282,7 +3288,7 @@
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>51</v>
@@ -3291,25 +3297,25 @@
         <v>145</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G9" s="12">
         <v>0.25</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>151</v>
@@ -3317,7 +3323,7 @@
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>51</v>
@@ -3326,13 +3332,13 @@
         <v>145</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G10" s="12">
         <v>0.25</v>
@@ -3344,7 +3350,7 @@
         <v>61</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>151</v>
@@ -3352,7 +3358,7 @@
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>51</v>
@@ -3361,13 +3367,13 @@
         <v>145</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G11" s="12">
         <v>0.5</v>
@@ -3379,7 +3385,7 @@
         <v>61</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K11" s="11" t="s">
         <v>151</v>
@@ -3387,7 +3393,7 @@
     </row>
     <row r="12" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>51</v>
@@ -3396,13 +3402,13 @@
         <v>145</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G12" s="12">
         <v>0.25</v>
@@ -3411,10 +3417,10 @@
         <v>149</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>151</v>
@@ -3422,7 +3428,7 @@
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>51</v>
@@ -3431,13 +3437,13 @@
         <v>145</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G13" s="12">
         <v>0.25</v>
@@ -3446,10 +3452,10 @@
         <v>149</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>151</v>
@@ -3457,7 +3463,7 @@
     </row>
     <row r="14" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>51</v>
@@ -3466,13 +3472,13 @@
         <v>145</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G14" s="12">
         <v>0.5</v>
@@ -3484,7 +3490,7 @@
         <v>61</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>151</v>
@@ -3492,22 +3498,22 @@
     </row>
     <row r="15" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G15" s="12">
         <v>0.5</v>
@@ -3519,7 +3525,7 @@
         <v>61</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>151</v>
@@ -3527,22 +3533,22 @@
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G16" s="12">
         <v>0.75</v>
@@ -3551,10 +3557,10 @@
         <v>149</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="K16" s="11" t="s">
         <v>151</v>
@@ -3562,22 +3568,22 @@
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G17" s="12">
         <v>0.75</v>
@@ -3586,10 +3592,10 @@
         <v>149</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>151</v>
@@ -3597,22 +3603,22 @@
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G18" s="12">
         <v>0.5</v>
@@ -3621,10 +3627,10 @@
         <v>149</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>151</v>
@@ -3632,22 +3638,22 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G19" s="12">
         <v>0.5</v>
@@ -3659,15 +3665,15 @@
         <v>61</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -3676,13 +3682,13 @@
         <v>145</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G20" s="12">
         <v>0.25</v>
@@ -3691,10 +3697,10 @@
         <v>149</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>151</v>
@@ -3702,22 +3708,22 @@
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G21" s="12">
         <v>0.5</v>
@@ -3726,10 +3732,10 @@
         <v>149</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>151</v>
@@ -3737,7 +3743,7 @@
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -3746,13 +3752,13 @@
         <v>145</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G22" s="12">
         <v>0.25</v>
@@ -3764,7 +3770,7 @@
         <v>61</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="K22" s="11" t="s">
         <v>151</v>
@@ -3772,22 +3778,22 @@
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G23" s="12">
         <v>0.5</v>
@@ -3799,30 +3805,30 @@
         <v>61</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G24" s="12">
         <v>0.25</v>
@@ -3831,10 +3837,10 @@
         <v>149</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>151</v>
@@ -3842,22 +3848,22 @@
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>57</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G25" s="12">
         <v>3</v>
@@ -3869,7 +3875,7 @@
         <v>144</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>151</v>
@@ -3877,22 +3883,22 @@
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3901,10 +3907,10 @@
         <v>149</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>151</v>
@@ -3912,22 +3918,22 @@
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3936,10 +3942,10 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>151</v>
@@ -3947,22 +3953,22 @@
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3971,10 +3977,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3982,22 +3988,22 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4006,10 +4012,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4017,22 +4023,22 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4041,10 +4047,10 @@
         <v>149</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4052,22 +4058,22 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4076,10 +4082,10 @@
         <v>149</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4087,22 +4093,22 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4111,10 +4117,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4122,22 +4128,22 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4146,10 +4152,10 @@
         <v>149</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4157,22 +4163,22 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4181,10 +4187,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4192,22 +4198,22 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4216,10 +4222,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4227,22 +4233,22 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4251,10 +4257,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4262,22 +4268,22 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4286,10 +4292,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4297,22 +4303,22 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4321,10 +4327,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4332,22 +4338,22 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4356,10 +4362,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4367,22 +4373,22 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4391,10 +4397,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4402,22 +4408,22 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4426,10 +4432,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4437,22 +4443,22 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4461,10 +4467,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4472,22 +4478,22 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4496,10 +4502,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4507,22 +4513,22 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4531,10 +4537,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4542,34 +4548,34 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4577,22 +4583,22 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4601,10 +4607,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4612,22 +4618,22 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4636,10 +4642,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4647,22 +4653,22 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4671,10 +4677,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4682,22 +4688,22 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4706,10 +4712,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4717,22 +4723,22 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4741,10 +4747,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4752,22 +4758,22 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4776,10 +4782,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4787,22 +4793,22 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4811,10 +4817,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4822,22 +4828,22 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4846,10 +4852,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4857,22 +4863,22 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4881,10 +4887,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4892,22 +4898,22 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4916,10 +4922,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4927,22 +4933,22 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4951,10 +4957,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4962,22 +4968,22 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4986,10 +4992,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -4997,22 +5003,22 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5021,10 +5027,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5032,22 +5038,22 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5056,10 +5062,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5067,22 +5073,22 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D60" s="11" t="s">
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5091,10 +5097,10 @@
         <v>149</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5102,22 +5108,22 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D61" s="11" t="s">
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5126,10 +5132,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5137,22 +5143,22 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D62" s="11" t="s">
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5161,10 +5167,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5172,22 +5178,22 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5196,10 +5202,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5207,22 +5213,22 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5231,10 +5237,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5242,22 +5248,22 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5266,10 +5272,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5277,22 +5283,22 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5301,10 +5307,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5312,22 +5318,22 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C67" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5336,10 +5342,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5347,22 +5353,22 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5371,10 +5377,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5382,34 +5388,34 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
       </c>
       <c r="H69" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5417,34 +5423,34 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
       </c>
       <c r="H70" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5452,22 +5458,22 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D71" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5476,10 +5482,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5487,7 +5493,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5496,13 +5502,13 @@
         <v>145</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5511,10 +5517,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5522,22 +5528,22 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5546,10 +5552,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5557,7 +5563,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5566,13 +5572,13 @@
         <v>145</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5581,10 +5587,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5592,22 +5598,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5616,10 +5622,10 @@
         <v>149</v>
       </c>
       <c r="I75" s="23" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5627,22 +5633,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C76" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5651,10 +5657,10 @@
         <v>149</v>
       </c>
       <c r="I76" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5662,22 +5668,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C77" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5686,10 +5692,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5697,22 +5703,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C78" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5721,10 +5727,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5732,22 +5738,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5756,10 +5762,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5767,22 +5773,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C80" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5791,10 +5797,10 @@
         <v>149</v>
       </c>
       <c r="I80" s="23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5802,22 +5808,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5826,10 +5832,10 @@
         <v>149</v>
       </c>
       <c r="I81" s="23" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5837,34 +5843,34 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
       </c>
       <c r="H82" s="23" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5872,34 +5878,34 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
       </c>
       <c r="H83" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5907,34 +5913,34 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D84" s="26" t="s">
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
       </c>
       <c r="H84" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5974,12 +5980,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5993,19 +5999,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6028,10 +6034,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6054,10 +6060,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6080,10 +6086,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6106,7 +6112,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6130,7 +6136,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6154,10 +6160,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6180,7 +6186,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6204,7 +6210,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6228,10 +6234,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6254,7 +6260,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6278,7 +6284,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6302,7 +6308,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6326,7 +6332,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6350,15 +6356,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6366,7 +6372,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6374,7 +6380,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6403,7 +6409,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6420,10 +6426,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6431,7 +6437,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6440,10 +6446,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6451,7 +6457,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6463,7 +6469,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6471,7 +6477,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6480,10 +6486,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6491,7 +6497,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6500,10 +6506,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6517,18 +6523,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6537,53 +6543,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
   </sheetData>
@@ -6608,26 +6614,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6635,13 +6641,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6649,13 +6655,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6663,13 +6669,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6677,13 +6683,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6691,13 +6697,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6705,13 +6711,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6719,13 +6725,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6733,13 +6739,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6747,13 +6753,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6761,13 +6767,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6775,21 +6781,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6825,7 +6831,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6833,7 +6839,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6845,167 +6851,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>
@@ -7037,7 +7043,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7057,47 +7063,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7108,16 +7114,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7125,19 +7131,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7145,19 +7151,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7165,19 +7171,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W00-11: mark Done in workbook (PR #1, GH006 evidence)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="584">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -618,6 +618,9 @@
   </si>
   <si>
     <t>A direct push to main is rejected</t>
+  </si>
+  <si>
+    <t>✅ Done (e8f134b)</t>
   </si>
   <si>
     <t>W00-12</t>
@@ -3528,12 +3531,12 @@
         <v>198</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>51</v>
@@ -3545,10 +3548,10 @@
         <v>146</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G16" s="12">
         <v>0.75</v>
@@ -3560,7 +3563,7 @@
         <v>194</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K16" s="11" t="s">
         <v>151</v>
@@ -3568,7 +3571,7 @@
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>51</v>
@@ -3580,10 +3583,10 @@
         <v>146</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G17" s="12">
         <v>0.75</v>
@@ -3592,10 +3595,10 @@
         <v>149</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>151</v>
@@ -3603,7 +3606,7 @@
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>51</v>
@@ -3615,10 +3618,10 @@
         <v>146</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G18" s="12">
         <v>0.5</v>
@@ -3627,10 +3630,10 @@
         <v>149</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>151</v>
@@ -3638,7 +3641,7 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>51</v>
@@ -3647,13 +3650,13 @@
         <v>195</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G19" s="12">
         <v>0.5</v>
@@ -3665,15 +3668,15 @@
         <v>61</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -3685,10 +3688,10 @@
         <v>190</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G20" s="12">
         <v>0.25</v>
@@ -3700,7 +3703,7 @@
         <v>189</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>151</v>
@@ -3708,7 +3711,7 @@
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
@@ -3720,10 +3723,10 @@
         <v>70</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G21" s="12">
         <v>0.5</v>
@@ -3732,10 +3735,10 @@
         <v>149</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>151</v>
@@ -3743,7 +3746,7 @@
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -3755,10 +3758,10 @@
         <v>177</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G22" s="12">
         <v>0.25</v>
@@ -3770,7 +3773,7 @@
         <v>61</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K22" s="11" t="s">
         <v>151</v>
@@ -3778,7 +3781,7 @@
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
@@ -3790,10 +3793,10 @@
         <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G23" s="12">
         <v>0.5</v>
@@ -3805,30 +3808,30 @@
         <v>61</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G24" s="12">
         <v>0.25</v>
@@ -3837,10 +3840,10 @@
         <v>149</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>151</v>
@@ -3848,7 +3851,7 @@
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>57</v>
@@ -3860,10 +3863,10 @@
         <v>146</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G25" s="12">
         <v>3</v>
@@ -3875,7 +3878,7 @@
         <v>144</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>151</v>
@@ -3883,7 +3886,7 @@
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3895,10 +3898,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3907,10 +3910,10 @@
         <v>149</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>151</v>
@@ -3918,7 +3921,7 @@
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3930,10 +3933,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3942,10 +3945,10 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>151</v>
@@ -3953,7 +3956,7 @@
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3965,10 +3968,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3977,10 +3980,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3988,7 +3991,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4000,10 +4003,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4012,10 +4015,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4023,7 +4026,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4035,10 +4038,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4047,10 +4050,10 @@
         <v>149</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4058,7 +4061,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4070,10 +4073,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4082,10 +4085,10 @@
         <v>149</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4093,7 +4096,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4105,10 +4108,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4117,10 +4120,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4128,7 +4131,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4140,10 +4143,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4152,10 +4155,10 @@
         <v>149</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4163,7 +4166,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4175,10 +4178,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4187,10 +4190,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4198,7 +4201,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4210,10 +4213,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4222,10 +4225,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4233,7 +4236,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4245,10 +4248,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4257,10 +4260,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4268,7 +4271,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4277,13 +4280,13 @@
         <v>195</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4292,10 +4295,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4303,7 +4306,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4312,13 +4315,13 @@
         <v>195</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4327,10 +4330,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4338,7 +4341,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4347,13 +4350,13 @@
         <v>195</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4362,10 +4365,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4373,7 +4376,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4382,13 +4385,13 @@
         <v>195</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4397,10 +4400,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4408,7 +4411,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4417,13 +4420,13 @@
         <v>195</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4432,10 +4435,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4443,7 +4446,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4452,13 +4455,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4467,10 +4470,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4478,7 +4481,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4487,13 +4490,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4502,10 +4505,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4513,7 +4516,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4522,13 +4525,13 @@
         <v>195</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4537,10 +4540,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4548,7 +4551,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4557,13 +4560,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4572,10 +4575,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4583,7 +4586,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4592,13 +4595,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4607,10 +4610,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4618,7 +4621,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4627,13 +4630,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4642,10 +4645,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4653,7 +4656,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4662,13 +4665,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4677,10 +4680,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4688,7 +4691,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4697,13 +4700,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4712,10 +4715,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4723,7 +4726,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4732,13 +4735,13 @@
         <v>195</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4747,10 +4750,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4758,7 +4761,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4767,13 +4770,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4782,10 +4785,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4793,7 +4796,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4802,13 +4805,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4817,10 +4820,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4828,7 +4831,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4837,13 +4840,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4852,10 +4855,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4863,7 +4866,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4872,13 +4875,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4887,10 +4890,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4898,7 +4901,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4907,13 +4910,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4922,10 +4925,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4933,7 +4936,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4942,13 +4945,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4957,10 +4960,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4968,7 +4971,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4977,13 +4980,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4992,10 +4995,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5003,7 +5006,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5012,13 +5015,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5027,10 +5030,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5038,7 +5041,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5047,13 +5050,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5062,10 +5065,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5073,7 +5076,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5085,10 +5088,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5097,10 +5100,10 @@
         <v>149</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5108,7 +5111,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5120,10 +5123,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5132,10 +5135,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5143,7 +5146,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5155,10 +5158,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5167,10 +5170,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5178,7 +5181,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5187,13 +5190,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5202,10 +5205,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5213,7 +5216,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5222,13 +5225,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5237,10 +5240,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5248,7 +5251,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5257,13 +5260,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5272,10 +5275,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5283,7 +5286,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5292,13 +5295,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5307,10 +5310,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5318,7 +5321,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5327,13 +5330,13 @@
         <v>195</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5342,10 +5345,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5353,7 +5356,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5362,13 +5365,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5377,10 +5380,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5388,7 +5391,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5397,13 +5400,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5412,10 +5415,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5423,7 +5426,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5432,13 +5435,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5447,10 +5450,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5458,22 +5461,22 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D71" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5482,10 +5485,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5493,7 +5496,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5505,10 +5508,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5517,10 +5520,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5528,22 +5531,22 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5552,10 +5555,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5563,7 +5566,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5575,10 +5578,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5587,10 +5590,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5598,22 +5601,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5625,7 +5628,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5633,22 +5636,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5660,7 +5663,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5668,22 +5671,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5692,10 +5695,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5703,22 +5706,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5727,10 +5730,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5738,22 +5741,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5762,10 +5765,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5773,22 +5776,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5800,7 +5803,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5808,22 +5811,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5835,7 +5838,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5843,22 +5846,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5867,10 +5870,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5878,22 +5881,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5902,10 +5905,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5913,10 +5916,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5925,10 +5928,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5937,10 +5940,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5980,12 +5983,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5999,19 +6002,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6034,10 +6037,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6060,10 +6063,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6086,10 +6089,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6112,7 +6115,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6136,7 +6139,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6160,10 +6163,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6186,7 +6189,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6210,7 +6213,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6234,10 +6237,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6260,7 +6263,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6284,7 +6287,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6308,7 +6311,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6332,7 +6335,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6356,15 +6359,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6372,7 +6375,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6380,7 +6383,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6409,7 +6412,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6426,10 +6429,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6437,7 +6440,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6446,10 +6449,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6457,7 +6460,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6469,7 +6472,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6477,7 +6480,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6486,10 +6489,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6497,7 +6500,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6506,10 +6509,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6523,18 +6526,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6543,53 +6546,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
   </sheetData>
@@ -6614,26 +6617,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6641,13 +6644,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6655,13 +6658,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6669,13 +6672,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6683,13 +6686,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6697,13 +6700,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6711,13 +6714,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6725,13 +6728,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6739,13 +6742,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6753,13 +6756,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6767,13 +6770,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6781,21 +6784,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6831,7 +6834,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6839,7 +6842,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6851,167 +6854,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -7043,7 +7046,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7063,47 +7066,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7114,16 +7117,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7131,19 +7134,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7151,19 +7154,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7171,19 +7174,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W00-11: mark Done in workbook (PR #1, GH006 evidence) (#2)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="584">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -618,6 +618,9 @@
   </si>
   <si>
     <t>A direct push to main is rejected</t>
+  </si>
+  <si>
+    <t>✅ Done (e8f134b)</t>
   </si>
   <si>
     <t>W00-12</t>
@@ -3528,12 +3531,12 @@
         <v>198</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>51</v>
@@ -3545,10 +3548,10 @@
         <v>146</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G16" s="12">
         <v>0.75</v>
@@ -3560,7 +3563,7 @@
         <v>194</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K16" s="11" t="s">
         <v>151</v>
@@ -3568,7 +3571,7 @@
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>51</v>
@@ -3580,10 +3583,10 @@
         <v>146</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G17" s="12">
         <v>0.75</v>
@@ -3592,10 +3595,10 @@
         <v>149</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>151</v>
@@ -3603,7 +3606,7 @@
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>51</v>
@@ -3615,10 +3618,10 @@
         <v>146</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G18" s="12">
         <v>0.5</v>
@@ -3627,10 +3630,10 @@
         <v>149</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>151</v>
@@ -3638,7 +3641,7 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>51</v>
@@ -3647,13 +3650,13 @@
         <v>195</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G19" s="12">
         <v>0.5</v>
@@ -3665,15 +3668,15 @@
         <v>61</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -3685,10 +3688,10 @@
         <v>190</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G20" s="12">
         <v>0.25</v>
@@ -3700,7 +3703,7 @@
         <v>189</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>151</v>
@@ -3708,7 +3711,7 @@
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
@@ -3720,10 +3723,10 @@
         <v>70</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G21" s="12">
         <v>0.5</v>
@@ -3732,10 +3735,10 @@
         <v>149</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>151</v>
@@ -3743,7 +3746,7 @@
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -3755,10 +3758,10 @@
         <v>177</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G22" s="12">
         <v>0.25</v>
@@ -3770,7 +3773,7 @@
         <v>61</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K22" s="11" t="s">
         <v>151</v>
@@ -3778,7 +3781,7 @@
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
@@ -3790,10 +3793,10 @@
         <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G23" s="12">
         <v>0.5</v>
@@ -3805,30 +3808,30 @@
         <v>61</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G24" s="12">
         <v>0.25</v>
@@ -3837,10 +3840,10 @@
         <v>149</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>151</v>
@@ -3848,7 +3851,7 @@
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>57</v>
@@ -3860,10 +3863,10 @@
         <v>146</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G25" s="12">
         <v>3</v>
@@ -3875,7 +3878,7 @@
         <v>144</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>151</v>
@@ -3883,7 +3886,7 @@
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3895,10 +3898,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3907,10 +3910,10 @@
         <v>149</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>151</v>
@@ -3918,7 +3921,7 @@
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3930,10 +3933,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3942,10 +3945,10 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>151</v>
@@ -3953,7 +3956,7 @@
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3965,10 +3968,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3977,10 +3980,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3988,7 +3991,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4000,10 +4003,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4012,10 +4015,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4023,7 +4026,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4035,10 +4038,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4047,10 +4050,10 @@
         <v>149</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4058,7 +4061,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4070,10 +4073,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4082,10 +4085,10 @@
         <v>149</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4093,7 +4096,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4105,10 +4108,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4117,10 +4120,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4128,7 +4131,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4140,10 +4143,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4152,10 +4155,10 @@
         <v>149</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4163,7 +4166,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4175,10 +4178,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4187,10 +4190,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4198,7 +4201,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4210,10 +4213,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4222,10 +4225,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4233,7 +4236,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4245,10 +4248,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4257,10 +4260,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4268,7 +4271,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4277,13 +4280,13 @@
         <v>195</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4292,10 +4295,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4303,7 +4306,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4312,13 +4315,13 @@
         <v>195</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4327,10 +4330,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4338,7 +4341,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4347,13 +4350,13 @@
         <v>195</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4362,10 +4365,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4373,7 +4376,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4382,13 +4385,13 @@
         <v>195</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4397,10 +4400,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4408,7 +4411,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4417,13 +4420,13 @@
         <v>195</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4432,10 +4435,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4443,7 +4446,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4452,13 +4455,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4467,10 +4470,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4478,7 +4481,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4487,13 +4490,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4502,10 +4505,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4513,7 +4516,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4522,13 +4525,13 @@
         <v>195</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4537,10 +4540,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4548,7 +4551,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4557,13 +4560,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4572,10 +4575,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4583,7 +4586,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4592,13 +4595,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4607,10 +4610,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4618,7 +4621,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4627,13 +4630,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4642,10 +4645,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4653,7 +4656,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4662,13 +4665,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4677,10 +4680,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4688,7 +4691,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4697,13 +4700,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4712,10 +4715,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4723,7 +4726,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4732,13 +4735,13 @@
         <v>195</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4747,10 +4750,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4758,7 +4761,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4767,13 +4770,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4782,10 +4785,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4793,7 +4796,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4802,13 +4805,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4817,10 +4820,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4828,7 +4831,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4837,13 +4840,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4852,10 +4855,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4863,7 +4866,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4872,13 +4875,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4887,10 +4890,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4898,7 +4901,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4907,13 +4910,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4922,10 +4925,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4933,7 +4936,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4942,13 +4945,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4957,10 +4960,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4968,7 +4971,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4977,13 +4980,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4992,10 +4995,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5003,7 +5006,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5012,13 +5015,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5027,10 +5030,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5038,7 +5041,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5047,13 +5050,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5062,10 +5065,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5073,7 +5076,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5085,10 +5088,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5097,10 +5100,10 @@
         <v>149</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5108,7 +5111,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5120,10 +5123,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5132,10 +5135,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5143,7 +5146,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5155,10 +5158,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5167,10 +5170,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5178,7 +5181,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5187,13 +5190,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5202,10 +5205,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5213,7 +5216,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5222,13 +5225,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5237,10 +5240,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5248,7 +5251,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5257,13 +5260,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5272,10 +5275,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5283,7 +5286,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5292,13 +5295,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5307,10 +5310,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5318,7 +5321,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5327,13 +5330,13 @@
         <v>195</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5342,10 +5345,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5353,7 +5356,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5362,13 +5365,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5377,10 +5380,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5388,7 +5391,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5397,13 +5400,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5412,10 +5415,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5423,7 +5426,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5432,13 +5435,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5447,10 +5450,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5458,22 +5461,22 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D71" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5482,10 +5485,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5493,7 +5496,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5505,10 +5508,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5517,10 +5520,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5528,22 +5531,22 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5552,10 +5555,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5563,7 +5566,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5575,10 +5578,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5587,10 +5590,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5598,22 +5601,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5625,7 +5628,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5633,22 +5636,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5660,7 +5663,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5668,22 +5671,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5692,10 +5695,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5703,22 +5706,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5727,10 +5730,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5738,22 +5741,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5762,10 +5765,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5773,22 +5776,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5800,7 +5803,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5808,22 +5811,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5835,7 +5838,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5843,22 +5846,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5867,10 +5870,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5878,22 +5881,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5902,10 +5905,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5913,10 +5916,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5925,10 +5928,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5937,10 +5940,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5980,12 +5983,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5999,19 +6002,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6034,10 +6037,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6060,10 +6063,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6086,10 +6089,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6112,7 +6115,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6136,7 +6139,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6160,10 +6163,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6186,7 +6189,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6210,7 +6213,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6234,10 +6237,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>497</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6260,7 +6263,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6284,7 +6287,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6308,7 +6311,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6332,7 +6335,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6356,15 +6359,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6372,7 +6375,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6380,7 +6383,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6409,7 +6412,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6426,10 +6429,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6437,7 +6440,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6446,10 +6449,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6457,7 +6460,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6469,7 +6472,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6477,7 +6480,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6486,10 +6489,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6497,7 +6500,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6506,10 +6509,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6523,18 +6526,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6543,53 +6546,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
   </sheetData>
@@ -6614,26 +6617,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6641,13 +6644,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6655,13 +6658,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6669,13 +6672,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6683,13 +6686,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6697,13 +6700,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6711,13 +6714,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6725,13 +6728,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6739,13 +6742,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6753,13 +6756,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6767,13 +6770,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6781,21 +6784,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6831,7 +6834,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6839,7 +6842,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6851,167 +6854,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -7043,7 +7046,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7063,47 +7066,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7114,16 +7117,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7131,19 +7134,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7151,19 +7154,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7171,19 +7174,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W00-12: mark Done in workbook (PR #3 — preview URL + green check verified)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="585">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -633,6 +633,9 @@
   </si>
   <si>
     <t>A PR produces a preview URL and a green check</t>
+  </si>
+  <si>
+    <t>✅ Done (a469d5e)</t>
   </si>
   <si>
     <t>W00-13</t>
@@ -3566,12 +3569,12 @@
         <v>203</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>151</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>51</v>
@@ -3583,10 +3586,10 @@
         <v>146</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G17" s="12">
         <v>0.75</v>
@@ -3598,7 +3601,7 @@
         <v>200</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>151</v>
@@ -3606,7 +3609,7 @@
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>51</v>
@@ -3618,10 +3621,10 @@
         <v>146</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G18" s="12">
         <v>0.5</v>
@@ -3630,10 +3633,10 @@
         <v>149</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>151</v>
@@ -3641,7 +3644,7 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>51</v>
@@ -3650,13 +3653,13 @@
         <v>195</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G19" s="12">
         <v>0.5</v>
@@ -3668,15 +3671,15 @@
         <v>61</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -3688,10 +3691,10 @@
         <v>190</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G20" s="12">
         <v>0.25</v>
@@ -3703,7 +3706,7 @@
         <v>189</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>151</v>
@@ -3711,7 +3714,7 @@
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
@@ -3723,10 +3726,10 @@
         <v>70</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G21" s="12">
         <v>0.5</v>
@@ -3735,10 +3738,10 @@
         <v>149</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>151</v>
@@ -3746,7 +3749,7 @@
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -3758,10 +3761,10 @@
         <v>177</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G22" s="12">
         <v>0.25</v>
@@ -3773,7 +3776,7 @@
         <v>61</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K22" s="11" t="s">
         <v>151</v>
@@ -3781,7 +3784,7 @@
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
@@ -3793,10 +3796,10 @@
         <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G23" s="12">
         <v>0.5</v>
@@ -3808,30 +3811,30 @@
         <v>61</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G24" s="12">
         <v>0.25</v>
@@ -3840,10 +3843,10 @@
         <v>149</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>151</v>
@@ -3851,7 +3854,7 @@
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>57</v>
@@ -3863,10 +3866,10 @@
         <v>146</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G25" s="12">
         <v>3</v>
@@ -3878,7 +3881,7 @@
         <v>144</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>151</v>
@@ -3886,7 +3889,7 @@
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3898,10 +3901,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3910,10 +3913,10 @@
         <v>149</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>151</v>
@@ -3921,7 +3924,7 @@
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3933,10 +3936,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3945,10 +3948,10 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>151</v>
@@ -3956,7 +3959,7 @@
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3968,10 +3971,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3980,10 +3983,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3991,7 +3994,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4003,10 +4006,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4015,10 +4018,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4026,7 +4029,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4038,10 +4041,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4050,10 +4053,10 @@
         <v>149</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4061,7 +4064,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4073,10 +4076,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4085,10 +4088,10 @@
         <v>149</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4096,7 +4099,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4108,10 +4111,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4120,10 +4123,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4131,7 +4134,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4143,10 +4146,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4155,10 +4158,10 @@
         <v>149</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4166,7 +4169,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4178,10 +4181,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4190,10 +4193,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4201,7 +4204,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4213,10 +4216,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4225,10 +4228,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4236,7 +4239,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4248,10 +4251,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4260,10 +4263,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4271,7 +4274,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4280,13 +4283,13 @@
         <v>195</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4295,10 +4298,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4306,7 +4309,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4315,13 +4318,13 @@
         <v>195</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4330,10 +4333,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4341,7 +4344,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4350,13 +4353,13 @@
         <v>195</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4365,10 +4368,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4376,7 +4379,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4385,13 +4388,13 @@
         <v>195</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4400,10 +4403,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4411,7 +4414,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4420,13 +4423,13 @@
         <v>195</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4435,10 +4438,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4446,7 +4449,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4455,13 +4458,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4470,10 +4473,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4481,7 +4484,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4490,13 +4493,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4505,10 +4508,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4516,7 +4519,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4525,13 +4528,13 @@
         <v>195</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4540,10 +4543,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4551,7 +4554,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4560,13 +4563,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4575,10 +4578,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4586,7 +4589,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4595,13 +4598,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4610,10 +4613,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4621,7 +4624,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4630,13 +4633,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4645,10 +4648,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4656,7 +4659,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4665,13 +4668,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4680,10 +4683,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4691,7 +4694,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4700,13 +4703,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4715,10 +4718,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4726,7 +4729,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4735,13 +4738,13 @@
         <v>195</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4750,10 +4753,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4761,7 +4764,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4770,13 +4773,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4785,10 +4788,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4796,7 +4799,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4805,13 +4808,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4820,10 +4823,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4831,7 +4834,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4840,13 +4843,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4855,10 +4858,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4866,7 +4869,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4875,13 +4878,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4890,10 +4893,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4901,7 +4904,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4910,13 +4913,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4925,10 +4928,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4936,7 +4939,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4945,13 +4948,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4960,10 +4963,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4971,7 +4974,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4980,13 +4983,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4995,10 +4998,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5006,7 +5009,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5015,13 +5018,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5030,10 +5033,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5041,7 +5044,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5050,13 +5053,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5065,10 +5068,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5076,7 +5079,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5088,10 +5091,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5100,10 +5103,10 @@
         <v>149</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5111,7 +5114,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5123,10 +5126,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5135,10 +5138,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5146,7 +5149,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5158,10 +5161,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5170,10 +5173,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5181,7 +5184,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5190,13 +5193,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5205,10 +5208,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5216,7 +5219,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5225,13 +5228,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5240,10 +5243,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5251,7 +5254,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5260,13 +5263,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5275,10 +5278,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5286,7 +5289,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5295,13 +5298,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5310,10 +5313,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5321,7 +5324,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5330,13 +5333,13 @@
         <v>195</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5345,10 +5348,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5356,7 +5359,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5365,13 +5368,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5380,10 +5383,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5391,7 +5394,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5400,13 +5403,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5415,10 +5418,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5426,7 +5429,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5435,13 +5438,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5450,10 +5453,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5461,22 +5464,22 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D71" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5485,10 +5488,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5496,7 +5499,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5508,10 +5511,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5520,10 +5523,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5531,22 +5534,22 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5555,10 +5558,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5566,7 +5569,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5578,10 +5581,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5590,10 +5593,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5601,22 +5604,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5628,7 +5631,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5636,22 +5639,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5663,7 +5666,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5671,22 +5674,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5695,10 +5698,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5706,22 +5709,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5730,10 +5733,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5741,22 +5744,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5765,10 +5768,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5776,22 +5779,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5803,7 +5806,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5811,22 +5814,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5838,7 +5841,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5846,22 +5849,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5870,10 +5873,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5881,22 +5884,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5905,10 +5908,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5916,10 +5919,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5928,10 +5931,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5940,10 +5943,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5983,12 +5986,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6002,19 +6005,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6037,10 +6040,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6063,10 +6066,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6089,10 +6092,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6115,7 +6118,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6139,7 +6142,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6163,10 +6166,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6189,7 +6192,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6213,7 +6216,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6237,10 +6240,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6263,7 +6266,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6287,7 +6290,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6311,7 +6314,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6335,7 +6338,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6359,15 +6362,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6375,7 +6378,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6383,7 +6386,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6412,7 +6415,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6429,10 +6432,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6440,7 +6443,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6449,10 +6452,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6460,7 +6463,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6472,7 +6475,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6480,7 +6483,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6489,10 +6492,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6500,7 +6503,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6509,10 +6512,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6526,18 +6529,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6546,53 +6549,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
   </sheetData>
@@ -6617,26 +6620,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6644,13 +6647,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6658,13 +6661,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6672,13 +6675,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6686,13 +6689,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6700,13 +6703,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6714,13 +6717,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6728,13 +6731,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6742,13 +6745,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6756,13 +6759,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6770,13 +6773,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6784,21 +6787,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6834,7 +6837,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6842,7 +6845,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6854,167 +6857,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
   </sheetData>
@@ -7046,7 +7049,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7066,47 +7069,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7117,16 +7120,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7134,19 +7137,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7154,19 +7157,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7174,19 +7177,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W00-12: mark Done in workbook (PR #3 — preview URL + green check verified) (#4)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="585">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -633,6 +633,9 @@
   </si>
   <si>
     <t>A PR produces a preview URL and a green check</t>
+  </si>
+  <si>
+    <t>✅ Done (a469d5e)</t>
   </si>
   <si>
     <t>W00-13</t>
@@ -3566,12 +3569,12 @@
         <v>203</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>151</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>51</v>
@@ -3583,10 +3586,10 @@
         <v>146</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G17" s="12">
         <v>0.75</v>
@@ -3598,7 +3601,7 @@
         <v>200</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>151</v>
@@ -3606,7 +3609,7 @@
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>51</v>
@@ -3618,10 +3621,10 @@
         <v>146</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G18" s="12">
         <v>0.5</v>
@@ -3630,10 +3633,10 @@
         <v>149</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>151</v>
@@ -3641,7 +3644,7 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>51</v>
@@ -3650,13 +3653,13 @@
         <v>195</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G19" s="12">
         <v>0.5</v>
@@ -3668,15 +3671,15 @@
         <v>61</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -3688,10 +3691,10 @@
         <v>190</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G20" s="12">
         <v>0.25</v>
@@ -3703,7 +3706,7 @@
         <v>189</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>151</v>
@@ -3711,7 +3714,7 @@
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
@@ -3723,10 +3726,10 @@
         <v>70</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G21" s="12">
         <v>0.5</v>
@@ -3735,10 +3738,10 @@
         <v>149</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>151</v>
@@ -3746,7 +3749,7 @@
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -3758,10 +3761,10 @@
         <v>177</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G22" s="12">
         <v>0.25</v>
@@ -3773,7 +3776,7 @@
         <v>61</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K22" s="11" t="s">
         <v>151</v>
@@ -3781,7 +3784,7 @@
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
@@ -3793,10 +3796,10 @@
         <v>107</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G23" s="12">
         <v>0.5</v>
@@ -3808,30 +3811,30 @@
         <v>61</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G24" s="12">
         <v>0.25</v>
@@ -3840,10 +3843,10 @@
         <v>149</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>151</v>
@@ -3851,7 +3854,7 @@
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>57</v>
@@ -3863,10 +3866,10 @@
         <v>146</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G25" s="12">
         <v>3</v>
@@ -3878,7 +3881,7 @@
         <v>144</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>151</v>
@@ -3886,7 +3889,7 @@
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3898,10 +3901,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3910,10 +3913,10 @@
         <v>149</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>151</v>
@@ -3921,7 +3924,7 @@
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3933,10 +3936,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3945,10 +3948,10 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>151</v>
@@ -3956,7 +3959,7 @@
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3968,10 +3971,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3980,10 +3983,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3991,7 +3994,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4003,10 +4006,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4015,10 +4018,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4026,7 +4029,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4038,10 +4041,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4050,10 +4053,10 @@
         <v>149</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4061,7 +4064,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4073,10 +4076,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4085,10 +4088,10 @@
         <v>149</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4096,7 +4099,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4108,10 +4111,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4120,10 +4123,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4131,7 +4134,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4143,10 +4146,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4155,10 +4158,10 @@
         <v>149</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4166,7 +4169,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4178,10 +4181,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4190,10 +4193,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4201,7 +4204,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4213,10 +4216,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4225,10 +4228,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4236,7 +4239,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4248,10 +4251,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4260,10 +4263,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4271,7 +4274,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4280,13 +4283,13 @@
         <v>195</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4295,10 +4298,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4306,7 +4309,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4315,13 +4318,13 @@
         <v>195</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4330,10 +4333,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4341,7 +4344,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4350,13 +4353,13 @@
         <v>195</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4365,10 +4368,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4376,7 +4379,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4385,13 +4388,13 @@
         <v>195</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4400,10 +4403,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4411,7 +4414,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4420,13 +4423,13 @@
         <v>195</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4435,10 +4438,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4446,7 +4449,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4455,13 +4458,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4470,10 +4473,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4481,7 +4484,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4490,13 +4493,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4505,10 +4508,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4516,7 +4519,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4525,13 +4528,13 @@
         <v>195</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4540,10 +4543,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4551,7 +4554,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4560,13 +4563,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4575,10 +4578,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4586,7 +4589,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4595,13 +4598,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4610,10 +4613,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4621,7 +4624,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4630,13 +4633,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4645,10 +4648,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4656,7 +4659,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4665,13 +4668,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4680,10 +4683,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4691,7 +4694,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4700,13 +4703,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4715,10 +4718,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4726,7 +4729,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4735,13 +4738,13 @@
         <v>195</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4750,10 +4753,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4761,7 +4764,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4770,13 +4773,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4785,10 +4788,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4796,7 +4799,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4805,13 +4808,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4820,10 +4823,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4831,7 +4834,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4840,13 +4843,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4855,10 +4858,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4866,7 +4869,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4875,13 +4878,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4890,10 +4893,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4901,7 +4904,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4910,13 +4913,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4925,10 +4928,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4936,7 +4939,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4945,13 +4948,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4960,10 +4963,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4971,7 +4974,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4980,13 +4983,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4995,10 +4998,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5006,7 +5009,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5015,13 +5018,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5030,10 +5033,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5041,7 +5044,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5050,13 +5053,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5065,10 +5068,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5076,7 +5079,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5088,10 +5091,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5100,10 +5103,10 @@
         <v>149</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5111,7 +5114,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5123,10 +5126,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5135,10 +5138,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5146,7 +5149,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5158,10 +5161,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5170,10 +5173,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5181,7 +5184,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5190,13 +5193,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5205,10 +5208,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5216,7 +5219,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5225,13 +5228,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5240,10 +5243,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5251,7 +5254,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5260,13 +5263,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5275,10 +5278,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5286,7 +5289,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5295,13 +5298,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5310,10 +5313,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5321,7 +5324,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5330,13 +5333,13 @@
         <v>195</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5345,10 +5348,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5356,7 +5359,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5365,13 +5368,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5380,10 +5383,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5391,7 +5394,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5400,13 +5403,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5415,10 +5418,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5426,7 +5429,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5435,13 +5438,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5450,10 +5453,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5461,22 +5464,22 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D71" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5485,10 +5488,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5496,7 +5499,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5508,10 +5511,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5520,10 +5523,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5531,22 +5534,22 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5555,10 +5558,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5566,7 +5569,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5578,10 +5581,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5590,10 +5593,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5601,22 +5604,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5628,7 +5631,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5636,22 +5639,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5663,7 +5666,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5671,22 +5674,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5695,10 +5698,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5706,22 +5709,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5730,10 +5733,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5741,22 +5744,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5765,10 +5768,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5776,22 +5779,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5803,7 +5806,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5811,22 +5814,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5838,7 +5841,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5846,22 +5849,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5870,10 +5873,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5881,22 +5884,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5905,10 +5908,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5916,10 +5919,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5928,10 +5931,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5940,10 +5943,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5983,12 +5986,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6002,19 +6005,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6037,10 +6040,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6063,10 +6066,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6089,10 +6092,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6115,7 +6118,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6139,7 +6142,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6163,10 +6166,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6189,7 +6192,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6213,7 +6216,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6237,10 +6240,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>498</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6263,7 +6266,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6287,7 +6290,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6311,7 +6314,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6335,7 +6338,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6359,15 +6362,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6375,7 +6378,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6383,7 +6386,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6412,7 +6415,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6429,10 +6432,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6440,7 +6443,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6449,10 +6452,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6460,7 +6463,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6472,7 +6475,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6480,7 +6483,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6489,10 +6492,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6500,7 +6503,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6509,10 +6512,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6526,18 +6529,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6546,53 +6549,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
   </sheetData>
@@ -6617,26 +6620,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6644,13 +6647,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6658,13 +6661,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6672,13 +6675,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6686,13 +6689,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6700,13 +6703,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6714,13 +6717,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6728,13 +6731,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6742,13 +6745,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6756,13 +6759,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6770,13 +6773,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6784,21 +6787,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6834,7 +6837,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6842,7 +6845,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6854,167 +6857,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
   </sheetData>
@@ -7046,7 +7049,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7066,47 +7069,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7117,16 +7120,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7134,19 +7137,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7154,19 +7157,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7174,19 +7177,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S01-01/S01-02/S01-03: mark Done in workbook (PR #5 — schema+RLS+isolation verified)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="588">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -761,6 +761,9 @@
     <t>Runs clean from an empty database; ERD committed</t>
   </si>
   <si>
+    <t>Done (PR #5 — 25/25 db incl. clean-from-empty on scratch; 4 review rounds)</t>
+  </si>
+  <si>
     <t>S01-02</t>
   </si>
   <si>
@@ -773,6 +776,9 @@
     <t>A query without tenant context returns zero rows</t>
   </si>
   <si>
+    <t>Done (PR #5 — zero-row AC asserted on all 21 tenant tables + withTenant guard)</t>
+  </si>
+  <si>
     <t>S01-03</t>
   </si>
   <si>
@@ -783,6 +789,9 @@
   </si>
   <si>
     <t>Suite runs in CI and fails the build on a leak</t>
+  </si>
+  <si>
+    <t>Done (PR #5 — policy-derived enumeration + leak sweep + ci db-test job, 5 review rounds)</t>
   </si>
   <si>
     <t>S02-01</t>
@@ -3884,12 +3893,12 @@
         <v>245</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>151</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3901,10 +3910,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3916,15 +3925,15 @@
         <v>242</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>151</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3936,10 +3945,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3948,18 +3957,18 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>151</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3971,10 +3980,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3986,7 +3995,7 @@
         <v>242</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3994,7 +4003,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4006,10 +4015,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4018,10 +4027,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4029,7 +4038,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4041,10 +4050,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4056,7 +4065,7 @@
         <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4064,7 +4073,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4076,10 +4085,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4091,7 +4100,7 @@
         <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4099,7 +4108,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4111,10 +4120,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4123,10 +4132,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4134,7 +4143,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4146,10 +4155,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4161,7 +4170,7 @@
         <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4169,7 +4178,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4181,10 +4190,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4193,10 +4202,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4204,7 +4213,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4216,10 +4225,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4228,10 +4237,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4239,7 +4248,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4251,10 +4260,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4263,10 +4272,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4274,7 +4283,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4286,10 +4295,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4298,10 +4307,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4309,7 +4318,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4321,10 +4330,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4333,10 +4342,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4344,7 +4353,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4356,10 +4365,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4368,10 +4377,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4379,7 +4388,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4391,10 +4400,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4403,10 +4412,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4414,7 +4423,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4426,10 +4435,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4438,10 +4447,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4449,7 +4458,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4458,13 +4467,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4473,10 +4482,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4484,7 +4493,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4493,13 +4502,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4508,10 +4517,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4519,7 +4528,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4531,10 +4540,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4543,10 +4552,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4554,7 +4563,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4563,13 +4572,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4578,10 +4587,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4589,7 +4598,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4598,13 +4607,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4613,10 +4622,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4624,7 +4633,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4633,13 +4642,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4648,10 +4657,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4659,7 +4668,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4668,13 +4677,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4683,10 +4692,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4694,7 +4703,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4703,13 +4712,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4718,10 +4727,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4729,7 +4738,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4741,10 +4750,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4753,10 +4762,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4764,7 +4773,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4773,13 +4782,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4788,10 +4797,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4799,7 +4808,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4808,13 +4817,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4823,10 +4832,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4834,7 +4843,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4843,13 +4852,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4858,10 +4867,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4869,7 +4878,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4878,13 +4887,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4893,10 +4902,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4904,7 +4913,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4913,13 +4922,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4928,10 +4937,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4939,7 +4948,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4948,13 +4957,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4963,10 +4972,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4974,7 +4983,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4983,13 +4992,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4998,10 +5007,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5009,7 +5018,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5018,13 +5027,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5033,10 +5042,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5044,7 +5053,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5053,13 +5062,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5068,10 +5077,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5079,7 +5088,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5091,10 +5100,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5106,7 +5115,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5114,7 +5123,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5126,10 +5135,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5138,10 +5147,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5149,7 +5158,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5161,10 +5170,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5173,10 +5182,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5184,7 +5193,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5193,13 +5202,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5208,10 +5217,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5219,7 +5228,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5228,13 +5237,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5243,10 +5252,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5254,7 +5263,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5263,13 +5272,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5278,10 +5287,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5289,7 +5298,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5298,13 +5307,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5313,10 +5322,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5324,7 +5333,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5336,10 +5345,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5348,10 +5357,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5359,7 +5368,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5368,13 +5377,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5383,10 +5392,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5394,7 +5403,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5403,13 +5412,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5418,10 +5427,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5429,7 +5438,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5438,13 +5447,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5453,10 +5462,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5464,7 +5473,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5476,10 +5485,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5488,10 +5497,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5499,7 +5508,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5511,10 +5520,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5523,10 +5532,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5534,7 +5543,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5546,10 +5555,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5558,10 +5567,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5569,7 +5578,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5581,10 +5590,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5593,10 +5602,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5604,22 +5613,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5631,7 +5640,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5639,22 +5648,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5666,7 +5675,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5674,22 +5683,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5698,10 +5707,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5709,22 +5718,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5733,10 +5742,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5744,22 +5753,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5768,10 +5777,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5779,22 +5788,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5806,7 +5815,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5814,22 +5823,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5841,7 +5850,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5849,22 +5858,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5873,10 +5882,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5884,22 +5893,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5908,10 +5917,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5919,10 +5928,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5931,10 +5940,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5943,10 +5952,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5986,12 +5995,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6005,19 +6014,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6040,10 +6049,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6066,10 +6075,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6092,10 +6101,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6118,7 +6127,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6142,7 +6151,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6166,10 +6175,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6192,7 +6201,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6216,7 +6225,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6240,10 +6249,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6266,7 +6275,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6290,7 +6299,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6314,7 +6323,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6338,7 +6347,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6362,15 +6371,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6378,7 +6387,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6386,7 +6395,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6415,7 +6424,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6432,10 +6441,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6443,7 +6452,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6452,10 +6461,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6463,7 +6472,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6475,7 +6484,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6483,7 +6492,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6492,10 +6501,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6503,7 +6512,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6512,10 +6521,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6529,18 +6538,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6549,53 +6558,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -6620,26 +6629,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6647,13 +6656,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6661,13 +6670,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6675,13 +6684,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6689,13 +6698,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6703,13 +6712,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6717,13 +6726,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6731,13 +6740,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6745,13 +6754,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6759,13 +6768,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6773,13 +6782,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6787,21 +6796,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6837,7 +6846,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6845,7 +6854,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6857,167 +6866,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>
@@ -7049,7 +7058,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7069,47 +7078,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7120,16 +7129,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7137,19 +7146,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7157,19 +7166,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7177,19 +7186,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S01-01/S01-02/S01-03: mark Done in workbook (PR #5 — schema+RLS+isolation verified) (#6)
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="588">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -761,6 +761,9 @@
     <t>Runs clean from an empty database; ERD committed</t>
   </si>
   <si>
+    <t>Done (PR #5 — 25/25 db incl. clean-from-empty on scratch; 4 review rounds)</t>
+  </si>
+  <si>
     <t>S01-02</t>
   </si>
   <si>
@@ -773,6 +776,9 @@
     <t>A query without tenant context returns zero rows</t>
   </si>
   <si>
+    <t>Done (PR #5 — zero-row AC asserted on all 21 tenant tables + withTenant guard)</t>
+  </si>
+  <si>
     <t>S01-03</t>
   </si>
   <si>
@@ -783,6 +789,9 @@
   </si>
   <si>
     <t>Suite runs in CI and fails the build on a leak</t>
+  </si>
+  <si>
+    <t>Done (PR #5 — policy-derived enumeration + leak sweep + ci db-test job, 5 review rounds)</t>
   </si>
   <si>
     <t>S02-01</t>
@@ -3884,12 +3893,12 @@
         <v>245</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>151</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>57</v>
@@ -3901,10 +3910,10 @@
         <v>146</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G26" s="12">
         <v>2</v>
@@ -3916,15 +3925,15 @@
         <v>242</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>151</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>57</v>
@@ -3936,10 +3945,10 @@
         <v>146</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G27" s="12">
         <v>0.75</v>
@@ -3948,18 +3957,18 @@
         <v>149</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>151</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>63</v>
@@ -3971,10 +3980,10 @@
         <v>146</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G28" s="12">
         <v>2</v>
@@ -3986,7 +3995,7 @@
         <v>242</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="K28" s="11" t="s">
         <v>151</v>
@@ -3994,7 +4003,7 @@
     </row>
     <row r="29" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>63</v>
@@ -4006,10 +4015,10 @@
         <v>146</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G29" s="12">
         <v>1</v>
@@ -4018,10 +4027,10 @@
         <v>149</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="K29" s="11" t="s">
         <v>151</v>
@@ -4029,7 +4038,7 @@
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4041,10 +4050,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4056,7 +4065,7 @@
         <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4064,7 +4073,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4076,10 +4085,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4091,7 +4100,7 @@
         <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4099,7 +4108,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4111,10 +4120,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4123,10 +4132,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4134,7 +4143,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4146,10 +4155,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4161,7 +4170,7 @@
         <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4169,7 +4178,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4181,10 +4190,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4193,10 +4202,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4204,7 +4213,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4216,10 +4225,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4228,10 +4237,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4239,7 +4248,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4251,10 +4260,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4263,10 +4272,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4274,7 +4283,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4286,10 +4295,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4298,10 +4307,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4309,7 +4318,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4321,10 +4330,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4333,10 +4342,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4344,7 +4353,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4356,10 +4365,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4368,10 +4377,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4379,7 +4388,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4391,10 +4400,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4403,10 +4412,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4414,7 +4423,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4426,10 +4435,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4438,10 +4447,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4449,7 +4458,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4458,13 +4467,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4473,10 +4482,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4484,7 +4493,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4493,13 +4502,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4508,10 +4517,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4519,7 +4528,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4531,10 +4540,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4543,10 +4552,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4554,7 +4563,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4563,13 +4572,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4578,10 +4587,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4589,7 +4598,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4598,13 +4607,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4613,10 +4622,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4624,7 +4633,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4633,13 +4642,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4648,10 +4657,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4659,7 +4668,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4668,13 +4677,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4683,10 +4692,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4694,7 +4703,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4703,13 +4712,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4718,10 +4727,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4729,7 +4738,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4741,10 +4750,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4753,10 +4762,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4764,7 +4773,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4773,13 +4782,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4788,10 +4797,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4799,7 +4808,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4808,13 +4817,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4823,10 +4832,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4834,7 +4843,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4843,13 +4852,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4858,10 +4867,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4869,7 +4878,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4878,13 +4887,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4893,10 +4902,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4904,7 +4913,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4913,13 +4922,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4928,10 +4937,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4939,7 +4948,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4948,13 +4957,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4963,10 +4972,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4974,7 +4983,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4983,13 +4992,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -4998,10 +5007,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5009,7 +5018,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5018,13 +5027,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5033,10 +5042,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5044,7 +5053,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5053,13 +5062,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5068,10 +5077,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5079,7 +5088,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5091,10 +5100,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5106,7 +5115,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5114,7 +5123,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5126,10 +5135,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5138,10 +5147,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5149,7 +5158,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5161,10 +5170,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5173,10 +5182,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5184,7 +5193,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5193,13 +5202,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5208,10 +5217,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5219,7 +5228,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5228,13 +5237,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5243,10 +5252,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5254,7 +5263,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5263,13 +5272,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5278,10 +5287,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5289,7 +5298,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5298,13 +5307,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5313,10 +5322,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5324,7 +5333,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5336,10 +5345,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5348,10 +5357,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5359,7 +5368,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5368,13 +5377,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5383,10 +5392,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5394,7 +5403,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5403,13 +5412,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5418,10 +5427,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5429,7 +5438,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5438,13 +5447,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5453,10 +5462,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5464,7 +5473,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5476,10 +5485,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5488,10 +5497,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5499,7 +5508,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5511,10 +5520,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5523,10 +5532,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5534,7 +5543,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5546,10 +5555,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5558,10 +5567,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5569,7 +5578,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5581,10 +5590,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5593,10 +5602,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5604,22 +5613,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5631,7 +5640,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5639,22 +5648,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5666,7 +5675,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5674,22 +5683,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5698,10 +5707,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5709,22 +5718,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5733,10 +5742,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5744,22 +5753,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5768,10 +5777,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5779,22 +5788,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5806,7 +5815,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5814,22 +5823,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5841,7 +5850,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5849,22 +5858,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5873,10 +5882,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5884,22 +5893,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5908,10 +5917,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5919,10 +5928,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5931,10 +5940,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5943,10 +5952,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5986,12 +5995,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6005,19 +6014,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6040,10 +6049,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6066,10 +6075,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6092,10 +6101,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6118,7 +6127,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6142,7 +6151,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6166,10 +6175,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6192,7 +6201,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6216,7 +6225,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6240,10 +6249,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6266,7 +6275,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6290,7 +6299,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6314,7 +6323,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6338,7 +6347,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6362,15 +6371,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6378,7 +6387,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6386,7 +6395,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6415,7 +6424,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6432,10 +6441,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6443,7 +6452,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6452,10 +6461,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6463,7 +6472,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6475,7 +6484,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6483,7 +6492,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6492,10 +6501,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6503,7 +6512,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6512,10 +6521,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6529,18 +6538,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6549,53 +6558,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -6620,26 +6629,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6647,13 +6656,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6661,13 +6670,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6675,13 +6684,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6689,13 +6698,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6703,13 +6712,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6717,13 +6726,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6731,13 +6740,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6745,13 +6754,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6759,13 +6768,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6773,13 +6782,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6787,21 +6796,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6837,7 +6846,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6845,7 +6854,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6857,167 +6866,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>
@@ -7049,7 +7058,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7069,47 +7078,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7120,16 +7129,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7137,19 +7146,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7157,19 +7166,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7177,19 +7186,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S02-02: mark Done in workbook
AC met and verified on main (PR #15): 0006 validator/default/language CHECK,
path-aware parser, pure policy, RLS-scoped store. 62 db / 94 unit, CI green.
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="589">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -816,6 +816,9 @@
   </si>
   <si>
     <t>AI policy layer reads settings, does not hardcode</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
   <si>
     <t>S02-03</t>
@@ -4033,12 +4036,12 @@
         <v>264</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>151</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4050,10 +4053,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4065,7 +4068,7 @@
         <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4073,7 +4076,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4085,10 +4088,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4100,7 +4103,7 @@
         <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4108,7 +4111,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4120,10 +4123,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4132,10 +4135,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4143,7 +4146,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4155,10 +4158,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4170,7 +4173,7 @@
         <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4178,7 +4181,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4190,10 +4193,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4202,10 +4205,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4213,7 +4216,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4225,10 +4228,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4237,10 +4240,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4248,7 +4251,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4260,10 +4263,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4272,10 +4275,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4283,7 +4286,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4295,10 +4298,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4307,10 +4310,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4318,7 +4321,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4330,10 +4333,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4342,10 +4345,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4353,7 +4356,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4365,10 +4368,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4377,10 +4380,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4388,7 +4391,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4400,10 +4403,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4412,10 +4415,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4423,7 +4426,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4435,10 +4438,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4447,10 +4450,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4458,7 +4461,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4467,13 +4470,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4482,10 +4485,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4493,7 +4496,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4502,13 +4505,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4517,10 +4520,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4528,7 +4531,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4540,10 +4543,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4552,10 +4555,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4563,7 +4566,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4572,13 +4575,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4587,10 +4590,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4598,7 +4601,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4607,13 +4610,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4622,10 +4625,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4633,7 +4636,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4642,13 +4645,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4657,10 +4660,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4668,7 +4671,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4677,13 +4680,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4692,10 +4695,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4703,7 +4706,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4712,13 +4715,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4727,10 +4730,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4738,7 +4741,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4750,10 +4753,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4762,10 +4765,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4773,7 +4776,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4782,13 +4785,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4797,10 +4800,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4808,7 +4811,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4817,13 +4820,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4832,10 +4835,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4843,7 +4846,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4852,13 +4855,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4867,10 +4870,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4878,7 +4881,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4887,13 +4890,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4902,10 +4905,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4913,7 +4916,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4922,13 +4925,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4937,10 +4940,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4948,7 +4951,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4957,13 +4960,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4972,10 +4975,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4983,7 +4986,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4992,13 +4995,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5007,10 +5010,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5018,7 +5021,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5027,13 +5030,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5042,10 +5045,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5053,7 +5056,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5062,13 +5065,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5077,10 +5080,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5088,7 +5091,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5100,10 +5103,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5115,7 +5118,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5123,7 +5126,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5135,10 +5138,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5147,10 +5150,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5158,7 +5161,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5170,10 +5173,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5182,10 +5185,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5193,7 +5196,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5202,13 +5205,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5217,10 +5220,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5228,7 +5231,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5237,13 +5240,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5252,10 +5255,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5263,7 +5266,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5272,13 +5275,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5287,10 +5290,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5298,7 +5301,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5307,13 +5310,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5322,10 +5325,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5333,7 +5336,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5345,10 +5348,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5357,10 +5360,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5368,7 +5371,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5377,13 +5380,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5392,10 +5395,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5403,7 +5406,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5412,13 +5415,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5427,10 +5430,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5438,7 +5441,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5447,13 +5450,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5462,10 +5465,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5473,7 +5476,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5485,10 +5488,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5497,10 +5500,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5508,7 +5511,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5520,10 +5523,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5532,10 +5535,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5543,7 +5546,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5555,10 +5558,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5567,10 +5570,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5578,7 +5581,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5590,10 +5593,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5602,10 +5605,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5613,22 +5616,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5640,7 +5643,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5648,22 +5651,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5675,7 +5678,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5683,22 +5686,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5707,10 +5710,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5718,22 +5721,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5742,10 +5745,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5753,22 +5756,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5777,10 +5780,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5788,22 +5791,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5815,7 +5818,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5823,22 +5826,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5850,7 +5853,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5858,22 +5861,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5882,10 +5885,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5893,22 +5896,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5917,10 +5920,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5928,10 +5931,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5940,10 +5943,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5952,10 +5955,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5995,12 +5998,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6014,19 +6017,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6049,10 +6052,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6075,10 +6078,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6101,10 +6104,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6127,7 +6130,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6151,7 +6154,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6175,10 +6178,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6201,7 +6204,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6225,7 +6228,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6249,10 +6252,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6275,7 +6278,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6299,7 +6302,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6323,7 +6326,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6347,7 +6350,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6371,15 +6374,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6387,7 +6390,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6395,7 +6398,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6424,7 +6427,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6441,10 +6444,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6452,7 +6455,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6461,10 +6464,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6472,7 +6475,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6484,7 +6487,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6492,7 +6495,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6501,10 +6504,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6512,7 +6515,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6521,10 +6524,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6538,18 +6541,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6558,53 +6561,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
   </sheetData>
@@ -6629,26 +6632,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6656,13 +6659,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6670,13 +6673,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6684,13 +6687,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6698,13 +6701,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6712,13 +6715,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6726,13 +6729,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6740,13 +6743,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6754,13 +6757,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6768,13 +6771,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6782,13 +6785,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6796,21 +6799,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6846,7 +6849,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6854,7 +6857,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6866,167 +6869,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -7058,7 +7061,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7078,47 +7081,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7129,16 +7132,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7146,19 +7149,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7166,19 +7169,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7186,19 +7189,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S02-02: mark Done in workbook (#16)
Workbook status follows the merged S02-02 implementation (PR #15) and its green CI evidence.
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="589">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -816,6 +816,9 @@
   </si>
   <si>
     <t>AI policy layer reads settings, does not hardcode</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
   <si>
     <t>S02-03</t>
@@ -4033,12 +4036,12 @@
         <v>264</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>151</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
@@ -4050,10 +4053,10 @@
         <v>146</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G30" s="12">
         <v>1</v>
@@ -4065,7 +4068,7 @@
         <v>242</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K30" s="11" t="s">
         <v>151</v>
@@ -4073,7 +4076,7 @@
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>63</v>
@@ -4085,10 +4088,10 @@
         <v>146</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G31" s="12">
         <v>1</v>
@@ -4100,7 +4103,7 @@
         <v>242</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K31" s="11" t="s">
         <v>151</v>
@@ -4108,7 +4111,7 @@
     </row>
     <row r="32" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>63</v>
@@ -4120,10 +4123,10 @@
         <v>70</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G32" s="12">
         <v>0.5</v>
@@ -4132,10 +4135,10 @@
         <v>149</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>151</v>
@@ -4143,7 +4146,7 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>68</v>
@@ -4155,10 +4158,10 @@
         <v>70</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G33" s="12">
         <v>2</v>
@@ -4170,7 +4173,7 @@
         <v>242</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>151</v>
@@ -4178,7 +4181,7 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4190,10 +4193,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4202,10 +4205,10 @@
         <v>149</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4213,7 +4216,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4225,10 +4228,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4237,10 +4240,10 @@
         <v>149</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4248,7 +4251,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4260,10 +4263,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4272,10 +4275,10 @@
         <v>149</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4283,7 +4286,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4295,10 +4298,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4307,10 +4310,10 @@
         <v>149</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4318,7 +4321,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4330,10 +4333,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4342,10 +4345,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4353,7 +4356,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4365,10 +4368,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4377,10 +4380,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4388,7 +4391,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4400,10 +4403,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4412,10 +4415,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4423,7 +4426,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4435,10 +4438,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4447,10 +4450,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4458,7 +4461,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4467,13 +4470,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4482,10 +4485,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4493,7 +4496,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4502,13 +4505,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4517,10 +4520,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4528,7 +4531,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4540,10 +4543,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4552,10 +4555,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4563,7 +4566,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4572,13 +4575,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4587,10 +4590,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4598,7 +4601,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4607,13 +4610,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4622,10 +4625,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4633,7 +4636,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4642,13 +4645,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4657,10 +4660,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4668,7 +4671,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4677,13 +4680,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4692,10 +4695,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4703,7 +4706,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4712,13 +4715,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4727,10 +4730,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4738,7 +4741,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4750,10 +4753,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4762,10 +4765,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4773,7 +4776,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4782,13 +4785,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4797,10 +4800,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4808,7 +4811,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4817,13 +4820,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4832,10 +4835,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4843,7 +4846,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4852,13 +4855,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4867,10 +4870,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4878,7 +4881,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4887,13 +4890,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4902,10 +4905,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4913,7 +4916,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4922,13 +4925,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4937,10 +4940,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4948,7 +4951,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4957,13 +4960,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4972,10 +4975,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4983,7 +4986,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4992,13 +4995,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5007,10 +5010,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5018,7 +5021,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5027,13 +5030,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5042,10 +5045,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5053,7 +5056,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5062,13 +5065,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5077,10 +5080,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5088,7 +5091,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5100,10 +5103,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5115,7 +5118,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5123,7 +5126,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5135,10 +5138,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5147,10 +5150,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5158,7 +5161,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5170,10 +5173,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5182,10 +5185,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5193,7 +5196,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5202,13 +5205,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5217,10 +5220,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5228,7 +5231,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5237,13 +5240,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5252,10 +5255,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5263,7 +5266,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5272,13 +5275,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5287,10 +5290,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5298,7 +5301,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5307,13 +5310,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5322,10 +5325,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5333,7 +5336,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5345,10 +5348,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5357,10 +5360,10 @@
         <v>149</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5368,7 +5371,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5377,13 +5380,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5392,10 +5395,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5403,7 +5406,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5412,13 +5415,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5427,10 +5430,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5438,7 +5441,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5447,13 +5450,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5462,10 +5465,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5473,7 +5476,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5485,10 +5488,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5497,10 +5500,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5508,7 +5511,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5520,10 +5523,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5532,10 +5535,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5543,7 +5546,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5555,10 +5558,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5567,10 +5570,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5578,7 +5581,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5590,10 +5593,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5602,10 +5605,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5613,22 +5616,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5640,7 +5643,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5648,22 +5651,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5675,7 +5678,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5683,22 +5686,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5707,10 +5710,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5718,22 +5721,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5742,10 +5745,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5753,22 +5756,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5777,10 +5780,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5788,22 +5791,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5815,7 +5818,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5823,22 +5826,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5850,7 +5853,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5858,22 +5861,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5882,10 +5885,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5893,22 +5896,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5917,10 +5920,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5928,10 +5931,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5940,10 +5943,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5952,10 +5955,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5995,12 +5998,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6014,19 +6017,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6049,10 +6052,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6075,10 +6078,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6101,10 +6104,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6127,7 +6130,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6151,7 +6154,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6175,10 +6178,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6201,7 +6204,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6225,7 +6228,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6249,10 +6252,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6275,7 +6278,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6299,7 +6302,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6323,7 +6326,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6347,7 +6350,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6371,15 +6374,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6387,7 +6390,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6395,7 +6398,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6424,7 +6427,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6441,10 +6444,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6452,7 +6455,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6461,10 +6464,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6472,7 +6475,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6484,7 +6487,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6492,7 +6495,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6501,10 +6504,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6512,7 +6515,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6521,10 +6524,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6538,18 +6541,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6558,53 +6561,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
   </sheetData>
@@ -6629,26 +6632,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6656,13 +6659,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6670,13 +6673,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6684,13 +6687,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6698,13 +6701,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6712,13 +6715,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6726,13 +6729,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6740,13 +6743,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6754,13 +6757,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6768,13 +6771,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6782,13 +6785,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6796,21 +6799,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6846,7 +6849,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6854,7 +6857,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6866,167 +6869,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -7058,7 +7061,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7078,47 +7081,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7129,16 +7132,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7146,19 +7149,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7166,19 +7169,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7186,19 +7189,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S03-01: mark Done in workbook
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="590">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -867,6 +867,9 @@
   </si>
   <si>
     <t>Editing never alters a historical version</t>
+  </si>
+  <si>
+    <t>Done (2026-10-24) - article create/edit/list/version services; 95 db / 120 unit</t>
   </si>
   <si>
     <t>S03-02</t>
@@ -4176,12 +4179,12 @@
         <v>281</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>151</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4193,10 +4196,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4208,7 +4211,7 @@
         <v>278</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4216,7 +4219,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4228,10 +4231,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4243,7 +4246,7 @@
         <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4251,7 +4254,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4263,10 +4266,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4278,7 +4281,7 @@
         <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4286,7 +4289,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4298,10 +4301,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4313,7 +4316,7 @@
         <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4321,7 +4324,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4333,10 +4336,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4345,10 +4348,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4356,7 +4359,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4368,10 +4371,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4380,10 +4383,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4391,7 +4394,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4403,10 +4406,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4415,10 +4418,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4426,7 +4429,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4438,10 +4441,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4450,10 +4453,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4461,7 +4464,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4470,13 +4473,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4485,10 +4488,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4496,7 +4499,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4505,13 +4508,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4520,10 +4523,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4531,7 +4534,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4543,10 +4546,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4555,10 +4558,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4566,7 +4569,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4575,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4590,10 +4593,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4601,7 +4604,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4610,13 +4613,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4625,10 +4628,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4636,7 +4639,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4645,13 +4648,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4660,10 +4663,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4671,7 +4674,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4680,13 +4683,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4695,10 +4698,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4706,7 +4709,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4715,13 +4718,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4730,10 +4733,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4741,7 +4744,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4753,10 +4756,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4765,10 +4768,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4776,7 +4779,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4785,13 +4788,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4800,10 +4803,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4811,7 +4814,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4820,13 +4823,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4835,10 +4838,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4846,7 +4849,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4855,13 +4858,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4870,10 +4873,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4881,7 +4884,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4890,13 +4893,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4905,10 +4908,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4916,7 +4919,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4925,13 +4928,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4940,10 +4943,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4951,7 +4954,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4960,13 +4963,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4975,10 +4978,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4986,7 +4989,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4995,13 +4998,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5010,10 +5013,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5021,7 +5024,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5030,13 +5033,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5045,10 +5048,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5056,7 +5059,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5065,13 +5068,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5080,10 +5083,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5091,7 +5094,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5103,10 +5106,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5118,7 +5121,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5126,7 +5129,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5138,10 +5141,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5150,10 +5153,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5161,7 +5164,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5173,10 +5176,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5185,10 +5188,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5196,7 +5199,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5205,13 +5208,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5220,10 +5223,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5231,7 +5234,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5240,13 +5243,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5255,10 +5258,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5266,7 +5269,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5275,13 +5278,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5290,10 +5293,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5301,7 +5304,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5310,13 +5313,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5325,10 +5328,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5336,7 +5339,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5348,10 +5351,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5363,7 +5366,7 @@
         <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5371,7 +5374,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5380,13 +5383,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5395,10 +5398,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5406,7 +5409,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5415,13 +5418,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5430,10 +5433,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5441,7 +5444,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5450,13 +5453,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5465,10 +5468,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5476,7 +5479,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5488,10 +5491,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5500,10 +5503,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5511,7 +5514,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5523,10 +5526,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5535,10 +5538,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5546,7 +5549,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5558,10 +5561,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5570,10 +5573,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5581,7 +5584,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5593,10 +5596,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5605,10 +5608,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5616,22 +5619,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5643,7 +5646,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5651,22 +5654,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5678,7 +5681,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5686,22 +5689,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5710,10 +5713,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5721,22 +5724,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5745,10 +5748,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5756,22 +5759,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5780,10 +5783,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5791,22 +5794,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5818,7 +5821,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5826,22 +5829,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5853,7 +5856,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5861,22 +5864,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5885,10 +5888,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5896,22 +5899,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5920,10 +5923,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5931,10 +5934,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5943,10 +5946,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5955,10 +5958,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5998,12 +6001,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6017,19 +6020,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6052,10 +6055,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6078,10 +6081,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6104,10 +6107,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6130,7 +6133,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6154,7 +6157,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6178,10 +6181,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6204,7 +6207,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6228,7 +6231,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6252,10 +6255,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6278,7 +6281,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6302,7 +6305,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6326,7 +6329,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6350,7 +6353,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6374,15 +6377,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6390,7 +6393,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6398,7 +6401,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6427,7 +6430,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6444,10 +6447,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6455,7 +6458,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6464,10 +6467,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6475,7 +6478,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6487,7 +6490,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6495,7 +6498,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6504,10 +6507,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6515,7 +6518,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6524,10 +6527,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6541,18 +6544,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6561,53 +6564,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -6632,26 +6635,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6659,13 +6662,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6673,13 +6676,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6687,13 +6690,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6701,13 +6704,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6715,13 +6718,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6729,13 +6732,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6743,13 +6746,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6757,13 +6760,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6771,13 +6774,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6785,13 +6788,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6799,21 +6802,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6849,7 +6852,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6857,7 +6860,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6869,167 +6872,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -7061,7 +7064,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7081,47 +7084,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7132,16 +7135,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7149,19 +7152,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7169,19 +7172,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7189,19 +7192,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S03-01: mark Done in workbook (#29)
Workbook tick after PR #28. Evidence: 95 db / 120 unit; runbook S03-01.
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="590">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -867,6 +867,9 @@
   </si>
   <si>
     <t>Editing never alters a historical version</t>
+  </si>
+  <si>
+    <t>Done (2026-10-24) - article create/edit/list/version services; 95 db / 120 unit</t>
   </si>
   <si>
     <t>S03-02</t>
@@ -4176,12 +4179,12 @@
         <v>281</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>151</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
@@ -4193,10 +4196,10 @@
         <v>70</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G34" s="12">
         <v>1</v>
@@ -4208,7 +4211,7 @@
         <v>278</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K34" s="11" t="s">
         <v>151</v>
@@ -4216,7 +4219,7 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4228,10 +4231,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4243,7 +4246,7 @@
         <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4251,7 +4254,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4263,10 +4266,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4278,7 +4281,7 @@
         <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4286,7 +4289,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4298,10 +4301,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4313,7 +4316,7 @@
         <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4321,7 +4324,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4333,10 +4336,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4345,10 +4348,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4356,7 +4359,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4368,10 +4371,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4380,10 +4383,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4391,7 +4394,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4403,10 +4406,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4415,10 +4418,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4426,7 +4429,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4438,10 +4441,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4450,10 +4453,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4461,7 +4464,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4470,13 +4473,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4485,10 +4488,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4496,7 +4499,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4505,13 +4508,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4520,10 +4523,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4531,7 +4534,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4543,10 +4546,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4555,10 +4558,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4566,7 +4569,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4575,13 +4578,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4590,10 +4593,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4601,7 +4604,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4610,13 +4613,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4625,10 +4628,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4636,7 +4639,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4645,13 +4648,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4660,10 +4663,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4671,7 +4674,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4680,13 +4683,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4695,10 +4698,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4706,7 +4709,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4715,13 +4718,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4730,10 +4733,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4741,7 +4744,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4753,10 +4756,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4765,10 +4768,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4776,7 +4779,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4785,13 +4788,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4800,10 +4803,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4811,7 +4814,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4820,13 +4823,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4835,10 +4838,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4846,7 +4849,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4855,13 +4858,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4870,10 +4873,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4881,7 +4884,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4890,13 +4893,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4905,10 +4908,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4916,7 +4919,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4925,13 +4928,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4940,10 +4943,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4951,7 +4954,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4960,13 +4963,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4975,10 +4978,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4986,7 +4989,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4995,13 +4998,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5010,10 +5013,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5021,7 +5024,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5030,13 +5033,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5045,10 +5048,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5056,7 +5059,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5065,13 +5068,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5080,10 +5083,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5091,7 +5094,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5103,10 +5106,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5118,7 +5121,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5126,7 +5129,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5138,10 +5141,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5150,10 +5153,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5161,7 +5164,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5173,10 +5176,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5185,10 +5188,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5196,7 +5199,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5205,13 +5208,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5220,10 +5223,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5231,7 +5234,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5240,13 +5243,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5255,10 +5258,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5266,7 +5269,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5275,13 +5278,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5290,10 +5293,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5301,7 +5304,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5310,13 +5313,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5325,10 +5328,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5336,7 +5339,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5348,10 +5351,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5363,7 +5366,7 @@
         <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5371,7 +5374,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5380,13 +5383,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5395,10 +5398,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5406,7 +5409,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5415,13 +5418,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5430,10 +5433,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5441,7 +5444,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5450,13 +5453,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5465,10 +5468,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5476,7 +5479,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5488,10 +5491,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5500,10 +5503,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5511,7 +5514,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5523,10 +5526,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5535,10 +5538,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5546,7 +5549,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5558,10 +5561,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5570,10 +5573,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5581,7 +5584,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5593,10 +5596,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5605,10 +5608,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5616,22 +5619,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5643,7 +5646,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5651,22 +5654,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5678,7 +5681,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5686,22 +5689,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5710,10 +5713,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5721,22 +5724,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5745,10 +5748,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5756,22 +5759,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5780,10 +5783,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5791,22 +5794,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5818,7 +5821,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5826,22 +5829,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5853,7 +5856,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5861,22 +5864,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5885,10 +5888,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5896,22 +5899,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5920,10 +5923,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5931,10 +5934,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5943,10 +5946,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5955,10 +5958,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -5998,12 +6001,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6017,19 +6020,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6052,10 +6055,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6078,10 +6081,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6104,10 +6107,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6130,7 +6133,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6154,7 +6157,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6178,10 +6181,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6204,7 +6207,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6228,7 +6231,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6252,10 +6255,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6278,7 +6281,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6302,7 +6305,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6326,7 +6329,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6350,7 +6353,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6374,15 +6377,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6390,7 +6393,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6398,7 +6401,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6427,7 +6430,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6444,10 +6447,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6455,7 +6458,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6464,10 +6467,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6475,7 +6478,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6487,7 +6490,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6495,7 +6498,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6504,10 +6507,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6515,7 +6518,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6524,10 +6527,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6541,18 +6544,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6561,53 +6564,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -6632,26 +6635,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6659,13 +6662,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6673,13 +6676,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6687,13 +6690,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6701,13 +6704,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6715,13 +6718,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6729,13 +6732,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6743,13 +6746,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6757,13 +6760,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6771,13 +6774,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6785,13 +6788,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6799,21 +6802,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6849,7 +6852,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6857,7 +6860,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6869,167 +6872,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -7061,7 +7064,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7081,47 +7084,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7132,16 +7135,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7149,19 +7152,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7169,19 +7172,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7189,19 +7192,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S03-02: mark Done in workbook
Workbook tick after PR #30. Evidence: 107 db / 138 unit; runbook S03-02.
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="591">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -882,6 +882,9 @@
   </si>
   <si>
     <t>A 100-row CSV imports with a preview step and no silent failures</t>
+  </si>
+  <si>
+    <t>Done (2026-10-25) - RFC 4180 parser + pure preview, atomic commit; 107 db / 138 unit (PR #30)</t>
   </si>
   <si>
     <t>S03-03</t>
@@ -4214,12 +4217,12 @@
         <v>286</v>
       </c>
       <c r="K34" s="11" t="s">
-        <v>151</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4231,10 +4234,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4246,7 +4249,7 @@
         <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4254,7 +4257,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4266,10 +4269,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4281,7 +4284,7 @@
         <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4289,7 +4292,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4301,10 +4304,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4316,7 +4319,7 @@
         <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4324,7 +4327,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4336,10 +4339,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4348,10 +4351,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4359,7 +4362,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4371,10 +4374,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4383,10 +4386,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4394,7 +4397,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4406,10 +4409,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4418,10 +4421,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4429,7 +4432,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4441,10 +4444,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4453,10 +4456,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4464,7 +4467,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4473,13 +4476,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4488,10 +4491,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4499,7 +4502,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4508,13 +4511,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4523,10 +4526,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4534,7 +4537,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4546,10 +4549,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4558,10 +4561,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4569,7 +4572,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4578,13 +4581,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4593,10 +4596,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4604,7 +4607,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4613,13 +4616,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4628,10 +4631,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4639,7 +4642,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4648,13 +4651,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4663,10 +4666,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4674,7 +4677,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4683,13 +4686,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4698,10 +4701,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4709,7 +4712,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4718,13 +4721,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4733,10 +4736,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4744,7 +4747,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4756,10 +4759,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4768,10 +4771,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4779,7 +4782,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4788,13 +4791,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4803,10 +4806,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4814,7 +4817,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4823,13 +4826,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4838,10 +4841,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4849,7 +4852,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4858,13 +4861,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4873,10 +4876,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4884,7 +4887,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4893,13 +4896,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4908,10 +4911,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4919,7 +4922,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4928,13 +4931,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4943,10 +4946,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4954,7 +4957,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4963,13 +4966,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4978,10 +4981,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4989,7 +4992,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4998,13 +5001,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5013,10 +5016,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5024,7 +5027,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5033,13 +5036,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5048,10 +5051,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5059,7 +5062,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5068,13 +5071,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5083,10 +5086,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5094,7 +5097,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5106,10 +5109,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5121,7 +5124,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5129,7 +5132,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5141,10 +5144,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5153,10 +5156,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5164,7 +5167,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5176,10 +5179,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5188,10 +5191,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5199,7 +5202,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5208,13 +5211,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5223,10 +5226,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5234,7 +5237,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5243,13 +5246,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5258,10 +5261,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5269,7 +5272,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5278,13 +5281,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5293,10 +5296,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5304,7 +5307,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5313,13 +5316,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5328,10 +5331,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5339,7 +5342,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5351,10 +5354,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5366,7 +5369,7 @@
         <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5374,7 +5377,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5383,13 +5386,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5398,10 +5401,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5409,7 +5412,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5418,13 +5421,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5433,10 +5436,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5444,7 +5447,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5453,13 +5456,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5468,10 +5471,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5479,7 +5482,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5491,10 +5494,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5503,10 +5506,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5514,7 +5517,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5526,10 +5529,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5538,10 +5541,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5549,7 +5552,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5561,10 +5564,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5573,10 +5576,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5584,7 +5587,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5596,10 +5599,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5608,10 +5611,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5619,22 +5622,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5646,7 +5649,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5654,22 +5657,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5681,7 +5684,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5689,22 +5692,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5713,10 +5716,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5724,22 +5727,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5748,10 +5751,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5759,22 +5762,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5783,10 +5786,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5794,22 +5797,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5821,7 +5824,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5829,22 +5832,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5856,7 +5859,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5864,22 +5867,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5888,10 +5891,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5899,22 +5902,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5923,10 +5926,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5934,10 +5937,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5946,10 +5949,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5958,10 +5961,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -6001,12 +6004,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6020,19 +6023,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6055,10 +6058,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6081,10 +6084,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6107,10 +6110,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6133,7 +6136,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6157,7 +6160,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6181,10 +6184,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6207,7 +6210,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6231,7 +6234,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6255,10 +6258,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6281,7 +6284,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6305,7 +6308,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6329,7 +6332,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6353,7 +6356,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6377,15 +6380,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6393,7 +6396,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6401,7 +6404,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6430,7 +6433,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6447,10 +6450,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6458,7 +6461,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6467,10 +6470,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6478,7 +6481,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6490,7 +6493,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6498,7 +6501,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6507,10 +6510,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6518,7 +6521,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6527,10 +6530,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6544,18 +6547,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6564,53 +6567,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
   </sheetData>
@@ -6635,26 +6638,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6662,13 +6665,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6676,13 +6679,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6690,13 +6693,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6704,13 +6707,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6718,13 +6721,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6732,13 +6735,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6746,13 +6749,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6760,13 +6763,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6774,13 +6777,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6788,13 +6791,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6802,21 +6805,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6852,7 +6855,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6860,7 +6863,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6872,167 +6875,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -7064,7 +7067,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7084,47 +7087,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7135,16 +7138,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7152,19 +7155,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7172,19 +7175,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7192,19 +7195,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S03-02: mark Done in workbook (#31)
Workbook tick after PR #30. Evidence: 107 db / 138 unit; runbook S03-02.
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="591">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -882,6 +882,9 @@
   </si>
   <si>
     <t>A 100-row CSV imports with a preview step and no silent failures</t>
+  </si>
+  <si>
+    <t>Done (2026-10-25) - RFC 4180 parser + pure preview, atomic commit; 107 db / 138 unit (PR #30)</t>
   </si>
   <si>
     <t>S03-03</t>
@@ -4214,12 +4217,12 @@
         <v>286</v>
       </c>
       <c r="K34" s="11" t="s">
-        <v>151</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>68</v>
@@ -4231,10 +4234,10 @@
         <v>70</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G35" s="12">
         <v>2</v>
@@ -4246,7 +4249,7 @@
         <v>278</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K35" s="11" t="s">
         <v>151</v>
@@ -4254,7 +4257,7 @@
     </row>
     <row r="36" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>74</v>
@@ -4266,10 +4269,10 @@
         <v>70</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G36" s="12">
         <v>2</v>
@@ -4281,7 +4284,7 @@
         <v>278</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K36" s="11" t="s">
         <v>151</v>
@@ -4289,7 +4292,7 @@
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>74</v>
@@ -4301,10 +4304,10 @@
         <v>214</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G37" s="12">
         <v>1</v>
@@ -4316,7 +4319,7 @@
         <v>278</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>151</v>
@@ -4324,7 +4327,7 @@
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>74</v>
@@ -4336,10 +4339,10 @@
         <v>214</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G38" s="12">
         <v>2</v>
@@ -4348,10 +4351,10 @@
         <v>149</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>151</v>
@@ -4359,7 +4362,7 @@
     </row>
     <row r="39" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>79</v>
@@ -4371,10 +4374,10 @@
         <v>214</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G39" s="12">
         <v>2</v>
@@ -4383,10 +4386,10 @@
         <v>149</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>151</v>
@@ -4394,7 +4397,7 @@
     </row>
     <row r="40" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>79</v>
@@ -4406,10 +4409,10 @@
         <v>214</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G40" s="12">
         <v>2.5</v>
@@ -4418,10 +4421,10 @@
         <v>149</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>151</v>
@@ -4429,7 +4432,7 @@
     </row>
     <row r="41" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>79</v>
@@ -4441,10 +4444,10 @@
         <v>214</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G41" s="12">
         <v>1</v>
@@ -4453,10 +4456,10 @@
         <v>149</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>151</v>
@@ -4464,7 +4467,7 @@
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4473,13 +4476,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4488,10 +4491,10 @@
         <v>149</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4499,7 +4502,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4508,13 +4511,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4523,10 +4526,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4534,7 +4537,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4546,10 +4549,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4558,10 +4561,10 @@
         <v>149</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4569,7 +4572,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4578,13 +4581,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4593,10 +4596,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4604,7 +4607,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4613,13 +4616,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4628,10 +4631,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4639,7 +4642,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4648,13 +4651,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4663,10 +4666,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4674,7 +4677,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4683,13 +4686,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4698,10 +4701,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4709,7 +4712,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4718,13 +4721,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4733,10 +4736,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4744,7 +4747,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4756,10 +4759,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4768,10 +4771,10 @@
         <v>149</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4779,7 +4782,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4788,13 +4791,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4803,10 +4806,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4814,7 +4817,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4823,13 +4826,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4838,10 +4841,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4849,7 +4852,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4858,13 +4861,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4873,10 +4876,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4884,7 +4887,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4893,13 +4896,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4908,10 +4911,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4919,7 +4922,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4928,13 +4931,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4943,10 +4946,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4954,7 +4957,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4963,13 +4966,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4978,10 +4981,10 @@
         <v>149</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -4989,7 +4992,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -4998,13 +5001,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5013,10 +5016,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5024,7 +5027,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5033,13 +5036,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5048,10 +5051,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5059,7 +5062,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5068,13 +5071,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5083,10 +5086,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5094,7 +5097,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5106,10 +5109,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5121,7 +5124,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5129,7 +5132,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5141,10 +5144,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5153,10 +5156,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5164,7 +5167,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5176,10 +5179,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5188,10 +5191,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5199,7 +5202,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5208,13 +5211,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5223,10 +5226,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5234,7 +5237,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5243,13 +5246,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5258,10 +5261,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5269,7 +5272,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5278,13 +5281,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5293,10 +5296,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5304,7 +5307,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5313,13 +5316,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5328,10 +5331,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5339,7 +5342,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5351,10 +5354,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5366,7 +5369,7 @@
         <v>274</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5374,7 +5377,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5383,13 +5386,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5398,10 +5401,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5409,7 +5412,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5418,13 +5421,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5433,10 +5436,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5444,7 +5447,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5453,13 +5456,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5468,10 +5471,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5479,7 +5482,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5491,10 +5494,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5503,10 +5506,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5514,7 +5517,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5526,10 +5529,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5538,10 +5541,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5549,7 +5552,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5561,10 +5564,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5573,10 +5576,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5584,7 +5587,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5596,10 +5599,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5608,10 +5611,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5619,22 +5622,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5646,7 +5649,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5654,22 +5657,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5681,7 +5684,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5689,22 +5692,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5713,10 +5716,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5724,22 +5727,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5748,10 +5751,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5759,22 +5762,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5783,10 +5786,10 @@
         <v>149</v>
       </c>
       <c r="I79" s="23" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5794,22 +5797,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5821,7 +5824,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5829,22 +5832,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5856,7 +5859,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5864,22 +5867,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5888,10 +5891,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5899,22 +5902,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5923,10 +5926,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5934,10 +5937,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5946,10 +5949,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5958,10 +5961,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -6001,12 +6004,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6020,19 +6023,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6055,10 +6058,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6081,10 +6084,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6107,10 +6110,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6133,7 +6136,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6157,7 +6160,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6181,10 +6184,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6207,7 +6210,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6231,7 +6234,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6255,10 +6258,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6281,7 +6284,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6305,7 +6308,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6329,7 +6332,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6353,7 +6356,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6377,15 +6380,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6393,7 +6396,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6401,7 +6404,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6430,7 +6433,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6447,10 +6450,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6458,7 +6461,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6467,10 +6470,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6478,7 +6481,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6490,7 +6493,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6498,7 +6501,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6507,10 +6510,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6518,7 +6521,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6527,10 +6530,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6544,18 +6547,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6564,53 +6567,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
   </sheetData>
@@ -6635,26 +6638,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6662,13 +6665,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6676,13 +6679,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6690,13 +6693,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6704,13 +6707,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6718,13 +6721,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6732,13 +6735,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6746,13 +6749,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6760,13 +6763,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6774,13 +6777,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6788,13 +6791,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6802,21 +6805,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6852,7 +6855,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6860,7 +6863,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6872,167 +6875,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -7064,7 +7067,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7084,47 +7087,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7135,16 +7138,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7152,19 +7155,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7172,19 +7175,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7192,19 +7195,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S05-03: answer reconstruction, ai_runs indexes, usage shape check
- 0014_ai_runs_indexes.sql: ai_runs_property_time, citations_run, and
  CHECK (jsonb_typeof(usage) = 'object'). Number rebased from the charter's
  0013, which S04-03 now occupies.
- src/ai/history.ts: reconstructAnswer joins ai_runs -> citations ->
  article_versions (bodies AS CITED, immutable since 0003 / D5) and carries
  the conversation's handoff reasons. Foreign or unknown run ->
  AiRunNotFoundError rather than an empty citation list.
- tests/db/ai-history.db.test.ts: 6 cases incl. cited body surviving an
  article edit with isCurrent: false, cross-tenant refusal, both indexes,
  non-object usage rejected.
- Migration inventories 13 -> 14; runbook, charter and workbook updated.
- 180 db tests / 333 unit tests, typecheck + lint + build clean.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="597">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -984,6 +984,9 @@
   </si>
   <si>
     <t>Any historical answer reconstructable from the database</t>
+  </si>
+  <si>
+    <t>✅ Done (180 db + 333 unit; reconstructAnswer)</t>
   </si>
   <si>
     <t>S06-01</t>
@@ -4477,12 +4480,12 @@
         <v>320</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>151</v>
+        <v>321</v>
       </c>
     </row>
     <row r="42" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>85</v>
@@ -4491,13 +4494,13 @@
         <v>195</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G42" s="12">
         <v>2</v>
@@ -4509,7 +4512,7 @@
         <v>308</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="K42" s="11" t="s">
         <v>151</v>
@@ -4517,7 +4520,7 @@
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>85</v>
@@ -4526,13 +4529,13 @@
         <v>195</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G43" s="12">
         <v>1.5</v>
@@ -4541,10 +4544,10 @@
         <v>149</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>151</v>
@@ -4552,7 +4555,7 @@
     </row>
     <row r="44" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>85</v>
@@ -4564,10 +4567,10 @@
         <v>214</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G44" s="12">
         <v>1.5</v>
@@ -4579,7 +4582,7 @@
         <v>313</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>151</v>
@@ -4587,7 +4590,7 @@
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>90</v>
@@ -4596,13 +4599,13 @@
         <v>195</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G45" s="12">
         <v>0.5</v>
@@ -4611,10 +4614,10 @@
         <v>170</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>151</v>
@@ -4622,7 +4625,7 @@
     </row>
     <row r="46" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>90</v>
@@ -4631,13 +4634,13 @@
         <v>195</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G46" s="12">
         <v>0.5</v>
@@ -4646,10 +4649,10 @@
         <v>149</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K46" s="11" t="s">
         <v>151</v>
@@ -4657,7 +4660,7 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>90</v>
@@ -4666,13 +4669,13 @@
         <v>195</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G47" s="12">
         <v>1</v>
@@ -4681,10 +4684,10 @@
         <v>149</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>151</v>
@@ -4692,7 +4695,7 @@
     </row>
     <row r="48" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>90</v>
@@ -4701,13 +4704,13 @@
         <v>195</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G48" s="12">
         <v>1</v>
@@ -4716,10 +4719,10 @@
         <v>149</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>151</v>
@@ -4727,7 +4730,7 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>90</v>
@@ -4736,13 +4739,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G49" s="12">
         <v>0.5</v>
@@ -4751,10 +4754,10 @@
         <v>149</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="K49" s="11" t="s">
         <v>151</v>
@@ -4762,7 +4765,7 @@
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>90</v>
@@ -4774,10 +4777,10 @@
         <v>214</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G50" s="12">
         <v>0.5</v>
@@ -4789,7 +4792,7 @@
         <v>308</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K50" s="11" t="s">
         <v>151</v>
@@ -4797,7 +4800,7 @@
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>95</v>
@@ -4806,13 +4809,13 @@
         <v>195</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G51" s="12">
         <v>2</v>
@@ -4821,10 +4824,10 @@
         <v>149</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K51" s="11" t="s">
         <v>151</v>
@@ -4832,7 +4835,7 @@
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>95</v>
@@ -4841,13 +4844,13 @@
         <v>195</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G52" s="12">
         <v>1</v>
@@ -4856,10 +4859,10 @@
         <v>149</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K52" s="11" t="s">
         <v>151</v>
@@ -4867,7 +4870,7 @@
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>95</v>
@@ -4876,13 +4879,13 @@
         <v>195</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G53" s="12">
         <v>1.5</v>
@@ -4891,10 +4894,10 @@
         <v>149</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K53" s="11" t="s">
         <v>151</v>
@@ -4902,7 +4905,7 @@
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>95</v>
@@ -4911,13 +4914,13 @@
         <v>195</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G54" s="12">
         <v>1</v>
@@ -4926,10 +4929,10 @@
         <v>149</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K54" s="11" t="s">
         <v>151</v>
@@ -4937,7 +4940,7 @@
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B55" s="11" t="s">
         <v>100</v>
@@ -4946,13 +4949,13 @@
         <v>195</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G55" s="12">
         <v>2</v>
@@ -4961,10 +4964,10 @@
         <v>149</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>151</v>
@@ -4972,7 +4975,7 @@
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -4981,13 +4984,13 @@
         <v>195</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -4999,7 +5002,7 @@
         <v>313</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K56" s="11" t="s">
         <v>151</v>
@@ -5007,7 +5010,7 @@
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -5016,13 +5019,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5031,10 +5034,10 @@
         <v>149</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>151</v>
@@ -5042,7 +5045,7 @@
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5051,13 +5054,13 @@
         <v>195</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5066,10 +5069,10 @@
         <v>149</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K58" s="11" t="s">
         <v>151</v>
@@ -5077,7 +5080,7 @@
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5086,13 +5089,13 @@
         <v>195</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5101,10 +5104,10 @@
         <v>149</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>151</v>
@@ -5112,7 +5115,7 @@
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5124,10 +5127,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5139,7 +5142,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5147,7 +5150,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5159,10 +5162,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5171,10 +5174,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5182,7 +5185,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5194,10 +5197,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5206,10 +5209,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5217,7 +5220,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5226,13 +5229,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5241,10 +5244,10 @@
         <v>149</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5252,7 +5255,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5261,13 +5264,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5276,10 +5279,10 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5287,7 +5290,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5296,13 +5299,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5311,10 +5314,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5322,7 +5325,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5331,13 +5334,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5346,10 +5349,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5357,7 +5360,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5369,10 +5372,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5384,7 +5387,7 @@
         <v>275</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5392,7 +5395,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5401,13 +5404,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5416,10 +5419,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5427,7 +5430,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5436,13 +5439,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5451,10 +5454,10 @@
         <v>170</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5462,7 +5465,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5471,13 +5474,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5486,10 +5489,10 @@
         <v>170</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5497,7 +5500,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5509,10 +5512,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5521,10 +5524,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5532,7 +5535,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5544,10 +5547,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5556,10 +5559,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5567,7 +5570,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5579,10 +5582,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5591,10 +5594,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5602,7 +5605,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5614,10 +5617,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5626,10 +5629,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5637,22 +5640,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5664,7 +5667,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5672,22 +5675,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5699,7 +5702,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5707,22 +5710,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5731,10 +5734,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5742,22 +5745,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5766,10 +5769,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5777,22 +5780,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5804,7 +5807,7 @@
         <v>313</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5812,22 +5815,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5839,7 +5842,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5847,22 +5850,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5874,7 +5877,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5882,22 +5885,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5906,10 +5909,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5917,22 +5920,22 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5941,10 +5944,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -5952,10 +5955,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -5964,10 +5967,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -5976,10 +5979,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -6019,12 +6022,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6038,19 +6041,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6073,10 +6076,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6099,10 +6102,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6125,10 +6128,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
+        <v>511</v>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>510</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6151,7 +6154,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6175,7 +6178,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6199,10 +6202,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
+        <v>511</v>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>510</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6225,7 +6228,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6249,7 +6252,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6273,10 +6276,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
+        <v>511</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>510</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6299,7 +6302,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6323,7 +6326,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6347,7 +6350,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6371,7 +6374,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6395,15 +6398,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6411,7 +6414,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6419,7 +6422,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6448,7 +6451,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6465,10 +6468,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6476,7 +6479,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6485,10 +6488,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6496,7 +6499,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6508,7 +6511,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6516,7 +6519,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6525,10 +6528,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6536,7 +6539,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6545,10 +6548,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6562,18 +6565,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6582,53 +6585,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
   </sheetData>
@@ -6653,26 +6656,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6680,13 +6683,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6694,13 +6697,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6708,13 +6711,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6722,13 +6725,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6736,13 +6739,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6750,13 +6753,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6764,13 +6767,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6778,13 +6781,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6792,13 +6795,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6806,13 +6809,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6820,21 +6823,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6870,7 +6873,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6878,7 +6881,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6890,167 +6893,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>
@@ -7082,7 +7085,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7102,47 +7105,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7153,16 +7156,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7170,19 +7173,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7190,19 +7193,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7210,19 +7213,19 @@
         <v>61</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S09: tick S09-01..05 in the workbook and regenerate progress
All five S09 items are done and verified locally, so column K carries the
evidence for each in the established format (what shipped, migration number,
db/unit counts, and any owed physical evidence).

S09-05 records "real delivery email owed": DEC-4 closed on the provider and
explicitly deferred credentials, so no real email has been sent and none was
attempted. Everything up to the send is tested and the single HTTP call is
exercised against an injected fetch, but charter 7's "staging inbox screenshot
of a real delivered email" stays outstanding rather than being claimed. It joins
S07-01's phone scan, S08-01's stopwatch and S08-02's sources screenshot.

progress.md is regenerated by scripts/progress.mjs, never edited by hand:
S09 0/5 -> 5/5 (4.5d), overall 31 -> 36 of 80 items and 35.5 -> 40 of 79 days,
44.94% -> 50.63%.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="617">
   <si>
     <t>Master Sprint Backlog v2</t>
   </si>
@@ -1211,6 +1211,9 @@
     <t>request_acknowledged is set by a real staff action</t>
   </si>
   <si>
+    <t>✅ Done (2026-10-26: request_transition_guard trigger — transition matrix + actor GUC + membership role, per-edge evidence, immutable (org,property,request); 4 endpoints + Acknowledge/Cancel UI, 0024, 315 db / 562 unit)</t>
+  </si>
+  <si>
     <t>S09-02</t>
   </si>
   <si>
@@ -1223,6 +1226,9 @@
     <t>Every no_answer lands in the queue automatically</t>
   </si>
   <si>
+    <t>✅ Done (2026-10-26: one gap writer (recordGap) upserting per property+question_key with hits, close event + median open age, /api/gaps + /gaps screen, 0025, 336 db / 567 unit)</t>
+  </si>
+  <si>
     <t>S09-03</t>
   </si>
   <si>
@@ -1235,6 +1241,9 @@
     <t>A flag is attributable to an ai_run</t>
   </si>
   <si>
+    <t>✅ Done (2026-10-26: answer_flags append-only with composite FK to ai_runs, one flag per (run, actor), actor/time/note, indicator on the answer + event, 0026, 352 db / 570 unit)</t>
+  </si>
+  <si>
     <t>S09-04</t>
   </si>
   <si>
@@ -1247,6 +1256,9 @@
     <t>Flagging an answer does not delay the guest reply</t>
   </si>
   <si>
+    <t>✅ Done (2026-10-26: review work off the guest's path via outbox kind='review' — first outbox consumer; NOLOGIN concierge_worker definer claim, 0027, 368 db / 576 unit; worker unscheduled, S11-01)</t>
+  </si>
+  <si>
     <t>S09-05</t>
   </si>
   <si>
@@ -1257,6 +1269,9 @@
   </si>
   <si>
     <t>A request with no staff view still reaches a human by email</t>
+  </si>
+  <si>
+    <t>✅ Done (2026-10-26: escalation email queued in the request's own transaction; Resend over plain fetch, settings contacts + redacted deployment fallback, claim_outbox generalised, 0028, 395 db / 610 unit; real delivery email owed)</t>
   </si>
   <si>
     <t>S10-01</t>
@@ -5015,12 +5030,12 @@
         <v>395</v>
       </c>
       <c r="K55" s="11" t="s">
-        <v>151</v>
+        <v>396</v>
       </c>
     </row>
     <row r="56" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>100</v>
@@ -5032,10 +5047,10 @@
         <v>371</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G56" s="12">
         <v>0.5</v>
@@ -5047,15 +5062,15 @@
         <v>314</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K56" s="11" t="s">
-        <v>151</v>
+        <v>401</v>
       </c>
     </row>
     <row r="57" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>100</v>
@@ -5067,10 +5082,10 @@
         <v>371</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="G57" s="12">
         <v>0.5</v>
@@ -5082,15 +5097,15 @@
         <v>376</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="K57" s="11" t="s">
-        <v>151</v>
+        <v>406</v>
       </c>
     </row>
     <row r="58" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>100</v>
@@ -5102,10 +5117,10 @@
         <v>371</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="G58" s="12">
         <v>0.5</v>
@@ -5117,15 +5132,15 @@
         <v>381</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="K58" s="11" t="s">
-        <v>151</v>
+        <v>411</v>
       </c>
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>100</v>
@@ -5137,10 +5152,10 @@
         <v>392</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="G59" s="12">
         <v>1</v>
@@ -5152,15 +5167,15 @@
         <v>391</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="K59" s="11" t="s">
-        <v>151</v>
+        <v>416</v>
       </c>
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>105</v>
@@ -5172,10 +5187,10 @@
         <v>107</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="G60" s="12">
         <v>1.5</v>
@@ -5187,7 +5202,7 @@
         <v>231</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="K60" s="11" t="s">
         <v>151</v>
@@ -5195,7 +5210,7 @@
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>105</v>
@@ -5207,10 +5222,10 @@
         <v>107</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="G61" s="12">
         <v>1</v>
@@ -5219,10 +5234,10 @@
         <v>149</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>151</v>
@@ -5230,7 +5245,7 @@
     </row>
     <row r="62" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>105</v>
@@ -5242,10 +5257,10 @@
         <v>107</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="G62" s="12">
         <v>2</v>
@@ -5254,10 +5269,10 @@
         <v>149</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="K62" s="11" t="s">
         <v>151</v>
@@ -5265,7 +5280,7 @@
     </row>
     <row r="63" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>110</v>
@@ -5274,13 +5289,13 @@
         <v>195</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="G63" s="12">
         <v>1.5</v>
@@ -5292,7 +5307,7 @@
         <v>324</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="K63" s="11" t="s">
         <v>151</v>
@@ -5300,7 +5315,7 @@
     </row>
     <row r="64" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>110</v>
@@ -5309,13 +5324,13 @@
         <v>195</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="G64" s="12">
         <v>1</v>
@@ -5327,7 +5342,7 @@
         <v>324</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="K64" s="11" t="s">
         <v>151</v>
@@ -5335,7 +5350,7 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>110</v>
@@ -5344,13 +5359,13 @@
         <v>195</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="G65" s="12">
         <v>1</v>
@@ -5359,10 +5374,10 @@
         <v>149</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="K65" s="11" t="s">
         <v>151</v>
@@ -5370,7 +5385,7 @@
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>110</v>
@@ -5379,13 +5394,13 @@
         <v>195</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="G66" s="12">
         <v>1</v>
@@ -5394,10 +5409,10 @@
         <v>149</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="K66" s="11" t="s">
         <v>151</v>
@@ -5405,7 +5420,7 @@
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>110</v>
@@ -5417,10 +5432,10 @@
         <v>214</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="G67" s="12">
         <v>0.5</v>
@@ -5432,7 +5447,7 @@
         <v>275</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="K67" s="11" t="s">
         <v>151</v>
@@ -5440,7 +5455,7 @@
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>115</v>
@@ -5449,13 +5464,13 @@
         <v>195</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="G68" s="12">
         <v>1</v>
@@ -5464,10 +5479,10 @@
         <v>149</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="K68" s="11" t="s">
         <v>151</v>
@@ -5475,7 +5490,7 @@
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>115</v>
@@ -5484,13 +5499,13 @@
         <v>195</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="G69" s="12">
         <v>1</v>
@@ -5502,7 +5517,7 @@
         <v>370</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>151</v>
@@ -5510,7 +5525,7 @@
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>115</v>
@@ -5519,13 +5534,13 @@
         <v>195</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="G70" s="12">
         <v>1</v>
@@ -5537,7 +5552,7 @@
         <v>370</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="K70" s="11" t="s">
         <v>151</v>
@@ -5545,7 +5560,7 @@
     </row>
     <row r="71" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>115</v>
@@ -5557,10 +5572,10 @@
         <v>190</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="G71" s="12">
         <v>1.5</v>
@@ -5569,10 +5584,10 @@
         <v>149</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>151</v>
@@ -5580,7 +5595,7 @@
     </row>
     <row r="72" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>121</v>
@@ -5592,10 +5607,10 @@
         <v>190</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="G72" s="12">
         <v>1</v>
@@ -5604,10 +5619,10 @@
         <v>149</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>151</v>
@@ -5615,7 +5630,7 @@
     </row>
     <row r="73" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>121</v>
@@ -5627,10 +5642,10 @@
         <v>190</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="G73" s="12">
         <v>0.5</v>
@@ -5639,10 +5654,10 @@
         <v>149</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>151</v>
@@ -5650,7 +5665,7 @@
     </row>
     <row r="74" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>121</v>
@@ -5662,10 +5677,10 @@
         <v>190</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="G74" s="12">
         <v>0.5</v>
@@ -5674,10 +5689,10 @@
         <v>149</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="K74" s="11" t="s">
         <v>151</v>
@@ -5685,22 +5700,22 @@
     </row>
     <row r="75" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="22" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C75" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="G75" s="24">
         <v>0.25</v>
@@ -5712,7 +5727,7 @@
         <v>181</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="K75" s="23" t="s">
         <v>151</v>
@@ -5720,22 +5735,22 @@
     </row>
     <row r="76" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="22" t="s">
+        <v>484</v>
+      </c>
+      <c r="B76" s="23" t="s">
         <v>479</v>
-      </c>
-      <c r="B76" s="23" t="s">
-        <v>474</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E76" s="23" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="F76" s="23" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="G76" s="24">
         <v>1.5</v>
@@ -5747,7 +5762,7 @@
         <v>185</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="K76" s="23" t="s">
         <v>151</v>
@@ -5755,22 +5770,22 @@
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C77" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E77" s="23" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="F77" s="23" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="G77" s="24">
         <v>1.5</v>
@@ -5779,10 +5794,10 @@
         <v>149</v>
       </c>
       <c r="I77" s="23" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="K77" s="23" t="s">
         <v>151</v>
@@ -5790,22 +5805,22 @@
     </row>
     <row r="78" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="22" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C78" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E78" s="23" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="F78" s="23" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="G78" s="24">
         <v>1</v>
@@ -5814,10 +5829,10 @@
         <v>149</v>
       </c>
       <c r="I78" s="23" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="K78" s="23" t="s">
         <v>151</v>
@@ -5825,22 +5840,22 @@
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="22" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="G79" s="24">
         <v>1</v>
@@ -5852,7 +5867,7 @@
         <v>314</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="K79" s="23" t="s">
         <v>151</v>
@@ -5860,22 +5875,22 @@
     </row>
     <row r="80" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="22" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="B80" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C80" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E80" s="23" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="F80" s="23" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="G80" s="24">
         <v>1</v>
@@ -5887,7 +5902,7 @@
         <v>185</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="K80" s="23" t="s">
         <v>151</v>
@@ -5895,22 +5910,22 @@
     </row>
     <row r="81" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="22" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="B81" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C81" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E81" s="23" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="F81" s="23" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="G81" s="24">
         <v>0.5</v>
@@ -5922,7 +5937,7 @@
         <v>162</v>
       </c>
       <c r="J81" s="23" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="K81" s="23" t="s">
         <v>151</v>
@@ -5930,22 +5945,22 @@
     </row>
     <row r="82" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B82" s="23" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C82" s="20" t="s">
         <v>195</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E82" s="23" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="F82" s="23" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="G82" s="24">
         <v>1</v>
@@ -5954,10 +5969,10 @@
         <v>170</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="J82" s="23" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="K82" s="23" t="s">
         <v>151</v>
@@ -5965,10 +5980,10 @@
     </row>
     <row r="83" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="25" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="B83" s="26" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="C83" s="20" t="s">
         <v>195</v>
@@ -5977,10 +5992,10 @@
         <v>392</v>
       </c>
       <c r="E83" s="26" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="G83" s="27">
         <v>1</v>
@@ -5989,10 +6004,10 @@
         <v>170</v>
       </c>
       <c r="I83" s="26" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="J83" s="26" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="K83" s="26" t="s">
         <v>151</v>
@@ -6000,10 +6015,10 @@
     </row>
     <row r="84" ht="40" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="25" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="B84" s="26" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="C84" s="20" t="s">
         <v>195</v>
@@ -6012,10 +6027,10 @@
         <v>107</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="G84" s="27">
         <v>0.5</v>
@@ -6024,10 +6039,10 @@
         <v>170</v>
       </c>
       <c r="I84" s="26" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="J84" s="26" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="K84" s="26" t="s">
         <v>151</v>
@@ -6067,12 +6082,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6086,19 +6101,19 @@
         <v>43</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>143</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6121,10 +6136,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="28" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6147,10 +6162,10 @@
         <v>5.75</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6173,10 +6188,10 @@
         <v>5.5</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6199,7 +6214,7 @@
         <v>5</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H8" s="11"/>
     </row>
@@ -6223,7 +6238,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H9" s="11"/>
     </row>
@@ -6247,10 +6262,10 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6273,7 +6288,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H11" s="11"/>
     </row>
@@ -6297,7 +6312,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H12" s="11"/>
     </row>
@@ -6321,10 +6336,10 @@
         <v>5.5</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6347,7 +6362,7 @@
         <v>4.5</v>
       </c>
       <c r="G14" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H14" s="11"/>
     </row>
@@ -6371,7 +6386,7 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H15" s="11"/>
     </row>
@@ -6395,7 +6410,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H16" s="11"/>
     </row>
@@ -6419,7 +6434,7 @@
         <v>4.5</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -6443,15 +6458,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" s="5" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="F20" s="30">
         <v>69.75</v>
@@ -6459,7 +6474,7 @@
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C21" s="18" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="F21" s="18">
         <v>70</v>
@@ -6467,7 +6482,7 @@
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C22" s="5" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="F22" s="31">
         <v>0.25</v>
@@ -6496,7 +6511,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6513,10 +6528,10 @@
         <v>42</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6524,7 +6539,7 @@
         <v>55</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>51</v>
@@ -6533,10 +6548,10 @@
         <v>52</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6544,7 +6559,7 @@
         <v>72</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>68</v>
@@ -6556,7 +6571,7 @@
         <v>73</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6564,7 +6579,7 @@
         <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>79</v>
@@ -6573,10 +6588,10 @@
         <v>80</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6584,7 +6599,7 @@
         <v>119</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>115</v>
@@ -6593,10 +6608,10 @@
         <v>116</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6610,18 +6625,18 @@
         <v>121</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>129</v>
@@ -6630,53 +6645,53 @@
         <v>61</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -6701,26 +6716,26 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6728,13 +6743,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6742,13 +6757,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6756,13 +6771,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6770,13 +6785,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6784,13 +6799,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6798,13 +6813,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6812,13 +6827,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6826,13 +6841,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6846,7 +6861,7 @@
         <v>95</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6854,13 +6869,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6868,21 +6883,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="D17"/>
     </row>
@@ -6918,7 +6933,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6926,7 +6941,7 @@
         <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>137</v>
@@ -6938,167 +6953,167 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="E5" s="12">
         <v>0.25</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="E6" s="12">
         <v>1.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="E7" s="12">
         <v>1.5</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="E11" s="12">
         <v>0.5</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -7130,7 +7145,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7150,47 +7165,47 @@
         <v>140</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>392</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7201,16 +7216,16 @@
         <v>70</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="E7" s="12">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7218,19 +7233,19 @@
         <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="E8" s="12">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7238,19 +7253,19 @@
         <v>61</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="E9" s="12">
         <v>0</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7261,16 +7276,16 @@
         <v>371</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="E10" s="12">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S10-01, S10-01-1: mark Done in the master backlog
Both are merged:
- S10-01 (event emission across the product) shipped in PR #146 as 12ebab0.
- S10-01-1 (one clock for events and their business rows) shipped in PR #149
  as 44b31f0.

Column K updated only through scripts/update-workbook-status.mjs, and
docs/progress.md only through scripts/progress.mjs, per the standing
close-out rules. The S10-01 evidence keeps the owner's 2026-10-26 deferral
on the record: AC-1 is accepted at 16 of 18, with booking_link_clicked and
outbound_webhook_delivered reserved in the taxonomy and test-enforced until
DF-01/DF-02 land in MVP-1.5.

Progress: 40/82 items, 42.75/79.75 days (53.61%), 4 in flight.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -1286,7 +1286,7 @@
     <t>Dashboard numbers reconcile exactly to raw events</t>
   </si>
   <si>
-    <t>🚧 AC-2 and AC-3 met and verified (0029 hardening; reconcile() over 8 pairs, deltas 0; 100 actions -&gt; exactly 100 events; 39 db files / 415 + 48 unit / 629 green). AC-1 is 16 of 18: booking_link_clicked and outbound_webhook_delivered have no producer — they belong to DF-02 and DF-01, both deferred to MVP-1.5. Owner deferred on 2026-10-26; both names stay reserved in the taxonomy and a test fails if either gains a producer before the charter is updated.</t>
+    <t>✅ Done (merged in PR #146 as 12ebab0. AC-2 and AC-3 met and verified: 0029 append-only hardening, reconcile() over 8 business/event pairs with deltas 0, 100 actions produce exactly 100 events. AC-1 accepted at 16 of 18 — booking_link_clicked and outbound_webhook_delivered have no producer; they belong to DF-02 and DF-01, both deferred to MVP-1.5 by the owner on 2026-10-26. Both names stay reserved in the taxonomy and a test fails if either gains a producer before the charter is updated. Follow-ups: S10-01-2 merged in #146, S10-01-1 merged in #149.)</t>
   </si>
   <si>
     <t>S10-01-1</t>
@@ -1301,7 +1301,7 @@
     <t>Every reconciled pair agrees on created_at exactly, and no window reports a delta that is not real drift</t>
   </si>
   <si>
-    <t>🚧 Implemented and verified locally (clock-agreement: 12 tests over all 8 metrics; db 40 files / 427, unit 49 / 638) — pending merge, then ✅</t>
+    <t>✅ Done (merged in PR #149 as 44b31f0 — src/events/clock.ts; every producer reads created_at back from its own INSERT and hands that exact value to emitEvent, so a business row and its event carry one identical stamp and no reconcile window boundary can fall between them. tests/db/clock-agreement.db.test.ts: 12 tests drive the real producers for all 8 metrics and compare e.created_at &lt;&gt; b.created_at in SQL. Also fixed the ai_runs window metric, which counted answer_flagged_wrong as a run and so reported phantom drift; AI_RUN_TERMINAL_EVENT_TYPES now classifies it. db 40 files / 427, unit 49 files / 638, CI 8/8.)</t>
   </si>
   <si>
     <t>S10-01-2</t>

</xml_diff>

<commit_message>
S10-01, S10-01-1: mark Done in the master backlog (#150)
Both are merged:
- S10-01 (event emission across the product) shipped in PR #146 as 12ebab0.
- S10-01-1 (one clock for events and their business rows) shipped in PR #149
  as 44b31f0.

Column K updated only through scripts/update-workbook-status.mjs, and
docs/progress.md only through scripts/progress.mjs, per the standing
close-out rules. The S10-01 evidence keeps the owner's 2026-10-26 deferral
on the record: AC-1 is accepted at 16 of 18, with booking_link_clicked and
outbound_webhook_delivered reserved in the taxonomy and test-enforced until
DF-01/DF-02 land in MVP-1.5.

Progress: 40/82 items, 42.75/79.75 days (53.61%), 4 in flight.

Co-authored-by: jtanori <920148+jtanori@users.noreply.github.com>
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -1286,7 +1286,7 @@
     <t>Dashboard numbers reconcile exactly to raw events</t>
   </si>
   <si>
-    <t>🚧 AC-2 and AC-3 met and verified (0029 hardening; reconcile() over 8 pairs, deltas 0; 100 actions -&gt; exactly 100 events; 39 db files / 415 + 48 unit / 629 green). AC-1 is 16 of 18: booking_link_clicked and outbound_webhook_delivered have no producer — they belong to DF-02 and DF-01, both deferred to MVP-1.5. Owner deferred on 2026-10-26; both names stay reserved in the taxonomy and a test fails if either gains a producer before the charter is updated.</t>
+    <t>✅ Done (merged in PR #146 as 12ebab0. AC-2 and AC-3 met and verified: 0029 append-only hardening, reconcile() over 8 business/event pairs with deltas 0, 100 actions produce exactly 100 events. AC-1 accepted at 16 of 18 — booking_link_clicked and outbound_webhook_delivered have no producer; they belong to DF-02 and DF-01, both deferred to MVP-1.5 by the owner on 2026-10-26. Both names stay reserved in the taxonomy and a test fails if either gains a producer before the charter is updated. Follow-ups: S10-01-2 merged in #146, S10-01-1 merged in #149.)</t>
   </si>
   <si>
     <t>S10-01-1</t>
@@ -1301,7 +1301,7 @@
     <t>Every reconciled pair agrees on created_at exactly, and no window reports a delta that is not real drift</t>
   </si>
   <si>
-    <t>🚧 Implemented and verified locally (clock-agreement: 12 tests over all 8 metrics; db 40 files / 427, unit 49 / 638) — pending merge, then ✅</t>
+    <t>✅ Done (merged in PR #149 as 44b31f0 — src/events/clock.ts; every producer reads created_at back from its own INSERT and hands that exact value to emitEvent, so a business row and its event carry one identical stamp and no reconcile window boundary can fall between them. tests/db/clock-agreement.db.test.ts: 12 tests drive the real producers for all 8 metrics and compare e.created_at &lt;&gt; b.created_at in SQL. Also fixed the ai_runs window metric, which counted answer_flagged_wrong as a run and so reported phantom drift; AI_RUN_TERMINAL_EVENT_TYPES now classifies it. db 40 files / 427, unit 49 files / 638, CI 8/8.)</t>
   </si>
   <si>
     <t>S10-01-2</t>

</xml_diff>

<commit_message>
docs: plan S06A API, deploy and eval reliability
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -100,17 +100,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -182,17 +182,17 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -216,11 +216,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +605,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Single source of truth for the build · 81 items · 14 sprints · 21 Oct 2026</t>
+          <t>Single source of truth for the build · 88 items · 15 work blocks including ASAP S06A · 21 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -621,15 +621,15 @@
       </c>
       <c r="C6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Lean pilot path</t>
+          <t>Planned engineering path</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>70.00 dev-days across 14 sprints (W00, S01–S13). Pilot live Monday of W14.</t>
+          <t>84.50 dev-days across original 14 sprints plus ASAP S06A. Original W14 pilot forecast must be revised.</t>
         </is>
       </c>
     </row>
@@ -665,14 +665,14 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>79.25 dev-days across 81 items.</t>
+          <t>93.75 dev-days across 88 items.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Original capacity</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -684,12 +684,12 @@
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Slack</t>
+          <t>Net change</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>0.00 days unallocated. W13 carries 2.00 days of launch work, leaving ~3 days of carry-forward room in that week.</t>
+          <t>+14.50 days vs original 70-day plan; S06A adds 14.50 engineering days and is not absorbed by W13 slack.</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>14 sprints: goal, items, days, cumulative weeks, gate, exit criterion.</t>
+          <t>15 work blocks: goal, items, days, cumulative weeks, gate, exit criterion.</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>All 81 items with sprint, track, estimate, dependency and acceptance criteria. The working board.</t>
+          <t>All 88 items with sprint, track, estimate, dependency and acceptance criteria. The working board.</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -880,14 +880,14 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Sprint ladder — 14 sprints to pilot</t>
+          <t>Sprint ladder — original plan plus ASAP S06A</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Cumulative weeks is the true elapsed position. Work completes at 14.00 weeks; W14 is launch.</t>
+          <t>Cumulative effort is shown; ASAP S06A invalidates the original W14 launch forecast until resequenced.</t>
         </is>
       </c>
     </row>
@@ -1280,85 +1280,85 @@
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Chat hardening</t>
+          <t>API, deployment and eval reliability</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Abuse, outages and provider failure</t>
+          <t>Make release and answer-quality evidence trustworthy</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>4</v>
+        <v>14.5</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>44</v>
+        <v>54.5</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>10.9</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>G2 remediation</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>AI killed mid-conversation still yields an honest reply and a ticket · cap trip degrades gracefully</t>
+          <t>Full API surface has a documented contract and reachable deployment · deploys follow native Vercel Git integration with enforced CI · live canary diagnostics identify real retrieval/fact/guardrail cause · G2 measured on a sufficiently large, representative set</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Staff inbox</t>
+          <t>Chat hardening</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>The surface an agent actually uses</t>
+          <t>Abuse, outages and provider failure</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="12" t="n">
-        <v>5.5</v>
-      </c>
       <c r="G13" s="12" t="n">
-        <v>49.5</v>
+        <v>58.5</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>-0.5</v>
+        <v>11.7</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
@@ -1367,45 +1367,45 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>An agent triages a queue on a phone in under 60 seconds · takeover is atomic</t>
+          <t>AI killed mid-conversation still yields an honest reply and a ticket · cap trip degrades gracefully</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Requests and notifications</t>
+          <t>Staff inbox</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>A request nobody sees is not a request</t>
+          <t>The surface an agent actually uses</t>
         </is>
       </c>
       <c r="E14" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>0.5</v>
+        <v>12.8</v>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>-0.5</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -1414,42 +1414,42 @@
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>Ack timestamp set by a real staff action · a request with no staff view still reaches a human</t>
+          <t>An agent triages a queue on a phone in under 60 seconds · takeover is atomic</t>
         </is>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Requests and notifications</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>What guests ask, and what we cannot answer</t>
+          <t>A request nobody sees is not a request</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F15" s="12" t="n">
         <v>4.5</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>58.5</v>
+        <v>68.5</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>11.7</v>
+        <v>13.7</v>
       </c>
       <c r="I15" s="12" t="n">
         <v>0.5</v>
@@ -1461,45 +1461,45 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Dashboard numbers reconcile exactly to raw events · every tile traceable to a query</t>
+          <t>Ack timestamp set by a real staff action · a request with no staff view still reaches a human</t>
         </is>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Outbox, idempotency, redaction, observability</t>
+          <t>What guests ask, and what we cannot answer</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>63.5</v>
+        <v>73</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>12.7</v>
+        <v>14.6</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
@@ -1508,160 +1508,207 @@
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Provider outage causes delayed sends, not lost messages · no card number reaches logs</t>
+          <t>Dashboard numbers reconcile exactly to raw events · every tile traceable to a query</t>
         </is>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Pilot readiness</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Prove it works before a guest sees it</t>
+          <t>Outbox, idempotency, redaction, observability</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>13.6</v>
+        <v>15.6</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>G3</t>
+        <v>0</v>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Restore drilled and timed · three staff complete the flow unaided · runbook signed off</t>
+          <t>Provider outage causes delayed sends, not lost messages · no card number reaches logs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Pilot readiness</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Prove it works before a guest sees it</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>Restore drilled and timed · three staff complete the flow unaided · runbook signed off</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
           <t>S13</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Train the staff, fix the content, go/no-go</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E19" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="H18" s="12" t="n">
-        <v>14</v>
-      </c>
-      <c r="I18" s="12" t="n">
+      <c r="G19" s="12" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I19" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="11" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K18" s="11" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>Pilot property trained · content corrections applied · GM sign-off recorded</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>LEAN PILOT PATH</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="16" t="n">
-        <v>71</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="16" t="n">
-        <v>14</v>
-      </c>
-      <c r="I19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-    </row>
-    <row r="21">
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Pilot live</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Monday W14</t>
-        </is>
-      </c>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>PLANNED ENGINEERING PATH</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="16" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I20" s="16" t="n">
+        <v>-14.5</v>
+      </c>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Pilot readout</t>
+          <t>Pilot live</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>W17 (G4)</t>
+          <t>Forecast after S06A</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t>Pilot readout</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>W17 (G4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
           <t>WhatsApp live</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>W18 (G5)</t>
         </is>
@@ -1679,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4024,12 +4071,12 @@
     <row r="46" ht="40" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>S07-01</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr">
@@ -4039,35 +4086,35 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>QR + embeddable snippet</t>
+          <t>Eval attribution and retrieval diagnostics</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>Generated QR per property; one-line embed; logo and colour only.</t>
+          <t>Correctly distinguish pre-retrieval guardrails, structured facts, retrieval candidates, model refusals and provider outages; retain safe per-question diagnostics.</t>
         </is>
       </c>
       <c r="G46" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S06-03</t>
         </is>
       </c>
       <c r="J46" s="11" t="inlineStr">
         <is>
-          <t>QR resolves to the right property on a real phone</t>
+          <t>For every golden row, report pipeline stage, outcome/reason, target-topic retrieval hit and safe retrieved-topic diagnostics; synthetic tests reproduce each bucket and no failure is reported as retrieval-empty unless retrieval was actually empty</t>
         </is>
       </c>
       <c r="K46" s="11" t="inlineStr">
@@ -4079,12 +4126,12 @@
     <row r="47" ht="40" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>S07-02</t>
+          <t>S06A-02</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C47" s="20" t="inlineStr">
@@ -4094,21 +4141,21 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>AI disclosure + 'talk to a person'</t>
+          <t>Sensitive and policy classifier calibration</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Persistent, obvious, translated.</t>
+          <t>Replace broad phrase collisions with intent-aware, bilingual rules; protect deliberate escalation for refund, booking and safety requests while permitting factual property questions.</t>
         </is>
       </c>
       <c r="G47" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
@@ -4117,12 +4164,12 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>A human is reachable in one tap from any state</t>
+          <t>Regression tests cover price questions for known services, booking/transacting requests, extra-bed policy, pet policy, explicit handoff, refunds, allergy and accessibility; no escalation rule is weakened without safety tests</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
@@ -4134,12 +4181,12 @@
     <row r="48" ht="40" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>S07-03</t>
+          <t>S06A-03</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
@@ -4149,21 +4196,21 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>Request capture + honest acknowledgement</t>
+          <t>Guest intent classification and structured-fact routing</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>'I have sent your request' — never 'on the way'. Creates a service_request.</t>
+          <t>Add a conservative, auditable route from guest question to allowed topic/fact keys; unknown or ambiguous intent falls back to retrieval/handoff and never trusts golden labels at runtime.</t>
         </is>
       </c>
       <c r="G48" s="12" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
@@ -4172,12 +4219,12 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-02</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
         <is>
-          <t>No code path can claim a request is fulfilled</t>
+          <t>Property fact questions in English and Spanish reach verified fact lookup using inferred topic/fact keys; wrong/absent fact falls back safely; tests prove no caller-supplied tenant/topic label bypasses policy</t>
         </is>
       </c>
       <c r="K48" s="11" t="inlineStr">
@@ -4189,12 +4236,12 @@
     <row r="49" ht="40" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>S07-04</t>
+          <t>S06A-04</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C49" s="20" t="inlineStr">
@@ -4204,21 +4251,21 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Abuse + cost protection</t>
+          <t>Cross-language knowledge and retrieval quality</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Turnstile, per-IP/conversation/property rate limits, daily AI spend cap.</t>
+          <t>Ensure Spanish guest questions can retrieve approved English or Spanish knowledge without inventing translations or weakening tenant/current-version filters.</t>
         </is>
       </c>
       <c r="G49" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
@@ -4227,12 +4274,12 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>Cap trip degrades to 'a team member will reply' without an error</t>
+          <t>Bilingual paraphrase retrieval suite meets ≥90% target-topic recall on frozen cases; exact-language and cross-language cases, noise, no-match and tenant isolation are covered; only approved content is cited</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
@@ -4244,12 +4291,12 @@
     <row r="50" ht="40" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>S07-05</t>
+          <t>S06A-05</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
@@ -4259,21 +4306,21 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Outage fallback</t>
+          <t>API contract and runtime decision</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>If AI or provider is down, say so plainly and still capture a request.</t>
+          <t>Inventory all implemented and deployed routes; specify OpenAPI contracts; prove representative guest/staff paths against the selected runtime and document Vercel Functions versus persistent-service decision.</t>
         </is>
       </c>
       <c r="G50" s="12" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
@@ -4282,12 +4329,12 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>S07-04</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
-          <t>Kill the AI mid-conversation; guest still gets an honest message</t>
+          <t>Every route used by web is mapped to handler, auth/tenant policy, schema, response and deployment adapter; contract validation and HTTP integration tests pass; runtime decision cites measured duration, DB pooling and worker constraints</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
@@ -4299,12 +4346,12 @@
     <row r="51" ht="40" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>S07-06</t>
+          <t>S06A-06</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr">
@@ -4314,21 +4361,21 @@
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>LLM transport resilience</t>
+          <t>Native Vercel Git deploys for API and web</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>Timeouts, retry with jitter, circuit breaker, pinned model versions, parse-failure alerting.</t>
+          <t>Configure both Vercel projects for explicit roots/builds and Git-based preview/staging/production deployment; retire alias pinning/CLI deployment only after proof.</t>
         </is>
       </c>
       <c r="G51" s="12" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
@@ -4337,12 +4384,12 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>S05-01</t>
+          <t>S06A-05</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>Both providers killed; product degrades honestly</t>
+          <t>API and web preview from same commit; protected staging has stable Vercel branch/domain binding; production deploys from agreed branch; deliberately failing required CI check blocks promotion; no alias-pinning step or GitHub Vercel token needed for routine deploy</t>
         </is>
       </c>
       <c r="K51" s="11" t="inlineStr">
@@ -4354,12 +4401,12 @@
     <row r="52" ht="40" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06A-07</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
@@ -4369,21 +4416,21 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Phone-first shared inbox</t>
+          <t>Representative golden set and gate arming</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>Filters: needs attention, mine, unresolved, unassigned.</t>
+          <t>Expand and curate golden set to at least 50 reviewed cases with adequate answer/escalation and language/topic coverage; re-baseline deterministic eval and canary without hiding the current failure.</t>
         </is>
       </c>
       <c r="G52" s="12" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
@@ -4392,12 +4439,12 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-01, S06A-02, S06A-03, S06A-04</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
-          <t>An agent triages a queue on a phone in under 60 seconds</t>
+          <t>At least 50 reviewed questions include target language/topic, expected behaviour and source rationale; ≤2% false-answer gate is armed with explicit denominator; no-answer/fact/guardrail/outage strata are reported; current 20-case result remains visible as historical baseline</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
@@ -4409,12 +4456,12 @@
     <row r="53" ht="40" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>S08-02</t>
+          <t>S07-01</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C53" s="20" t="inlineStr">
@@ -4424,35 +4471,35 @@
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>Conversation detail with AI sources</t>
+          <t>QR + embeddable snippet</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>Shows the exact article version the model read.</t>
+          <t>Generated QR per property; one-line embed; logo and colour only.</t>
         </is>
       </c>
       <c r="G53" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>Staff can see the cited text verbatim</t>
+          <t>QR resolves to the right property on a real phone</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr">
@@ -4464,12 +4511,12 @@
     <row r="54" ht="40" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S07-02</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr">
@@ -4479,21 +4526,21 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>Reply, take over, assign, resolve</t>
+          <t>AI disclosure + 'talk to a person'</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>Takeover stops AI guest-facing replies immediately.</t>
+          <t>Persistent, obvious, translated.</t>
         </is>
       </c>
       <c r="G54" s="12" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
@@ -4502,12 +4549,12 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>No race where AI replies after a takeover</t>
+          <t>A human is reachable in one tap from any state</t>
         </is>
       </c>
       <c r="K54" s="11" t="inlineStr">
@@ -4519,12 +4566,12 @@
     <row r="55" ht="40" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>S08-04</t>
+          <t>S07-03</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C55" s="20" t="inlineStr">
@@ -4534,17 +4581,17 @@
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>AI operating modes</t>
+          <t>Request capture + honest acknowledgement</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>Auto / Draft / Human-only / After-hours, feature-flagged per property.</t>
+          <t>'I have sent your request' — never 'on the way'. Creates a service_request.</t>
         </is>
       </c>
       <c r="G55" s="12" t="n">
@@ -4557,12 +4604,12 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>Mode change applies to the next message, no deploy</t>
+          <t>No code path can claim a request is fulfilled</t>
         </is>
       </c>
       <c r="K55" s="11" t="inlineStr">
@@ -4574,12 +4621,12 @@
     <row r="56" ht="40" customHeight="1">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>S09-01</t>
+          <t>S07-04</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
@@ -4589,21 +4636,21 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Request lifecycle</t>
+          <t>Abuse + cost protection</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
         <is>
-          <t>Status, owner, timestamps, internal notes, priority, reopen.</t>
+          <t>Turnstile, per-IP/conversation/property rate limits, daily AI spend cap.</t>
         </is>
       </c>
       <c r="G56" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
@@ -4612,12 +4659,12 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>S07-03</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
         <is>
-          <t>request_acknowledged is set by a real staff action</t>
+          <t>Cap trip degrades to 'a team member will reply' without an error</t>
         </is>
       </c>
       <c r="K56" s="11" t="inlineStr">
@@ -4629,12 +4676,12 @@
     <row r="57" ht="40" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>S09-02</t>
+          <t>S07-05</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C57" s="20" t="inlineStr">
@@ -4644,17 +4691,17 @@
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>Knowledge-gap queue</t>
+          <t>Outage fallback</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>Unanswered and flagged questions with verbatim text, language, property.</t>
+          <t>If AI or provider is down, say so plainly and still capture a request.</t>
         </is>
       </c>
       <c r="G57" s="12" t="n">
@@ -4667,12 +4714,12 @@
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>S05-02</t>
+          <t>S07-04</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>Every no_answer lands in the queue automatically</t>
+          <t>Kill the AI mid-conversation; guest still gets an honest message</t>
         </is>
       </c>
       <c r="K57" s="11" t="inlineStr">
@@ -4684,12 +4731,12 @@
     <row r="58" ht="40" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>S09-03</t>
+          <t>S07-06</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr">
@@ -4699,17 +4746,17 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>One-click 'wrong or outdated'</t>
+          <t>LLM transport resilience</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>Creates or updates a knowledge gap with context.</t>
+          <t>Timeouts, retry with jitter, circuit breaker, pinned model versions, parse-failure alerting.</t>
         </is>
       </c>
       <c r="G58" s="12" t="n">
@@ -4722,12 +4769,12 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>S08-02</t>
+          <t>S05-01</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>A flag is attributable to an ai_run</t>
+          <t>Both providers killed; product degrades honestly</t>
         </is>
       </c>
       <c r="K58" s="11" t="inlineStr">
@@ -4739,12 +4786,12 @@
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>S09-04</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C59" s="20" t="inlineStr">
@@ -4759,16 +4806,16 @@
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>Non-blocking review queue</t>
+          <t>Phone-first shared inbox</t>
         </is>
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>Never gates guest delivery. Replaces Draft as the week-one mechanism.</t>
+          <t>Filters: needs attention, mine, unresolved, unassigned.</t>
         </is>
       </c>
       <c r="G59" s="12" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
@@ -4777,12 +4824,12 @@
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>Flagging an answer does not delay the guest reply</t>
+          <t>An agent triages a queue on a phone in under 60 seconds</t>
         </is>
       </c>
       <c r="K59" s="11" t="inlineStr">
@@ -4794,12 +4841,12 @@
     <row r="60" ht="40" customHeight="1">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>S09-05</t>
+          <t>S08-02</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
@@ -4809,17 +4856,17 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>Email notifications</t>
+          <t>Conversation detail with AI sources</t>
         </is>
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>New request, new handoff, unassigned over 15 minutes. On by default.</t>
+          <t>Shows the exact article version the model read.</t>
         </is>
       </c>
       <c r="G60" s="12" t="n">
@@ -4832,12 +4879,12 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>S09-01</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>A request with no staff view still reaches a human by email</t>
+          <t>Staff can see the cited text verbatim</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
@@ -4849,12 +4896,12 @@
     <row r="61" ht="40" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
@@ -4864,17 +4911,17 @@
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>Event emission across the product</t>
+          <t>Reply, take over, assign, resolve</t>
         </is>
       </c>
       <c r="F61" s="11" t="inlineStr">
         <is>
-          <t>All 18 taxonomy events wired with required context.</t>
+          <t>Takeover stops AI guest-facing replies immediately.</t>
         </is>
       </c>
       <c r="G61" s="12" t="n">
@@ -4887,12 +4934,12 @@
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>W00-19</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>Dashboard numbers reconcile exactly to raw events</t>
+          <t>No race where AI replies after a takeover</t>
         </is>
       </c>
       <c r="K61" s="11" t="inlineStr">
@@ -4904,12 +4951,12 @@
     <row r="62" ht="40" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>S10-02</t>
+          <t>S08-04</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
@@ -4919,17 +4966,17 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>Daily rollups</t>
+          <t>AI operating modes</t>
         </is>
       </c>
       <c r="F62" s="11" t="inlineStr">
         <is>
-          <t>Nightly SQL over events. Idempotent and re-runnable.</t>
+          <t>Auto / Draft / Human-only / After-hours, feature-flagged per property.</t>
         </is>
       </c>
       <c r="G62" s="12" t="n">
@@ -4942,12 +4989,12 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
         <is>
-          <t>A historical date can be recomputed without drift</t>
+          <t>Mode change applies to the next message, no deploy</t>
         </is>
       </c>
       <c r="K62" s="11" t="inlineStr">
@@ -4959,12 +5006,12 @@
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>S10-03</t>
+          <t>S09-01</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C63" s="20" t="inlineStr">
@@ -4974,17 +5021,17 @@
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>Management dashboard</t>
+          <t>Request lifecycle</t>
         </is>
       </c>
       <c r="F63" s="11" t="inlineStr">
         <is>
-          <t>Top questions by property and language, unanswered, request volume and resolution, handoff rate.</t>
+          <t>Status, owner, timestamps, internal notes, priority, reopen.</t>
         </is>
       </c>
       <c r="G63" s="12" t="n">
@@ -4997,12 +5044,12 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>S10-02</t>
+          <t>S07-03</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>Every tile traceable to a query a manager can explain</t>
+          <t>request_acknowledged is set by a real staff action</t>
         </is>
       </c>
       <c r="K63" s="11" t="inlineStr">
@@ -5014,12 +5061,12 @@
     <row r="64" ht="40" customHeight="1">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>S11-01</t>
+          <t>S09-02</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
@@ -5029,21 +5076,21 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>Transactional outbox + worker + DLQ</t>
+          <t>Knowledge-gap queue</t>
         </is>
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>Send outside the request handler; backoff; failures visible.</t>
+          <t>Unanswered and flagged questions with verbatim text, language, property.</t>
         </is>
       </c>
       <c r="G64" s="12" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
@@ -5052,12 +5099,12 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S05-02</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
-          <t>Provider outage delays sends, never loses them</t>
+          <t>Every no_answer lands in the queue automatically</t>
         </is>
       </c>
       <c r="K64" s="11" t="inlineStr">
@@ -5069,12 +5116,12 @@
     <row r="65" ht="40" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>S11-02</t>
+          <t>S09-03</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C65" s="20" t="inlineStr">
@@ -5084,21 +5131,21 @@
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
         <is>
-          <t>Idempotency + webhook dedupe</t>
+          <t>One-click 'wrong or outdated'</t>
         </is>
       </c>
       <c r="F65" s="11" t="inlineStr">
         <is>
-          <t>Unique on (channel_connection_id, channel_message_id).</t>
+          <t>Creates or updates a knowledge gap with context.</t>
         </is>
       </c>
       <c r="G65" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H65" s="11" t="inlineStr">
         <is>
@@ -5107,12 +5154,12 @@
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S08-02</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr">
         <is>
-          <t>Replaying a webhook 10× produces one message</t>
+          <t>A flag is attributable to an ai_run</t>
         </is>
       </c>
       <c r="K65" s="11" t="inlineStr">
@@ -5124,12 +5171,12 @@
     <row r="66" ht="40" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>S11-03</t>
+          <t>S09-04</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
@@ -5139,21 +5186,21 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>PII redaction + log hygiene</t>
+          <t>Non-blocking review queue</t>
         </is>
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>Luhn card detection, long digit runs, emails, phones. No message bodies to third parties.</t>
+          <t>Never gates guest delivery. Replaces Draft as the week-one mechanism.</t>
         </is>
       </c>
       <c r="G66" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H66" s="11" t="inlineStr">
         <is>
@@ -5162,12 +5209,12 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
         <is>
-          <t>A synthetic card number never reaches logs</t>
+          <t>Flagging an answer does not delay the guest reply</t>
         </is>
       </c>
       <c r="K66" s="11" t="inlineStr">
@@ -5179,12 +5226,12 @@
     <row r="67" ht="40" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>S11-04</t>
+          <t>S09-05</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C67" s="20" t="inlineStr">
@@ -5194,17 +5241,17 @@
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>Observability + alerting</t>
+          <t>Email notifications</t>
         </is>
       </c>
       <c r="F67" s="11" t="inlineStr">
         <is>
-          <t>Webhook failures, outbox backlog, LLM errors, spend caps, p95, eval regression.</t>
+          <t>New request, new handoff, unassigned over 15 minutes. On by default.</t>
         </is>
       </c>
       <c r="G67" s="12" t="n">
@@ -5217,12 +5264,12 @@
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>S11-01</t>
+          <t>S09-01</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
         <is>
-          <t>Every alert fires once in staging with a runbook link</t>
+          <t>A request with no staff view still reaches a human by email</t>
         </is>
       </c>
       <c r="K67" s="11" t="inlineStr">
@@ -5234,12 +5281,12 @@
     <row r="68" ht="40" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>S11-05</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr">
@@ -5249,21 +5296,21 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Nightly embedding reconciliation</t>
+          <t>Event emission across the product</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>Every current version has chunks; every chunk resolves to a current version; no orphans.</t>
+          <t>All 18 taxonomy events wired with required context.</t>
         </is>
       </c>
       <c r="G68" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
@@ -5272,12 +5319,12 @@
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>S02-05</t>
+          <t>W00-19</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr">
         <is>
-          <t>Job fails loudly on a seeded drift case</t>
+          <t>Dashboard numbers reconcile exactly to raw events</t>
         </is>
       </c>
       <c r="K68" s="11" t="inlineStr">
@@ -5289,12 +5336,12 @@
     <row r="69" ht="40" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>S12-01</t>
+          <t>S10-02</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C69" s="20" t="inlineStr">
@@ -5304,17 +5351,17 @@
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>Runbook + backup restore drill</t>
+          <t>Daily rollups</t>
         </is>
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>LLM down, WhatsApp down, DB failover, duplicate storm, spend-cap trip, deletion request.</t>
+          <t>Nightly SQL over events. Idempotent and re-runnable.</t>
         </is>
       </c>
       <c r="G69" s="12" t="n">
@@ -5327,12 +5374,12 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>S11-04</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>Restore completed and timed; runbook signed</t>
+          <t>A historical date can be recomputed without drift</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr">
@@ -5344,12 +5391,12 @@
     <row r="70" ht="40" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>S12-02</t>
+          <t>S10-03</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
@@ -5359,35 +5406,35 @@
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Accessibility + ES/EN audit</t>
+          <t>Management dashboard</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>Guest chat and staff UI; a mid-range Android on hotel wifi.</t>
+          <t>Top questions by property and language, unanswered, request volume and resolution, handoff rate.</t>
         </is>
       </c>
       <c r="G70" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S10-02</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
-          <t>Lighthouse a11y ≥90; no untranslated strings</t>
+          <t>Every tile traceable to a query a manager can explain</t>
         </is>
       </c>
       <c r="K70" s="11" t="inlineStr">
@@ -5399,12 +5446,12 @@
     <row r="71" ht="40" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>S12-03</t>
+          <t>S11-01</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C71" s="20" t="inlineStr">
@@ -5419,30 +5466,30 @@
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>Load test</t>
+          <t>Transactional outbox + worker + DLQ</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>300 concurrent guests on one property; 50 staff sessions.</t>
+          <t>Send outside the request handler; backoff; failures visible.</t>
         </is>
       </c>
       <c r="G71" s="12" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>p95 first token ≤3.5s at target load</t>
+          <t>Provider outage delays sends, never loses them</t>
         </is>
       </c>
       <c r="K71" s="11" t="inlineStr">
@@ -5454,36 +5501,36 @@
     <row r="72" ht="40" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S11-02</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
-        </is>
-      </c>
-      <c r="C72" s="21" t="inlineStr">
-        <is>
-          <t>Both</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Pilot dry run with real content</t>
+          <t>Idempotency + webhook dedupe</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Full scripted flow with the hotel's actual staff on their real content.</t>
+          <t>Unique on (channel_connection_id, channel_message_id).</t>
         </is>
       </c>
       <c r="G72" s="12" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
@@ -5492,12 +5539,12 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>S12-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>Three hotel staff complete the flow unaided</t>
+          <t>Replaying a webhook 10× produces one message</t>
         </is>
       </c>
       <c r="K72" s="11" t="inlineStr">
@@ -5509,32 +5556,32 @@
     <row r="73" ht="40" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>S13-01</t>
+          <t>S11-03</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C73" s="19" t="inlineStr">
-        <is>
-          <t>Founder</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>Staff training</t>
+          <t>PII redaction + log hygiene</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>Three staff, scripted flows, escalation expectations, the honest-answer rule.</t>
+          <t>Luhn card detection, long digit runs, emails, phones. No message bodies to third parties.</t>
         </is>
       </c>
       <c r="G73" s="12" t="n">
@@ -5547,12 +5594,12 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>Each staff member completes a live test conversation</t>
+          <t>A synthetic card number never reaches logs</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr">
@@ -5564,36 +5611,36 @@
     <row r="74" ht="40" customHeight="1">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>S13-02</t>
+          <t>S11-04</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C74" s="21" t="inlineStr">
-        <is>
-          <t>Both</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Content corrections from the dry run</t>
+          <t>Observability + alerting</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>Fix what the golden set and the dry run exposed.</t>
+          <t>Webhook failures, outbox backlog, LLM errors, spend caps, p95, eval regression.</t>
         </is>
       </c>
       <c r="G74" s="12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
@@ -5602,12 +5649,12 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S11-01</t>
         </is>
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>No known-wrong article in the published set</t>
+          <t>Every alert fires once in staging with a runbook link</t>
         </is>
       </c>
       <c r="K74" s="11" t="inlineStr">
@@ -5619,32 +5666,32 @@
     <row r="75" ht="40" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>S13-03</t>
+          <t>S11-05</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C75" s="19" t="inlineStr">
-        <is>
-          <t>Founder</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>Launch checklist + GM go/no-go</t>
+          <t>Nightly embedding reconciliation</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>Notifications live, escalation contact confirmed, QR printed, link on the website.</t>
+          <t>Every current version has chunks; every chunk resolves to a current version; no orphans.</t>
         </is>
       </c>
       <c r="G75" s="12" t="n">
@@ -5657,400 +5704,400 @@
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
+          <t>S02-05</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>Job fails loudly on a seeded drift case</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>S12-01</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>Runbook + backup restore drill</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>LLM down, WhatsApp down, DB failover, duplicate storm, spend-cap trip, deletion request.</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>S11-04</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>Restore completed and timed; runbook signed</t>
+        </is>
+      </c>
+      <c r="K76" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>S12-02</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>Accessibility + ES/EN audit</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>Guest chat and staff UI; a mid-range Android on hotel wifi.</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>S08-01</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>Lighthouse a11y ≥90; no untranslated strings</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>S12-03</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>Load test</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>300 concurrent guests on one property; 50 staff sessions.</t>
+        </is>
+      </c>
+      <c r="G78" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>S08-01</t>
+        </is>
+      </c>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>p95 first token ≤3.5s at target load</t>
+        </is>
+      </c>
+      <c r="K78" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C79" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>Pilot dry run with real content</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>Full scripted flow with the hotel's actual staff on their real content.</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>S12-01</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>Three hotel staff complete the flow unaided</t>
+        </is>
+      </c>
+      <c r="K79" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
           <t>S13-01</t>
         </is>
       </c>
-      <c r="J75" s="11" t="inlineStr">
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C80" s="19" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>Staff training</t>
+        </is>
+      </c>
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>Three staff, scripted flows, escalation expectations, the honest-answer rule.</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I80" s="11" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="J80" s="11" t="inlineStr">
+        <is>
+          <t>Each staff member completes a live test conversation</t>
+        </is>
+      </c>
+      <c r="K80" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>S13-02</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C81" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>Content corrections from the dry run</t>
+        </is>
+      </c>
+      <c r="F81" s="11" t="inlineStr">
+        <is>
+          <t>Fix what the golden set and the dry run exposed.</t>
+        </is>
+      </c>
+      <c r="G81" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>No known-wrong article in the published set</t>
+        </is>
+      </c>
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>S13-03</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C82" s="19" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>Launch checklist + GM go/no-go</t>
+        </is>
+      </c>
+      <c r="F82" s="11" t="inlineStr">
+        <is>
+          <t>Notifications live, escalation contact confirmed, QR printed, link on the website.</t>
+        </is>
+      </c>
+      <c r="G82" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H82" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>S13-01</t>
+        </is>
+      </c>
+      <c r="J82" s="11" t="inlineStr">
         <is>
           <t>Written go/no-go from the GM</t>
         </is>
       </c>
-      <c r="K75" s="11" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="22" t="inlineStr">
-        <is>
-          <t>WA-01</t>
-        </is>
-      </c>
-      <c r="B76" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C76" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D76" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E76" s="23" t="inlineStr">
-        <is>
-          <t>Payment method on WABA</t>
-        </is>
-      </c>
-      <c r="F76" s="23" t="inlineStr">
-        <is>
-          <t>Without it, service messages beyond 1,000/month do not deliver.</t>
-        </is>
-      </c>
-      <c r="G76" s="24" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H76" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I76" s="23" t="inlineStr">
-        <is>
-          <t>W00-08</t>
-        </is>
-      </c>
-      <c r="J76" s="23" t="inlineStr">
-        <is>
-          <t>Billing active; spend alert configured</t>
-        </is>
-      </c>
-      <c r="K76" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="22" t="inlineStr">
-        <is>
-          <t>WA-02</t>
-        </is>
-      </c>
-      <c r="B77" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C77" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D77" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E77" s="23" t="inlineStr">
-        <is>
-          <t>Adapter: webhook ingress</t>
-        </is>
-      </c>
-      <c r="F77" s="23" t="inlineStr">
-        <is>
-          <t>Verify signature, dedupe, normalise, acknowledge under 3 seconds.</t>
-        </is>
-      </c>
-      <c r="G77" s="24" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H77" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I77" s="23" t="inlineStr">
-        <is>
-          <t>W00-09</t>
-        </is>
-      </c>
-      <c r="J77" s="23" t="inlineStr">
-        <is>
-          <t>A replayed webhook produces exactly one message</t>
-        </is>
-      </c>
-      <c r="K77" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="22" t="inlineStr">
-        <is>
-          <t>WA-03</t>
-        </is>
-      </c>
-      <c r="B78" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D78" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E78" s="23" t="inlineStr">
-        <is>
-          <t>Adapter: send path + 24h window</t>
-        </is>
-      </c>
-      <c r="F78" s="23" t="inlineStr">
-        <is>
-          <t>Window tracking per conversation. Templates outside, free-form inside.</t>
-        </is>
-      </c>
-      <c r="G78" s="24" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H78" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I78" s="23" t="inlineStr">
-        <is>
-          <t>WA-02</t>
-        </is>
-      </c>
-      <c r="J78" s="23" t="inlineStr">
-        <is>
-          <t>Sending outside the window impossible without a template</t>
-        </is>
-      </c>
-      <c r="K78" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="22" t="inlineStr">
-        <is>
-          <t>WA-04</t>
-        </is>
-      </c>
-      <c r="B79" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D79" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E79" s="23" t="inlineStr">
-        <is>
-          <t>Consent + opt-out store</t>
-        </is>
-      </c>
-      <c r="F79" s="23" t="inlineStr">
-        <is>
-          <t>Explicit consent records, STOP handling, rules isolated in the adapter.</t>
-        </is>
-      </c>
-      <c r="G79" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I79" s="23" t="inlineStr">
-        <is>
-          <t>WA-03</t>
-        </is>
-      </c>
-      <c r="J79" s="23" t="inlineStr">
-        <is>
-          <t>Opt-out honoured across every send path</t>
-        </is>
-      </c>
-      <c r="K79" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="22" t="inlineStr">
-        <is>
-          <t>WA-05</t>
-        </is>
-      </c>
-      <c r="B80" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C80" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D80" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E80" s="23" t="inlineStr">
-        <is>
-          <t>Message-efficient reply composition</t>
-        </is>
-      </c>
-      <c r="F80" s="23" t="inlineStr">
-        <is>
-          <t>One complete reply per turn. No streaming into WhatsApp — every bubble is billable.</t>
-        </is>
-      </c>
-      <c r="G80" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H80" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I80" s="23" t="inlineStr">
-        <is>
-          <t>S05-02</t>
-        </is>
-      </c>
-      <c r="J80" s="23" t="inlineStr">
-        <is>
-          <t>A typical exchange stays within the message budget</t>
-        </is>
-      </c>
-      <c r="K80" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="40" customHeight="1">
-      <c r="A81" s="22" t="inlineStr">
-        <is>
-          <t>WA-06</t>
-        </is>
-      </c>
-      <c r="B81" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C81" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D81" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E81" s="23" t="inlineStr">
-        <is>
-          <t>Template submission + approval</t>
-        </is>
-      </c>
-      <c r="F81" s="23" t="inlineStr">
-        <is>
-          <t>Utility templates for outside-window replies.</t>
-        </is>
-      </c>
-      <c r="G81" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H81" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I81" s="23" t="inlineStr">
-        <is>
-          <t>W00-09</t>
-        </is>
-      </c>
-      <c r="J81" s="23" t="inlineStr">
-        <is>
-          <t>Templates approved and sendable</t>
-        </is>
-      </c>
-      <c r="K81" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="40" customHeight="1">
-      <c r="A82" s="22" t="inlineStr">
-        <is>
-          <t>WA-07</t>
-        </is>
-      </c>
-      <c r="B82" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C82" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D82" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E82" s="23" t="inlineStr">
-        <is>
-          <t>Number-migration safeguards</t>
-        </is>
-      </c>
-      <c r="F82" s="23" t="inlineStr">
-        <is>
-          <t>Warn that migrating a number deletes consumer WhatsApp history.</t>
-        </is>
-      </c>
-      <c r="G82" s="24" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H82" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I82" s="23" t="inlineStr">
-        <is>
-          <t>W00-04</t>
-        </is>
-      </c>
-      <c r="J82" s="23" t="inlineStr">
-        <is>
-          <t>Written acknowledgement captured in onboarding</t>
-        </is>
-      </c>
-      <c r="K82" s="23" t="inlineStr">
+      <c r="K82" s="11" t="inlineStr">
         <is>
           <t>☐ Not started</t>
         </is>
@@ -6059,163 +6106,548 @@
     <row r="83" ht="40" customHeight="1">
       <c r="A83" s="22" t="inlineStr">
         <is>
+          <t>WA-01</t>
+        </is>
+      </c>
+      <c r="B83" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D83" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E83" s="23" t="inlineStr">
+        <is>
+          <t>Payment method on WABA</t>
+        </is>
+      </c>
+      <c r="F83" s="23" t="inlineStr">
+        <is>
+          <t>Without it, service messages beyond 1,000/month do not deliver.</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H83" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I83" s="23" t="inlineStr">
+        <is>
+          <t>W00-08</t>
+        </is>
+      </c>
+      <c r="J83" s="23" t="inlineStr">
+        <is>
+          <t>Billing active; spend alert configured</t>
+        </is>
+      </c>
+      <c r="K83" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>WA-02</t>
+        </is>
+      </c>
+      <c r="B84" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E84" s="23" t="inlineStr">
+        <is>
+          <t>Adapter: webhook ingress</t>
+        </is>
+      </c>
+      <c r="F84" s="23" t="inlineStr">
+        <is>
+          <t>Verify signature, dedupe, normalise, acknowledge under 3 seconds.</t>
+        </is>
+      </c>
+      <c r="G84" s="24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H84" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I84" s="23" t="inlineStr">
+        <is>
+          <t>W00-09</t>
+        </is>
+      </c>
+      <c r="J84" s="23" t="inlineStr">
+        <is>
+          <t>A replayed webhook produces exactly one message</t>
+        </is>
+      </c>
+      <c r="K84" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>WA-03</t>
+        </is>
+      </c>
+      <c r="B85" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D85" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E85" s="23" t="inlineStr">
+        <is>
+          <t>Adapter: send path + 24h window</t>
+        </is>
+      </c>
+      <c r="F85" s="23" t="inlineStr">
+        <is>
+          <t>Window tracking per conversation. Templates outside, free-form inside.</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H85" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I85" s="23" t="inlineStr">
+        <is>
+          <t>WA-02</t>
+        </is>
+      </c>
+      <c r="J85" s="23" t="inlineStr">
+        <is>
+          <t>Sending outside the window impossible without a template</t>
+        </is>
+      </c>
+      <c r="K85" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>WA-04</t>
+        </is>
+      </c>
+      <c r="B86" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D86" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E86" s="23" t="inlineStr">
+        <is>
+          <t>Consent + opt-out store</t>
+        </is>
+      </c>
+      <c r="F86" s="23" t="inlineStr">
+        <is>
+          <t>Explicit consent records, STOP handling, rules isolated in the adapter.</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I86" s="23" t="inlineStr">
+        <is>
+          <t>WA-03</t>
+        </is>
+      </c>
+      <c r="J86" s="23" t="inlineStr">
+        <is>
+          <t>Opt-out honoured across every send path</t>
+        </is>
+      </c>
+      <c r="K86" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>WA-05</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D87" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E87" s="23" t="inlineStr">
+        <is>
+          <t>Message-efficient reply composition</t>
+        </is>
+      </c>
+      <c r="F87" s="23" t="inlineStr">
+        <is>
+          <t>One complete reply per turn. No streaming into WhatsApp — every bubble is billable.</t>
+        </is>
+      </c>
+      <c r="G87" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I87" s="23" t="inlineStr">
+        <is>
+          <t>S05-02</t>
+        </is>
+      </c>
+      <c r="J87" s="23" t="inlineStr">
+        <is>
+          <t>A typical exchange stays within the message budget</t>
+        </is>
+      </c>
+      <c r="K87" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="22" t="inlineStr">
+        <is>
+          <t>WA-06</t>
+        </is>
+      </c>
+      <c r="B88" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D88" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E88" s="23" t="inlineStr">
+        <is>
+          <t>Template submission + approval</t>
+        </is>
+      </c>
+      <c r="F88" s="23" t="inlineStr">
+        <is>
+          <t>Utility templates for outside-window replies.</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I88" s="23" t="inlineStr">
+        <is>
+          <t>W00-09</t>
+        </is>
+      </c>
+      <c r="J88" s="23" t="inlineStr">
+        <is>
+          <t>Templates approved and sendable</t>
+        </is>
+      </c>
+      <c r="K88" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="22" t="inlineStr">
+        <is>
+          <t>WA-07</t>
+        </is>
+      </c>
+      <c r="B89" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D89" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E89" s="23" t="inlineStr">
+        <is>
+          <t>Number-migration safeguards</t>
+        </is>
+      </c>
+      <c r="F89" s="23" t="inlineStr">
+        <is>
+          <t>Warn that migrating a number deletes consumer WhatsApp history.</t>
+        </is>
+      </c>
+      <c r="G89" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H89" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I89" s="23" t="inlineStr">
+        <is>
+          <t>W00-04</t>
+        </is>
+      </c>
+      <c r="J89" s="23" t="inlineStr">
+        <is>
+          <t>Written acknowledgement captured in onboarding</t>
+        </is>
+      </c>
+      <c r="K89" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="22" t="inlineStr">
+        <is>
           <t>WA-08</t>
         </is>
       </c>
-      <c r="B83" s="23" t="inlineStr">
+      <c r="B90" s="23" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="C83" s="20" t="inlineStr">
+      <c r="C90" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D83" s="23" t="inlineStr">
+      <c r="D90" s="23" t="inlineStr">
         <is>
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="E83" s="23" t="inlineStr">
+      <c r="E90" s="23" t="inlineStr">
         <is>
           <t>Shadow run on one property</t>
         </is>
       </c>
-      <c r="F83" s="23" t="inlineStr">
+      <c r="F90" s="23" t="inlineStr">
         <is>
           <t>Run alongside web chat for a week before switching traffic.</t>
         </is>
       </c>
-      <c r="G83" s="24" t="n">
+      <c r="G90" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="H83" s="23" t="inlineStr">
+      <c r="H90" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I83" s="23" t="inlineStr">
+      <c r="I90" s="23" t="inlineStr">
         <is>
           <t>WA-03</t>
         </is>
       </c>
-      <c r="J83" s="23" t="inlineStr">
+      <c r="J90" s="23" t="inlineStr">
         <is>
           <t>Zero delivery failures across 7 days</t>
         </is>
       </c>
-      <c r="K83" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="25" t="inlineStr">
+      <c r="K90" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="25" t="inlineStr">
         <is>
           <t>DF-01</t>
         </is>
       </c>
-      <c r="B84" s="26" t="inlineStr">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>DEF</t>
         </is>
       </c>
-      <c r="C84" s="20" t="inlineStr">
+      <c r="C91" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D84" s="26" t="inlineStr">
+      <c r="D91" s="26" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
       </c>
-      <c r="E84" s="26" t="inlineStr">
+      <c r="E91" s="26" t="inlineStr">
         <is>
           <t>Outbound webhook per property</t>
         </is>
       </c>
-      <c r="F84" s="26" t="inlineStr">
+      <c r="F91" s="26" t="inlineStr">
         <is>
           <t>Signed, retried events to Teams/Slack/hotel ops tools.</t>
         </is>
       </c>
-      <c r="G84" s="27" t="n">
+      <c r="G91" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="H84" s="26" t="inlineStr">
+      <c r="H91" s="26" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I84" s="26" t="inlineStr">
+      <c r="I91" s="26" t="inlineStr">
         <is>
           <t>S09-05</t>
         </is>
       </c>
-      <c r="J84" s="26" t="inlineStr">
+      <c r="J91" s="26" t="inlineStr">
         <is>
           <t>A group needs events piped into their own tools</t>
         </is>
       </c>
-      <c r="K84" s="26" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="25" t="inlineStr">
+      <c r="K91" s="26" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="25" t="inlineStr">
         <is>
           <t>DF-02</t>
         </is>
       </c>
-      <c r="B85" s="26" t="inlineStr">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>DEF</t>
         </is>
       </c>
-      <c r="C85" s="20" t="inlineStr">
+      <c r="C92" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D85" s="26" t="inlineStr">
+      <c r="D92" s="26" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="E85" s="26" t="inlineStr">
+      <c r="E92" s="26" t="inlineStr">
         <is>
           <t>Opportunity click tracking</t>
         </is>
       </c>
-      <c r="F85" s="26" t="inlineStr">
+      <c r="F92" s="26" t="inlineStr">
         <is>
           <t>Booking/dining/spa link clicks, labelled opportunities, never revenue.</t>
         </is>
       </c>
-      <c r="G85" s="27" t="n">
+      <c r="G92" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="H85" s="26" t="inlineStr">
+      <c r="H92" s="26" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I85" s="26" t="inlineStr">
+      <c r="I92" s="26" t="inlineStr">
         <is>
           <t>S10-01</t>
         </is>
       </c>
-      <c r="J85" s="26" t="inlineStr">
+      <c r="J92" s="26" t="inlineStr">
         <is>
           <t>After the pilot, against real traffic</t>
         </is>
       </c>
-      <c r="K85" s="26" t="inlineStr">
+      <c r="K92" s="26" t="inlineStr">
         <is>
           <t>☐ Not started</t>
         </is>
@@ -6223,7 +6655,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"☐ Not started,◐ In progress,☑ Done,✖ Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6238,7 +6670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6550,117 +6982,121 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Chat hardening</t>
+          <t>API, deployment and eval reliability</t>
         </is>
       </c>
       <c r="D12" s="12" t="n">
-        <v>4</v>
+        <v>14.5</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="29" t="inlineStr">
-        <is>
-          <t>Fits</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr"/>
+        <v>14.5</v>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>Over by 9.50</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Spills into the following week.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Staff inbox</t>
+          <t>Chat hardening</t>
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G13" s="28" t="inlineStr">
-        <is>
-          <t>Over by 0.50</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>Spills into the following week.</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>Fits</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Requests and notifications</t>
+          <t>Staff inbox</t>
         </is>
       </c>
       <c r="D14" s="12" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G14" s="29" t="inlineStr">
-        <is>
-          <t>Fits</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr"/>
+        <v>5.5</v>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Over by 0.50</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Spills into the following week.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Requests and notifications</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
@@ -6682,27 +7118,27 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="D16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G16" s="29" t="inlineStr">
         <is>
@@ -6714,27 +7150,27 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Pilot readiness</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G17" s="29" t="inlineStr">
         <is>
@@ -6746,67 +7182,99 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Pilot readiness</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>Fits</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
           <t>S13</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D19" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E19" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="29" t="inlineStr">
+      <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Fits</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Launch work plus ~3 days of carry-forward room.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="5" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Original launch date invalid after 14.50-day S06A; reforecast with owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Total demand</t>
         </is>
       </c>
-      <c r="F20" s="30" t="n">
+      <c r="F21" s="30" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Original capacity (14 × 5)</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="21">
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Capacity (14 × 5)</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Unallocated</t>
-        </is>
-      </c>
-      <c r="F22" s="31" t="n">
-        <v>0</v>
+    <row r="23">
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Over capacity</t>
+        </is>
+      </c>
+      <c r="F23" s="31" t="n">
+        <v>14.5</v>
       </c>
     </row>
   </sheetData>
@@ -7007,7 +7475,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Pilot live</t>
+          <t>Pilot live (original target; reforecast)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -7017,7 +7485,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>After S06A</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -7027,7 +7495,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Postpone a week; do not launch untrained</t>
+          <t>Do not commit to W14 until staffing/parallelism is re-estimated</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7517,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>Reforecast</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -7081,7 +7549,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>Reforecast</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -7158,7 +7626,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Each step blocks the next. Any slip here moves W14 one-for-one.</t>
+          <t>Each step blocks the next. S06A is inserted before S07; recalculate launch after sequencing.</t>
         </is>
       </c>
     </row>
@@ -7412,7 +7880,7 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Analytics (S10), reliability (S11), accessibility and load (S12) — each can slip a week without moving W14.</t>
+          <t>Original W14 date is unconfirmed after S06A; reforecast before using dates for commitments.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: plan S06A API, deploy and eval reliability (#174)
Co-authored-by: jtanori <920148+jtanori@users.noreply.github.com>
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/07-master-backlog.xlsx
+++ b/docs/07-master-backlog.xlsx
@@ -100,17 +100,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -182,17 +182,17 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -216,11 +216,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +605,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Single source of truth for the build · 81 items · 14 sprints · 21 Oct 2026</t>
+          <t>Single source of truth for the build · 88 items · 15 work blocks including ASAP S06A · 21 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -621,15 +621,15 @@
       </c>
       <c r="C6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Lean pilot path</t>
+          <t>Planned engineering path</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>70.00 dev-days across 14 sprints (W00, S01–S13). Pilot live Monday of W14.</t>
+          <t>84.50 dev-days across original 14 sprints plus ASAP S06A. Original W14 pilot forecast must be revised.</t>
         </is>
       </c>
     </row>
@@ -665,14 +665,14 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>79.25 dev-days across 81 items.</t>
+          <t>93.75 dev-days across 88 items.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Original capacity</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -684,12 +684,12 @@
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Slack</t>
+          <t>Net change</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>0.00 days unallocated. W13 carries 2.00 days of launch work, leaving ~3 days of carry-forward room in that week.</t>
+          <t>+14.50 days vs original 70-day plan; S06A adds 14.50 engineering days and is not absorbed by W13 slack.</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>14 sprints: goal, items, days, cumulative weeks, gate, exit criterion.</t>
+          <t>15 work blocks: goal, items, days, cumulative weeks, gate, exit criterion.</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>All 81 items with sprint, track, estimate, dependency and acceptance criteria. The working board.</t>
+          <t>All 88 items with sprint, track, estimate, dependency and acceptance criteria. The working board.</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -880,14 +880,14 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Sprint ladder — 14 sprints to pilot</t>
+          <t>Sprint ladder — original plan plus ASAP S06A</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Cumulative weeks is the true elapsed position. Work completes at 14.00 weeks; W14 is launch.</t>
+          <t>Cumulative effort is shown; ASAP S06A invalidates the original W14 launch forecast until resequenced.</t>
         </is>
       </c>
     </row>
@@ -1280,85 +1280,85 @@
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Chat hardening</t>
+          <t>API, deployment and eval reliability</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Abuse, outages and provider failure</t>
+          <t>Make release and answer-quality evidence trustworthy</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>4</v>
+        <v>14.5</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>44</v>
+        <v>54.5</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>10.9</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>G2 remediation</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>AI killed mid-conversation still yields an honest reply and a ticket · cap trip degrades gracefully</t>
+          <t>Full API surface has a documented contract and reachable deployment · deploys follow native Vercel Git integration with enforced CI · live canary diagnostics identify real retrieval/fact/guardrail cause · G2 measured on a sufficiently large, representative set</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Staff inbox</t>
+          <t>Chat hardening</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>The surface an agent actually uses</t>
+          <t>Abuse, outages and provider failure</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="12" t="n">
-        <v>5.5</v>
-      </c>
       <c r="G13" s="12" t="n">
-        <v>49.5</v>
+        <v>58.5</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>-0.5</v>
+        <v>11.7</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
@@ -1367,45 +1367,45 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>An agent triages a queue on a phone in under 60 seconds · takeover is atomic</t>
+          <t>AI killed mid-conversation still yields an honest reply and a ticket · cap trip degrades gracefully</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Requests and notifications</t>
+          <t>Staff inbox</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>A request nobody sees is not a request</t>
+          <t>The surface an agent actually uses</t>
         </is>
       </c>
       <c r="E14" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>0.5</v>
+        <v>12.8</v>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>-0.5</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -1414,42 +1414,42 @@
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>Ack timestamp set by a real staff action · a request with no staff view still reaches a human</t>
+          <t>An agent triages a queue on a phone in under 60 seconds · takeover is atomic</t>
         </is>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Requests and notifications</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>What guests ask, and what we cannot answer</t>
+          <t>A request nobody sees is not a request</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F15" s="12" t="n">
         <v>4.5</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>58.5</v>
+        <v>68.5</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>11.7</v>
+        <v>13.7</v>
       </c>
       <c r="I15" s="12" t="n">
         <v>0.5</v>
@@ -1461,45 +1461,45 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Dashboard numbers reconcile exactly to raw events · every tile traceable to a query</t>
+          <t>Ack timestamp set by a real staff action · a request with no staff view still reaches a human</t>
         </is>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Outbox, idempotency, redaction, observability</t>
+          <t>What guests ask, and what we cannot answer</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>63.5</v>
+        <v>73</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>12.7</v>
+        <v>14.6</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
@@ -1508,160 +1508,207 @@
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Provider outage causes delayed sends, not lost messages · no card number reaches logs</t>
+          <t>Dashboard numbers reconcile exactly to raw events · every tile traceable to a query</t>
         </is>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Pilot readiness</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Prove it works before a guest sees it</t>
+          <t>Outbox, idempotency, redaction, observability</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>13.6</v>
+        <v>15.6</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>G3</t>
+        <v>0</v>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Restore drilled and timed · three staff complete the flow unaided · runbook signed off</t>
+          <t>Provider outage causes delayed sends, not lost messages · no card number reaches logs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Pilot readiness</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Prove it works before a guest sees it</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>Restore drilled and timed · three staff complete the flow unaided · runbook signed off</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
           <t>S13</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Train the staff, fix the content, go/no-go</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E19" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="H18" s="12" t="n">
-        <v>14</v>
-      </c>
-      <c r="I18" s="12" t="n">
+      <c r="G19" s="12" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I19" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="11" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K18" s="11" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>Pilot property trained · content corrections applied · GM sign-off recorded</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>LEAN PILOT PATH</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="16" t="n">
-        <v>71</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="16" t="n">
-        <v>14</v>
-      </c>
-      <c r="I19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-    </row>
-    <row r="21">
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Pilot live</t>
-        </is>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>Monday W14</t>
-        </is>
-      </c>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>PLANNED ENGINEERING PATH</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="16" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I20" s="16" t="n">
+        <v>-14.5</v>
+      </c>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Pilot readout</t>
+          <t>Pilot live</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>W17 (G4)</t>
+          <t>Forecast after S06A</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t>Pilot readout</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>W17 (G4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
           <t>WhatsApp live</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>W18 (G5)</t>
         </is>
@@ -1679,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4024,12 +4071,12 @@
     <row r="46" ht="40" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>S07-01</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr">
@@ -4039,35 +4086,35 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>QR + embeddable snippet</t>
+          <t>Eval attribution and retrieval diagnostics</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>Generated QR per property; one-line embed; logo and colour only.</t>
+          <t>Correctly distinguish pre-retrieval guardrails, structured facts, retrieval candidates, model refusals and provider outages; retain safe per-question diagnostics.</t>
         </is>
       </c>
       <c r="G46" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S06-03</t>
         </is>
       </c>
       <c r="J46" s="11" t="inlineStr">
         <is>
-          <t>QR resolves to the right property on a real phone</t>
+          <t>For every golden row, report pipeline stage, outcome/reason, target-topic retrieval hit and safe retrieved-topic diagnostics; synthetic tests reproduce each bucket and no failure is reported as retrieval-empty unless retrieval was actually empty</t>
         </is>
       </c>
       <c r="K46" s="11" t="inlineStr">
@@ -4079,12 +4126,12 @@
     <row r="47" ht="40" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>S07-02</t>
+          <t>S06A-02</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C47" s="20" t="inlineStr">
@@ -4094,21 +4141,21 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>AI disclosure + 'talk to a person'</t>
+          <t>Sensitive and policy classifier calibration</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>Persistent, obvious, translated.</t>
+          <t>Replace broad phrase collisions with intent-aware, bilingual rules; protect deliberate escalation for refund, booking and safety requests while permitting factual property questions.</t>
         </is>
       </c>
       <c r="G47" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
@@ -4117,12 +4164,12 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>A human is reachable in one tap from any state</t>
+          <t>Regression tests cover price questions for known services, booking/transacting requests, extra-bed policy, pet policy, explicit handoff, refunds, allergy and accessibility; no escalation rule is weakened without safety tests</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
@@ -4134,12 +4181,12 @@
     <row r="48" ht="40" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>S07-03</t>
+          <t>S06A-03</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
@@ -4149,21 +4196,21 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>Request capture + honest acknowledgement</t>
+          <t>Guest intent classification and structured-fact routing</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>'I have sent your request' — never 'on the way'. Creates a service_request.</t>
+          <t>Add a conservative, auditable route from guest question to allowed topic/fact keys; unknown or ambiguous intent falls back to retrieval/handoff and never trusts golden labels at runtime.</t>
         </is>
       </c>
       <c r="G48" s="12" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
@@ -4172,12 +4219,12 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-02</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
         <is>
-          <t>No code path can claim a request is fulfilled</t>
+          <t>Property fact questions in English and Spanish reach verified fact lookup using inferred topic/fact keys; wrong/absent fact falls back safely; tests prove no caller-supplied tenant/topic label bypasses policy</t>
         </is>
       </c>
       <c r="K48" s="11" t="inlineStr">
@@ -4189,12 +4236,12 @@
     <row r="49" ht="40" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>S07-04</t>
+          <t>S06A-04</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C49" s="20" t="inlineStr">
@@ -4204,21 +4251,21 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Abuse + cost protection</t>
+          <t>Cross-language knowledge and retrieval quality</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Turnstile, per-IP/conversation/property rate limits, daily AI spend cap.</t>
+          <t>Ensure Spanish guest questions can retrieve approved English or Spanish knowledge without inventing translations or weakening tenant/current-version filters.</t>
         </is>
       </c>
       <c r="G49" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
@@ -4227,12 +4274,12 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>Cap trip degrades to 'a team member will reply' without an error</t>
+          <t>Bilingual paraphrase retrieval suite meets ≥90% target-topic recall on frozen cases; exact-language and cross-language cases, noise, no-match and tenant isolation are covered; only approved content is cited</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
@@ -4244,12 +4291,12 @@
     <row r="50" ht="40" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>S07-05</t>
+          <t>S06A-05</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
@@ -4259,21 +4306,21 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Outage fallback</t>
+          <t>API contract and runtime decision</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>If AI or provider is down, say so plainly and still capture a request.</t>
+          <t>Inventory all implemented and deployed routes; specify OpenAPI contracts; prove representative guest/staff paths against the selected runtime and document Vercel Functions versus persistent-service decision.</t>
         </is>
       </c>
       <c r="G50" s="12" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
@@ -4282,12 +4329,12 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>S07-04</t>
+          <t>S06A-01</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
-          <t>Kill the AI mid-conversation; guest still gets an honest message</t>
+          <t>Every route used by web is mapped to handler, auth/tenant policy, schema, response and deployment adapter; contract validation and HTTP integration tests pass; runtime decision cites measured duration, DB pooling and worker constraints</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
@@ -4299,12 +4346,12 @@
     <row r="51" ht="40" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>S07-06</t>
+          <t>S06A-06</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr">
@@ -4314,21 +4361,21 @@
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>LLM transport resilience</t>
+          <t>Native Vercel Git deploys for API and web</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>Timeouts, retry with jitter, circuit breaker, pinned model versions, parse-failure alerting.</t>
+          <t>Configure both Vercel projects for explicit roots/builds and Git-based preview/staging/production deployment; retire alias pinning/CLI deployment only after proof.</t>
         </is>
       </c>
       <c r="G51" s="12" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
@@ -4337,12 +4384,12 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>S05-01</t>
+          <t>S06A-05</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>Both providers killed; product degrades honestly</t>
+          <t>API and web preview from same commit; protected staging has stable Vercel branch/domain binding; production deploys from agreed branch; deliberately failing required CI check blocks promotion; no alias-pinning step or GitHub Vercel token needed for routine deploy</t>
         </is>
       </c>
       <c r="K51" s="11" t="inlineStr">
@@ -4354,12 +4401,12 @@
     <row r="52" ht="40" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06A-07</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
@@ -4369,21 +4416,21 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Phone-first shared inbox</t>
+          <t>Representative golden set and gate arming</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>Filters: needs attention, mine, unresolved, unassigned.</t>
+          <t>Expand and curate golden set to at least 50 reviewed cases with adequate answer/escalation and language/topic coverage; re-baseline deterministic eval and canary without hiding the current failure.</t>
         </is>
       </c>
       <c r="G52" s="12" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
@@ -4392,12 +4439,12 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>S06-02</t>
+          <t>S06A-01, S06A-02, S06A-03, S06A-04</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
-          <t>An agent triages a queue on a phone in under 60 seconds</t>
+          <t>At least 50 reviewed questions include target language/topic, expected behaviour and source rationale; ≤2% false-answer gate is armed with explicit denominator; no-answer/fact/guardrail/outage strata are reported; current 20-case result remains visible as historical baseline</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
@@ -4409,12 +4456,12 @@
     <row r="53" ht="40" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>S08-02</t>
+          <t>S07-01</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C53" s="20" t="inlineStr">
@@ -4424,35 +4471,35 @@
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>Conversation detail with AI sources</t>
+          <t>QR + embeddable snippet</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>Shows the exact article version the model read.</t>
+          <t>Generated QR per property; one-line embed; logo and colour only.</t>
         </is>
       </c>
       <c r="G53" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>Staff can see the cited text verbatim</t>
+          <t>QR resolves to the right property on a real phone</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr">
@@ -4464,12 +4511,12 @@
     <row r="54" ht="40" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S07-02</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr">
@@ -4479,21 +4526,21 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>Reply, take over, assign, resolve</t>
+          <t>AI disclosure + 'talk to a person'</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>Takeover stops AI guest-facing replies immediately.</t>
+          <t>Persistent, obvious, translated.</t>
         </is>
       </c>
       <c r="G54" s="12" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
@@ -4502,12 +4549,12 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>No race where AI replies after a takeover</t>
+          <t>A human is reachable in one tap from any state</t>
         </is>
       </c>
       <c r="K54" s="11" t="inlineStr">
@@ -4519,12 +4566,12 @@
     <row r="55" ht="40" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>S08-04</t>
+          <t>S07-03</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C55" s="20" t="inlineStr">
@@ -4534,17 +4581,17 @@
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>AI operating modes</t>
+          <t>Request capture + honest acknowledgement</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>Auto / Draft / Human-only / After-hours, feature-flagged per property.</t>
+          <t>'I have sent your request' — never 'on the way'. Creates a service_request.</t>
         </is>
       </c>
       <c r="G55" s="12" t="n">
@@ -4557,12 +4604,12 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>Mode change applies to the next message, no deploy</t>
+          <t>No code path can claim a request is fulfilled</t>
         </is>
       </c>
       <c r="K55" s="11" t="inlineStr">
@@ -4574,12 +4621,12 @@
     <row r="56" ht="40" customHeight="1">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>S09-01</t>
+          <t>S07-04</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
@@ -4589,21 +4636,21 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Request lifecycle</t>
+          <t>Abuse + cost protection</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
         <is>
-          <t>Status, owner, timestamps, internal notes, priority, reopen.</t>
+          <t>Turnstile, per-IP/conversation/property rate limits, daily AI spend cap.</t>
         </is>
       </c>
       <c r="G56" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
@@ -4612,12 +4659,12 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>S07-03</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
         <is>
-          <t>request_acknowledged is set by a real staff action</t>
+          <t>Cap trip degrades to 'a team member will reply' without an error</t>
         </is>
       </c>
       <c r="K56" s="11" t="inlineStr">
@@ -4629,12 +4676,12 @@
     <row r="57" ht="40" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>S09-02</t>
+          <t>S07-05</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C57" s="20" t="inlineStr">
@@ -4644,17 +4691,17 @@
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>Knowledge-gap queue</t>
+          <t>Outage fallback</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>Unanswered and flagged questions with verbatim text, language, property.</t>
+          <t>If AI or provider is down, say so plainly and still capture a request.</t>
         </is>
       </c>
       <c r="G57" s="12" t="n">
@@ -4667,12 +4714,12 @@
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>S05-02</t>
+          <t>S07-04</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>Every no_answer lands in the queue automatically</t>
+          <t>Kill the AI mid-conversation; guest still gets an honest message</t>
         </is>
       </c>
       <c r="K57" s="11" t="inlineStr">
@@ -4684,12 +4731,12 @@
     <row r="58" ht="40" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>S09-03</t>
+          <t>S07-06</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr">
@@ -4699,17 +4746,17 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Inbox</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>One-click 'wrong or outdated'</t>
+          <t>LLM transport resilience</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>Creates or updates a knowledge gap with context.</t>
+          <t>Timeouts, retry with jitter, circuit breaker, pinned model versions, parse-failure alerting.</t>
         </is>
       </c>
       <c r="G58" s="12" t="n">
@@ -4722,12 +4769,12 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>S08-02</t>
+          <t>S05-01</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>A flag is attributable to an ai_run</t>
+          <t>Both providers killed; product degrades honestly</t>
         </is>
       </c>
       <c r="K58" s="11" t="inlineStr">
@@ -4739,12 +4786,12 @@
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>S09-04</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C59" s="20" t="inlineStr">
@@ -4759,16 +4806,16 @@
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>Non-blocking review queue</t>
+          <t>Phone-first shared inbox</t>
         </is>
       </c>
       <c r="F59" s="11" t="inlineStr">
         <is>
-          <t>Never gates guest delivery. Replaces Draft as the week-one mechanism.</t>
+          <t>Filters: needs attention, mine, unresolved, unassigned.</t>
         </is>
       </c>
       <c r="G59" s="12" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
@@ -4777,12 +4824,12 @@
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>S08-03</t>
+          <t>S06-02</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>Flagging an answer does not delay the guest reply</t>
+          <t>An agent triages a queue on a phone in under 60 seconds</t>
         </is>
       </c>
       <c r="K59" s="11" t="inlineStr">
@@ -4794,12 +4841,12 @@
     <row r="60" ht="40" customHeight="1">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>S09-05</t>
+          <t>S08-02</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
@@ -4809,17 +4856,17 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>Email notifications</t>
+          <t>Conversation detail with AI sources</t>
         </is>
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>New request, new handoff, unassigned over 15 minutes. On by default.</t>
+          <t>Shows the exact article version the model read.</t>
         </is>
       </c>
       <c r="G60" s="12" t="n">
@@ -4832,12 +4879,12 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>S09-01</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>A request with no staff view still reaches a human by email</t>
+          <t>Staff can see the cited text verbatim</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
@@ -4849,12 +4896,12 @@
     <row r="61" ht="40" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
@@ -4864,17 +4911,17 @@
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>Event emission across the product</t>
+          <t>Reply, take over, assign, resolve</t>
         </is>
       </c>
       <c r="F61" s="11" t="inlineStr">
         <is>
-          <t>All 18 taxonomy events wired with required context.</t>
+          <t>Takeover stops AI guest-facing replies immediately.</t>
         </is>
       </c>
       <c r="G61" s="12" t="n">
@@ -4887,12 +4934,12 @@
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>W00-19</t>
+          <t>S08-01</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>Dashboard numbers reconcile exactly to raw events</t>
+          <t>No race where AI replies after a takeover</t>
         </is>
       </c>
       <c r="K61" s="11" t="inlineStr">
@@ -4904,12 +4951,12 @@
     <row r="62" ht="40" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>S10-02</t>
+          <t>S08-04</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
@@ -4919,17 +4966,17 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>Daily rollups</t>
+          <t>AI operating modes</t>
         </is>
       </c>
       <c r="F62" s="11" t="inlineStr">
         <is>
-          <t>Nightly SQL over events. Idempotent and re-runnable.</t>
+          <t>Auto / Draft / Human-only / After-hours, feature-flagged per property.</t>
         </is>
       </c>
       <c r="G62" s="12" t="n">
@@ -4942,12 +4989,12 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
         <is>
-          <t>A historical date can be recomputed without drift</t>
+          <t>Mode change applies to the next message, no deploy</t>
         </is>
       </c>
       <c r="K62" s="11" t="inlineStr">
@@ -4959,12 +5006,12 @@
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>S10-03</t>
+          <t>S09-01</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C63" s="20" t="inlineStr">
@@ -4974,17 +5021,17 @@
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>Management dashboard</t>
+          <t>Request lifecycle</t>
         </is>
       </c>
       <c r="F63" s="11" t="inlineStr">
         <is>
-          <t>Top questions by property and language, unanswered, request volume and resolution, handoff rate.</t>
+          <t>Status, owner, timestamps, internal notes, priority, reopen.</t>
         </is>
       </c>
       <c r="G63" s="12" t="n">
@@ -4997,12 +5044,12 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>S10-02</t>
+          <t>S07-03</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>Every tile traceable to a query a manager can explain</t>
+          <t>request_acknowledged is set by a real staff action</t>
         </is>
       </c>
       <c r="K63" s="11" t="inlineStr">
@@ -5014,12 +5061,12 @@
     <row r="64" ht="40" customHeight="1">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>S11-01</t>
+          <t>S09-02</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
@@ -5029,21 +5076,21 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>Transactional outbox + worker + DLQ</t>
+          <t>Knowledge-gap queue</t>
         </is>
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>Send outside the request handler; backoff; failures visible.</t>
+          <t>Unanswered and flagged questions with verbatim text, language, property.</t>
         </is>
       </c>
       <c r="G64" s="12" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
@@ -5052,12 +5099,12 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S05-02</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
-          <t>Provider outage delays sends, never loses them</t>
+          <t>Every no_answer lands in the queue automatically</t>
         </is>
       </c>
       <c r="K64" s="11" t="inlineStr">
@@ -5069,12 +5116,12 @@
     <row r="65" ht="40" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>S11-02</t>
+          <t>S09-03</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C65" s="20" t="inlineStr">
@@ -5084,21 +5131,21 @@
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
         <is>
-          <t>Idempotency + webhook dedupe</t>
+          <t>One-click 'wrong or outdated'</t>
         </is>
       </c>
       <c r="F65" s="11" t="inlineStr">
         <is>
-          <t>Unique on (channel_connection_id, channel_message_id).</t>
+          <t>Creates or updates a knowledge gap with context.</t>
         </is>
       </c>
       <c r="G65" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H65" s="11" t="inlineStr">
         <is>
@@ -5107,12 +5154,12 @@
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>S06-01</t>
+          <t>S08-02</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr">
         <is>
-          <t>Replaying a webhook 10× produces one message</t>
+          <t>A flag is attributable to an ai_run</t>
         </is>
       </c>
       <c r="K65" s="11" t="inlineStr">
@@ -5124,12 +5171,12 @@
     <row r="66" ht="40" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>S11-03</t>
+          <t>S09-04</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
@@ -5139,21 +5186,21 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Inbox</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>PII redaction + log hygiene</t>
+          <t>Non-blocking review queue</t>
         </is>
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>Luhn card detection, long digit runs, emails, phones. No message bodies to third parties.</t>
+          <t>Never gates guest delivery. Replaces Draft as the week-one mechanism.</t>
         </is>
       </c>
       <c r="G66" s="12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H66" s="11" t="inlineStr">
         <is>
@@ -5162,12 +5209,12 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>S10-01</t>
+          <t>S08-03</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
         <is>
-          <t>A synthetic card number never reaches logs</t>
+          <t>Flagging an answer does not delay the guest reply</t>
         </is>
       </c>
       <c r="K66" s="11" t="inlineStr">
@@ -5179,12 +5226,12 @@
     <row r="67" ht="40" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>S11-04</t>
+          <t>S09-05</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="C67" s="20" t="inlineStr">
@@ -5194,17 +5241,17 @@
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>Observability + alerting</t>
+          <t>Email notifications</t>
         </is>
       </c>
       <c r="F67" s="11" t="inlineStr">
         <is>
-          <t>Webhook failures, outbox backlog, LLM errors, spend caps, p95, eval regression.</t>
+          <t>New request, new handoff, unassigned over 15 minutes. On by default.</t>
         </is>
       </c>
       <c r="G67" s="12" t="n">
@@ -5217,12 +5264,12 @@
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>S11-01</t>
+          <t>S09-01</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
         <is>
-          <t>Every alert fires once in staging with a runbook link</t>
+          <t>A request with no staff view still reaches a human by email</t>
         </is>
       </c>
       <c r="K67" s="11" t="inlineStr">
@@ -5234,12 +5281,12 @@
     <row r="68" ht="40" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>S11-05</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr">
@@ -5249,21 +5296,21 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Nightly embedding reconciliation</t>
+          <t>Event emission across the product</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>Every current version has chunks; every chunk resolves to a current version; no orphans.</t>
+          <t>All 18 taxonomy events wired with required context.</t>
         </is>
       </c>
       <c r="G68" s="12" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
@@ -5272,12 +5319,12 @@
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>S02-05</t>
+          <t>W00-19</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr">
         <is>
-          <t>Job fails loudly on a seeded drift case</t>
+          <t>Dashboard numbers reconcile exactly to raw events</t>
         </is>
       </c>
       <c r="K68" s="11" t="inlineStr">
@@ -5289,12 +5336,12 @@
     <row r="69" ht="40" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>S12-01</t>
+          <t>S10-02</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C69" s="20" t="inlineStr">
@@ -5304,17 +5351,17 @@
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>Runbook + backup restore drill</t>
+          <t>Daily rollups</t>
         </is>
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>LLM down, WhatsApp down, DB failover, duplicate storm, spend-cap trip, deletion request.</t>
+          <t>Nightly SQL over events. Idempotent and re-runnable.</t>
         </is>
       </c>
       <c r="G69" s="12" t="n">
@@ -5327,12 +5374,12 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>S11-04</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>Restore completed and timed; runbook signed</t>
+          <t>A historical date can be recomputed without drift</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr">
@@ -5344,12 +5391,12 @@
     <row r="70" ht="40" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>S12-02</t>
+          <t>S10-03</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
@@ -5359,35 +5406,35 @@
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Hardening</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Accessibility + ES/EN audit</t>
+          <t>Management dashboard</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>Guest chat and staff UI; a mid-range Android on hotel wifi.</t>
+          <t>Top questions by property and language, unanswered, request volume and resolution, handoff rate.</t>
         </is>
       </c>
       <c r="G70" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S10-02</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
-          <t>Lighthouse a11y ≥90; no untranslated strings</t>
+          <t>Every tile traceable to a query a manager can explain</t>
         </is>
       </c>
       <c r="K70" s="11" t="inlineStr">
@@ -5399,12 +5446,12 @@
     <row r="71" ht="40" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>S12-03</t>
+          <t>S11-01</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C71" s="20" t="inlineStr">
@@ -5419,30 +5466,30 @@
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>Load test</t>
+          <t>Transactional outbox + worker + DLQ</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>300 concurrent guests on one property; 50 staff sessions.</t>
+          <t>Send outside the request handler; backoff; failures visible.</t>
         </is>
       </c>
       <c r="G71" s="12" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>S08-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>p95 first token ≤3.5s at target load</t>
+          <t>Provider outage delays sends, never loses them</t>
         </is>
       </c>
       <c r="K71" s="11" t="inlineStr">
@@ -5454,36 +5501,36 @@
     <row r="72" ht="40" customHeight="1">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S11-02</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
-        </is>
-      </c>
-      <c r="C72" s="21" t="inlineStr">
-        <is>
-          <t>Both</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Pilot dry run with real content</t>
+          <t>Idempotency + webhook dedupe</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Full scripted flow with the hotel's actual staff on their real content.</t>
+          <t>Unique on (channel_connection_id, channel_message_id).</t>
         </is>
       </c>
       <c r="G72" s="12" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
@@ -5492,12 +5539,12 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>S12-01</t>
+          <t>S06-01</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>Three hotel staff complete the flow unaided</t>
+          <t>Replaying a webhook 10× produces one message</t>
         </is>
       </c>
       <c r="K72" s="11" t="inlineStr">
@@ -5509,32 +5556,32 @@
     <row r="73" ht="40" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>S13-01</t>
+          <t>S11-03</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C73" s="19" t="inlineStr">
-        <is>
-          <t>Founder</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>Staff training</t>
+          <t>PII redaction + log hygiene</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>Three staff, scripted flows, escalation expectations, the honest-answer rule.</t>
+          <t>Luhn card detection, long digit runs, emails, phones. No message bodies to third parties.</t>
         </is>
       </c>
       <c r="G73" s="12" t="n">
@@ -5547,12 +5594,12 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S10-01</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>Each staff member completes a live test conversation</t>
+          <t>A synthetic card number never reaches logs</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr">
@@ -5564,36 +5611,36 @@
     <row r="74" ht="40" customHeight="1">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>S13-02</t>
+          <t>S11-04</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C74" s="21" t="inlineStr">
-        <is>
-          <t>Both</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>Hardening</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Content corrections from the dry run</t>
+          <t>Observability + alerting</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>Fix what the golden set and the dry run exposed.</t>
+          <t>Webhook failures, outbox backlog, LLM errors, spend caps, p95, eval regression.</t>
         </is>
       </c>
       <c r="G74" s="12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
@@ -5602,12 +5649,12 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>S12-04</t>
+          <t>S11-01</t>
         </is>
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>No known-wrong article in the published set</t>
+          <t>Every alert fires once in staging with a runbook link</t>
         </is>
       </c>
       <c r="K74" s="11" t="inlineStr">
@@ -5619,32 +5666,32 @@
     <row r="75" ht="40" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>S13-03</t>
+          <t>S11-05</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="C75" s="19" t="inlineStr">
-        <is>
-          <t>Founder</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>Pilot</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>Launch checklist + GM go/no-go</t>
+          <t>Nightly embedding reconciliation</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>Notifications live, escalation contact confirmed, QR printed, link on the website.</t>
+          <t>Every current version has chunks; every chunk resolves to a current version; no orphans.</t>
         </is>
       </c>
       <c r="G75" s="12" t="n">
@@ -5657,400 +5704,400 @@
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
+          <t>S02-05</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>Job fails loudly on a seeded drift case</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>S12-01</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>Runbook + backup restore drill</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>LLM down, WhatsApp down, DB failover, duplicate storm, spend-cap trip, deletion request.</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>S11-04</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>Restore completed and timed; runbook signed</t>
+        </is>
+      </c>
+      <c r="K76" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>S12-02</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>Accessibility + ES/EN audit</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>Guest chat and staff UI; a mid-range Android on hotel wifi.</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>S08-01</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>Lighthouse a11y ≥90; no untranslated strings</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>S12-03</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Hardening</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>Load test</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>300 concurrent guests on one property; 50 staff sessions.</t>
+        </is>
+      </c>
+      <c r="G78" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>S08-01</t>
+        </is>
+      </c>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>p95 first token ≤3.5s at target load</t>
+        </is>
+      </c>
+      <c r="K78" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C79" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>Pilot dry run with real content</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>Full scripted flow with the hotel's actual staff on their real content.</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>S12-01</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>Three hotel staff complete the flow unaided</t>
+        </is>
+      </c>
+      <c r="K79" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
           <t>S13-01</t>
         </is>
       </c>
-      <c r="J75" s="11" t="inlineStr">
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C80" s="19" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>Staff training</t>
+        </is>
+      </c>
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>Three staff, scripted flows, escalation expectations, the honest-answer rule.</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I80" s="11" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="J80" s="11" t="inlineStr">
+        <is>
+          <t>Each staff member completes a live test conversation</t>
+        </is>
+      </c>
+      <c r="K80" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>S13-02</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C81" s="21" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>Content corrections from the dry run</t>
+        </is>
+      </c>
+      <c r="F81" s="11" t="inlineStr">
+        <is>
+          <t>Fix what the golden set and the dry run exposed.</t>
+        </is>
+      </c>
+      <c r="G81" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>S12-04</t>
+        </is>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>No known-wrong article in the published set</t>
+        </is>
+      </c>
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>S13-03</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C82" s="19" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>Pilot</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>Launch checklist + GM go/no-go</t>
+        </is>
+      </c>
+      <c r="F82" s="11" t="inlineStr">
+        <is>
+          <t>Notifications live, escalation contact confirmed, QR printed, link on the website.</t>
+        </is>
+      </c>
+      <c r="G82" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H82" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>S13-01</t>
+        </is>
+      </c>
+      <c r="J82" s="11" t="inlineStr">
         <is>
           <t>Written go/no-go from the GM</t>
         </is>
       </c>
-      <c r="K75" s="11" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="22" t="inlineStr">
-        <is>
-          <t>WA-01</t>
-        </is>
-      </c>
-      <c r="B76" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C76" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D76" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E76" s="23" t="inlineStr">
-        <is>
-          <t>Payment method on WABA</t>
-        </is>
-      </c>
-      <c r="F76" s="23" t="inlineStr">
-        <is>
-          <t>Without it, service messages beyond 1,000/month do not deliver.</t>
-        </is>
-      </c>
-      <c r="G76" s="24" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H76" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I76" s="23" t="inlineStr">
-        <is>
-          <t>W00-08</t>
-        </is>
-      </c>
-      <c r="J76" s="23" t="inlineStr">
-        <is>
-          <t>Billing active; spend alert configured</t>
-        </is>
-      </c>
-      <c r="K76" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="22" t="inlineStr">
-        <is>
-          <t>WA-02</t>
-        </is>
-      </c>
-      <c r="B77" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C77" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D77" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E77" s="23" t="inlineStr">
-        <is>
-          <t>Adapter: webhook ingress</t>
-        </is>
-      </c>
-      <c r="F77" s="23" t="inlineStr">
-        <is>
-          <t>Verify signature, dedupe, normalise, acknowledge under 3 seconds.</t>
-        </is>
-      </c>
-      <c r="G77" s="24" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H77" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I77" s="23" t="inlineStr">
-        <is>
-          <t>W00-09</t>
-        </is>
-      </c>
-      <c r="J77" s="23" t="inlineStr">
-        <is>
-          <t>A replayed webhook produces exactly one message</t>
-        </is>
-      </c>
-      <c r="K77" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="22" t="inlineStr">
-        <is>
-          <t>WA-03</t>
-        </is>
-      </c>
-      <c r="B78" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D78" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E78" s="23" t="inlineStr">
-        <is>
-          <t>Adapter: send path + 24h window</t>
-        </is>
-      </c>
-      <c r="F78" s="23" t="inlineStr">
-        <is>
-          <t>Window tracking per conversation. Templates outside, free-form inside.</t>
-        </is>
-      </c>
-      <c r="G78" s="24" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H78" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I78" s="23" t="inlineStr">
-        <is>
-          <t>WA-02</t>
-        </is>
-      </c>
-      <c r="J78" s="23" t="inlineStr">
-        <is>
-          <t>Sending outside the window impossible without a template</t>
-        </is>
-      </c>
-      <c r="K78" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="22" t="inlineStr">
-        <is>
-          <t>WA-04</t>
-        </is>
-      </c>
-      <c r="B79" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D79" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E79" s="23" t="inlineStr">
-        <is>
-          <t>Consent + opt-out store</t>
-        </is>
-      </c>
-      <c r="F79" s="23" t="inlineStr">
-        <is>
-          <t>Explicit consent records, STOP handling, rules isolated in the adapter.</t>
-        </is>
-      </c>
-      <c r="G79" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I79" s="23" t="inlineStr">
-        <is>
-          <t>WA-03</t>
-        </is>
-      </c>
-      <c r="J79" s="23" t="inlineStr">
-        <is>
-          <t>Opt-out honoured across every send path</t>
-        </is>
-      </c>
-      <c r="K79" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="22" t="inlineStr">
-        <is>
-          <t>WA-05</t>
-        </is>
-      </c>
-      <c r="B80" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C80" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D80" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E80" s="23" t="inlineStr">
-        <is>
-          <t>Message-efficient reply composition</t>
-        </is>
-      </c>
-      <c r="F80" s="23" t="inlineStr">
-        <is>
-          <t>One complete reply per turn. No streaming into WhatsApp — every bubble is billable.</t>
-        </is>
-      </c>
-      <c r="G80" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H80" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I80" s="23" t="inlineStr">
-        <is>
-          <t>S05-02</t>
-        </is>
-      </c>
-      <c r="J80" s="23" t="inlineStr">
-        <is>
-          <t>A typical exchange stays within the message budget</t>
-        </is>
-      </c>
-      <c r="K80" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="40" customHeight="1">
-      <c r="A81" s="22" t="inlineStr">
-        <is>
-          <t>WA-06</t>
-        </is>
-      </c>
-      <c r="B81" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C81" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D81" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E81" s="23" t="inlineStr">
-        <is>
-          <t>Template submission + approval</t>
-        </is>
-      </c>
-      <c r="F81" s="23" t="inlineStr">
-        <is>
-          <t>Utility templates for outside-window replies.</t>
-        </is>
-      </c>
-      <c r="G81" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H81" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I81" s="23" t="inlineStr">
-        <is>
-          <t>W00-09</t>
-        </is>
-      </c>
-      <c r="J81" s="23" t="inlineStr">
-        <is>
-          <t>Templates approved and sendable</t>
-        </is>
-      </c>
-      <c r="K81" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="40" customHeight="1">
-      <c r="A82" s="22" t="inlineStr">
-        <is>
-          <t>WA-07</t>
-        </is>
-      </c>
-      <c r="B82" s="23" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="C82" s="20" t="inlineStr">
-        <is>
-          <t>Eng</t>
-        </is>
-      </c>
-      <c r="D82" s="23" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E82" s="23" t="inlineStr">
-        <is>
-          <t>Number-migration safeguards</t>
-        </is>
-      </c>
-      <c r="F82" s="23" t="inlineStr">
-        <is>
-          <t>Warn that migrating a number deletes consumer WhatsApp history.</t>
-        </is>
-      </c>
-      <c r="G82" s="24" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H82" s="23" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="I82" s="23" t="inlineStr">
-        <is>
-          <t>W00-04</t>
-        </is>
-      </c>
-      <c r="J82" s="23" t="inlineStr">
-        <is>
-          <t>Written acknowledgement captured in onboarding</t>
-        </is>
-      </c>
-      <c r="K82" s="23" t="inlineStr">
+      <c r="K82" s="11" t="inlineStr">
         <is>
           <t>☐ Not started</t>
         </is>
@@ -6059,163 +6106,548 @@
     <row r="83" ht="40" customHeight="1">
       <c r="A83" s="22" t="inlineStr">
         <is>
+          <t>WA-01</t>
+        </is>
+      </c>
+      <c r="B83" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D83" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E83" s="23" t="inlineStr">
+        <is>
+          <t>Payment method on WABA</t>
+        </is>
+      </c>
+      <c r="F83" s="23" t="inlineStr">
+        <is>
+          <t>Without it, service messages beyond 1,000/month do not deliver.</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H83" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I83" s="23" t="inlineStr">
+        <is>
+          <t>W00-08</t>
+        </is>
+      </c>
+      <c r="J83" s="23" t="inlineStr">
+        <is>
+          <t>Billing active; spend alert configured</t>
+        </is>
+      </c>
+      <c r="K83" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>WA-02</t>
+        </is>
+      </c>
+      <c r="B84" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E84" s="23" t="inlineStr">
+        <is>
+          <t>Adapter: webhook ingress</t>
+        </is>
+      </c>
+      <c r="F84" s="23" t="inlineStr">
+        <is>
+          <t>Verify signature, dedupe, normalise, acknowledge under 3 seconds.</t>
+        </is>
+      </c>
+      <c r="G84" s="24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H84" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I84" s="23" t="inlineStr">
+        <is>
+          <t>W00-09</t>
+        </is>
+      </c>
+      <c r="J84" s="23" t="inlineStr">
+        <is>
+          <t>A replayed webhook produces exactly one message</t>
+        </is>
+      </c>
+      <c r="K84" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>WA-03</t>
+        </is>
+      </c>
+      <c r="B85" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D85" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E85" s="23" t="inlineStr">
+        <is>
+          <t>Adapter: send path + 24h window</t>
+        </is>
+      </c>
+      <c r="F85" s="23" t="inlineStr">
+        <is>
+          <t>Window tracking per conversation. Templates outside, free-form inside.</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H85" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I85" s="23" t="inlineStr">
+        <is>
+          <t>WA-02</t>
+        </is>
+      </c>
+      <c r="J85" s="23" t="inlineStr">
+        <is>
+          <t>Sending outside the window impossible without a template</t>
+        </is>
+      </c>
+      <c r="K85" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>WA-04</t>
+        </is>
+      </c>
+      <c r="B86" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D86" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E86" s="23" t="inlineStr">
+        <is>
+          <t>Consent + opt-out store</t>
+        </is>
+      </c>
+      <c r="F86" s="23" t="inlineStr">
+        <is>
+          <t>Explicit consent records, STOP handling, rules isolated in the adapter.</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I86" s="23" t="inlineStr">
+        <is>
+          <t>WA-03</t>
+        </is>
+      </c>
+      <c r="J86" s="23" t="inlineStr">
+        <is>
+          <t>Opt-out honoured across every send path</t>
+        </is>
+      </c>
+      <c r="K86" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>WA-05</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D87" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E87" s="23" t="inlineStr">
+        <is>
+          <t>Message-efficient reply composition</t>
+        </is>
+      </c>
+      <c r="F87" s="23" t="inlineStr">
+        <is>
+          <t>One complete reply per turn. No streaming into WhatsApp — every bubble is billable.</t>
+        </is>
+      </c>
+      <c r="G87" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I87" s="23" t="inlineStr">
+        <is>
+          <t>S05-02</t>
+        </is>
+      </c>
+      <c r="J87" s="23" t="inlineStr">
+        <is>
+          <t>A typical exchange stays within the message budget</t>
+        </is>
+      </c>
+      <c r="K87" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="22" t="inlineStr">
+        <is>
+          <t>WA-06</t>
+        </is>
+      </c>
+      <c r="B88" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D88" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E88" s="23" t="inlineStr">
+        <is>
+          <t>Template submission + approval</t>
+        </is>
+      </c>
+      <c r="F88" s="23" t="inlineStr">
+        <is>
+          <t>Utility templates for outside-window replies.</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I88" s="23" t="inlineStr">
+        <is>
+          <t>W00-09</t>
+        </is>
+      </c>
+      <c r="J88" s="23" t="inlineStr">
+        <is>
+          <t>Templates approved and sendable</t>
+        </is>
+      </c>
+      <c r="K88" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="22" t="inlineStr">
+        <is>
+          <t>WA-07</t>
+        </is>
+      </c>
+      <c r="B89" s="23" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>Eng</t>
+        </is>
+      </c>
+      <c r="D89" s="23" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E89" s="23" t="inlineStr">
+        <is>
+          <t>Number-migration safeguards</t>
+        </is>
+      </c>
+      <c r="F89" s="23" t="inlineStr">
+        <is>
+          <t>Warn that migrating a number deletes consumer WhatsApp history.</t>
+        </is>
+      </c>
+      <c r="G89" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H89" s="23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I89" s="23" t="inlineStr">
+        <is>
+          <t>W00-04</t>
+        </is>
+      </c>
+      <c r="J89" s="23" t="inlineStr">
+        <is>
+          <t>Written acknowledgement captured in onboarding</t>
+        </is>
+      </c>
+      <c r="K89" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="22" t="inlineStr">
+        <is>
           <t>WA-08</t>
         </is>
       </c>
-      <c r="B83" s="23" t="inlineStr">
+      <c r="B90" s="23" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="C83" s="20" t="inlineStr">
+      <c r="C90" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D83" s="23" t="inlineStr">
+      <c r="D90" s="23" t="inlineStr">
         <is>
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="E83" s="23" t="inlineStr">
+      <c r="E90" s="23" t="inlineStr">
         <is>
           <t>Shadow run on one property</t>
         </is>
       </c>
-      <c r="F83" s="23" t="inlineStr">
+      <c r="F90" s="23" t="inlineStr">
         <is>
           <t>Run alongside web chat for a week before switching traffic.</t>
         </is>
       </c>
-      <c r="G83" s="24" t="n">
+      <c r="G90" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="H83" s="23" t="inlineStr">
+      <c r="H90" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I83" s="23" t="inlineStr">
+      <c r="I90" s="23" t="inlineStr">
         <is>
           <t>WA-03</t>
         </is>
       </c>
-      <c r="J83" s="23" t="inlineStr">
+      <c r="J90" s="23" t="inlineStr">
         <is>
           <t>Zero delivery failures across 7 days</t>
         </is>
       </c>
-      <c r="K83" s="23" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="25" t="inlineStr">
+      <c r="K90" s="23" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="25" t="inlineStr">
         <is>
           <t>DF-01</t>
         </is>
       </c>
-      <c r="B84" s="26" t="inlineStr">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>DEF</t>
         </is>
       </c>
-      <c r="C84" s="20" t="inlineStr">
+      <c r="C91" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D84" s="26" t="inlineStr">
+      <c r="D91" s="26" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
       </c>
-      <c r="E84" s="26" t="inlineStr">
+      <c r="E91" s="26" t="inlineStr">
         <is>
           <t>Outbound webhook per property</t>
         </is>
       </c>
-      <c r="F84" s="26" t="inlineStr">
+      <c r="F91" s="26" t="inlineStr">
         <is>
           <t>Signed, retried events to Teams/Slack/hotel ops tools.</t>
         </is>
       </c>
-      <c r="G84" s="27" t="n">
+      <c r="G91" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="H84" s="26" t="inlineStr">
+      <c r="H91" s="26" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I84" s="26" t="inlineStr">
+      <c r="I91" s="26" t="inlineStr">
         <is>
           <t>S09-05</t>
         </is>
       </c>
-      <c r="J84" s="26" t="inlineStr">
+      <c r="J91" s="26" t="inlineStr">
         <is>
           <t>A group needs events piped into their own tools</t>
         </is>
       </c>
-      <c r="K84" s="26" t="inlineStr">
-        <is>
-          <t>☐ Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="25" t="inlineStr">
+      <c r="K91" s="26" t="inlineStr">
+        <is>
+          <t>☐ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="25" t="inlineStr">
         <is>
           <t>DF-02</t>
         </is>
       </c>
-      <c r="B85" s="26" t="inlineStr">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>DEF</t>
         </is>
       </c>
-      <c r="C85" s="20" t="inlineStr">
+      <c r="C92" s="20" t="inlineStr">
         <is>
           <t>Eng</t>
         </is>
       </c>
-      <c r="D85" s="26" t="inlineStr">
+      <c r="D92" s="26" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="E85" s="26" t="inlineStr">
+      <c r="E92" s="26" t="inlineStr">
         <is>
           <t>Opportunity click tracking</t>
         </is>
       </c>
-      <c r="F85" s="26" t="inlineStr">
+      <c r="F92" s="26" t="inlineStr">
         <is>
           <t>Booking/dining/spa link clicks, labelled opportunities, never revenue.</t>
         </is>
       </c>
-      <c r="G85" s="27" t="n">
+      <c r="G92" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="H85" s="26" t="inlineStr">
+      <c r="H92" s="26" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I85" s="26" t="inlineStr">
+      <c r="I92" s="26" t="inlineStr">
         <is>
           <t>S10-01</t>
         </is>
       </c>
-      <c r="J85" s="26" t="inlineStr">
+      <c r="J92" s="26" t="inlineStr">
         <is>
           <t>After the pilot, against real traffic</t>
         </is>
       </c>
-      <c r="K85" s="26" t="inlineStr">
+      <c r="K92" s="26" t="inlineStr">
         <is>
           <t>☐ Not started</t>
         </is>
@@ -6223,7 +6655,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"☐ Not started,◐ In progress,☑ Done,✖ Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6238,7 +6670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6550,117 +6982,121 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06A</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Chat hardening</t>
+          <t>API, deployment and eval reliability</t>
         </is>
       </c>
       <c r="D12" s="12" t="n">
-        <v>4</v>
+        <v>14.5</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="29" t="inlineStr">
-        <is>
-          <t>Fits</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr"/>
+        <v>14.5</v>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>Over by 9.50</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Spills into the following week.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Staff inbox</t>
+          <t>Chat hardening</t>
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G13" s="28" t="inlineStr">
-        <is>
-          <t>Over by 0.50</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>Spills into the following week.</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>Fits</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Requests and notifications</t>
+          <t>Staff inbox</t>
         </is>
       </c>
       <c r="D14" s="12" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G14" s="29" t="inlineStr">
-        <is>
-          <t>Fits</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr"/>
+        <v>5.5</v>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Over by 0.50</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Spills into the following week.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Requests and notifications</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
@@ -6682,27 +7118,27 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="D16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G16" s="29" t="inlineStr">
         <is>
@@ -6714,27 +7150,27 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Pilot readiness</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G17" s="29" t="inlineStr">
         <is>
@@ -6746,67 +7182,99 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Pilot readiness</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>Fits</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
           <t>S13</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D19" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E19" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="29" t="inlineStr">
+      <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Fits</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Launch work plus ~3 days of carry-forward room.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="5" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Original launch date invalid after 14.50-day S06A; reforecast with owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Total demand</t>
         </is>
       </c>
-      <c r="F20" s="30" t="n">
+      <c r="F21" s="30" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Original capacity (14 × 5)</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="21">
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Capacity (14 × 5)</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Unallocated</t>
-        </is>
-      </c>
-      <c r="F22" s="31" t="n">
-        <v>0</v>
+    <row r="23">
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Over capacity</t>
+        </is>
+      </c>
+      <c r="F23" s="31" t="n">
+        <v>14.5</v>
       </c>
     </row>
   </sheetData>
@@ -7007,7 +7475,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Pilot live</t>
+          <t>Pilot live (original target; reforecast)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -7017,7 +7485,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>After S06A</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -7027,7 +7495,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Postpone a week; do not launch untrained</t>
+          <t>Do not commit to W14 until staffing/parallelism is re-estimated</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7517,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>Reforecast</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -7081,7 +7549,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>Reforecast</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -7158,7 +7626,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Each step blocks the next. Any slip here moves W14 one-for-one.</t>
+          <t>Each step blocks the next. S06A is inserted before S07; recalculate launch after sequencing.</t>
         </is>
       </c>
     </row>
@@ -7412,7 +7880,7 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Analytics (S10), reliability (S11), accessibility and load (S12) — each can slip a week without moving W14.</t>
+          <t>Original W14 date is unconfirmed after S06A; reforecast before using dates for commitments.</t>
         </is>
       </c>
     </row>

</xml_diff>